<commit_message>
docs: neutral wording, MIT license, working notes kept local
The documents, comments and workbooks say what was decided, not who
decided it. The working notes of the project stay on the machine and
leave the repository.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -698,7 +698,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>2026-10-09: to T08: lower a little the elemental resistances of the superbosses that wall magic off, keeping their flavour; 2026-10-11: not built; measured again, to decide with the postgame (six superbosses); the user, 2026-10-11: with the postgame; the user, 2026-10-12: lower it without abuse, the postgame stays hard and the mages keep some of their power; built as RES x0.9 (E213 - E223)</t>
+          <t>2026-10-09: to T08: lower a little the elemental resistances of the superbosses that wall magic off, keeping their flavour; 2026-10-11: not built; measured again, to decide with the postgame (six superbosses); decided 2026-10-11: with the postgame; decided 2026-10-12: lower it without abuse, the postgame stays hard and the mages keep some of their power; built as RES x0.9 (E213 - E223)</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>2026-10-09: a small cut to two-handed pieces anyway (W rows), the user asked for it</t>
+          <t>2026-10-09: a small cut to two-handed pieces anyway (W rows), it was asked for it</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1165,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Overstated: the party is not empty after 3 or 4 battles (see Vanilla_Result); closed by the user 2026-10-09</t>
+          <t>Overstated: the party is not empty after 3 or 4 battles (see Vanilla_Result); closed 2026-10-09</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>2026-10-09: faster chant for the top spells (J33, M rows); the user meets cancellations in play, the model completes 82 - 98% of chants</t>
+          <t>2026-10-09: faster chant for the top spells (J33, M rows); cancellations are met in play, the model completes 82 - 98% of chants</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>2026-10-09: accepted by the user</t>
+          <t>2026-10-09: accepted</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>T041 - T050, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Treasure Hunter 1.21 advanced (slow), 1.00 late; the user, 2026-10-11: what is left is not a problem</t>
+          <t>T041 - T050, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Treasure Hunter 1.21 advanced (slow), 1.00 late; decided 2026-10-11: what is left is not a problem</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2546,12 +2546,12 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>T041 - T050: Pursuit Stab -25% TP, x2 power | 2026-10-11, the user: what is left is not a problem. After T041 - T050 she is 25% slower than the median attacker at C22 - C40 with 14 - 21% of the damage, and level with it in the postgame (1.00); her build of the guide is passives of exploration. The Dagger and the Kukri are left alone: at twice their forge rate the reference party, which holds her, makes 17 bosses easier than vanilla instead of 7</t>
+          <t>T041 - T050: Pursuit Stab -25% TP, x2 power | 2026-10-11, decided: what is left is not a problem. After T041 - T050 she is 25% slower than the median attacker at C22 - C40 with 14 - 21% of the damage, and level with it in the postgame (1.00); her build of the guide is passives of exploration. The Dagger and the Kukri are left alone: at twice their forge rate the reference party, which holds her, makes 17 bosses easier than vanilla instead of 7</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>2026-10-09: accepted by the user</t>
+          <t>2026-10-09: accepted</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2782,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>2026-10-09: accepted by the user</t>
+          <t>2026-10-09: accepted</t>
         </is>
       </c>
     </row>
@@ -3353,7 +3353,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>ExePatches set balance in both program files (12 rows, 17 bytes each); seen working in the game by the user</t>
+          <t>ExePatches set balance in both program files (12 rows, 17 bytes each); seen working in the game</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>2026-10-10: no further change; party flexibility improved by T03 and class balance; 2026-10-12: reopened, the closing held no figure; waits for the user; the user, 2026-10-12: a fifth more TP from the fruit and no new cut of TP costs; the Maid keeps her part and a party without her gets through with effort</t>
+          <t>2026-10-10: no further change; party flexibility improved by T03 and class balance; 2026-10-12: reopened, the closing held no figure; waits for a decision; decided 2026-10-12: a fifth more TP from the fruit and no new cut of TP costs; the Maid keeps her part and a party without her gets through with effort</t>
         </is>
       </c>
     </row>
@@ -3619,7 +3619,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>2026-10-09: accepted by the user</t>
+          <t>2026-10-09: accepted</t>
         </is>
       </c>
     </row>
@@ -3696,7 +3696,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>2026-10-09: option B accepted by the user; the same time as the Papillon at C34 and C40, 23% slower at P24 while winning more</t>
+          <t>2026-10-09: option B accepted; the same time as the Papillon at C34 and C40, 23% slower at P24 while winning more</t>
         </is>
       </c>
     </row>
@@ -3773,7 +3773,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>2026-10-09: option B accepted by the user</t>
+          <t>2026-10-09: option B accepted</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3835,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Items and dolls (techniques) still act in the four anti-magic fights; closed by the user 2026-10-09</t>
+          <t>Items and dolls (techniques) still act in the four anti-magic fights; closed 2026-10-09</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -4568,7 +4568,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>2026-10-09: bosses open to slow and silence unless superbosses, to sleep in the story (A rows); poison opened on six story bosses (A rows, the user 2026-10-09)</t>
+          <t>2026-10-09: bosses open to slow and silence unless superbosses, to sleep in the story (A rows); poison opened on six story bosses (A rows, decided 2026-10-09)</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>2026-10-09: accepted by the user</t>
+          <t>2026-10-09: accepted</t>
         </is>
       </c>
     </row>
@@ -5047,7 +5047,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>L rows built; L002 dropped on 2026-10-11 (the user): its damage draw strikes any unit of the battle, the party included, so it stays at level x 10. Its heal of an enemy is 10% of max HP instead of all of it (L001). Cast every turn, rows of eight random battles last 3 - 25% longer and end with -1 to +3 points of HP: the cheap gamble of the base class (15 TP, one level), which can no longer sink a fight</t>
+          <t>L rows built; L002 dropped on 2026-10-11 : its damage draw strikes any unit of the battle, the party included, so it stays at level x 10. Its heal of an enemy is 10% of max HP instead of all of it (L001). Cast every turn, rows of eight random battles last 3 - 25% longer and end with -1 to +3 points of HP: the cheap gamble of the base class (15 TP, one level), which can no longer sink a fight</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -5735,7 +5735,7 @@
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>2026-10-09: accepted by the user</t>
+          <t>2026-10-09: accepted</t>
         </is>
       </c>
     </row>
@@ -5807,7 +5807,7 @@
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>2026-10-09: accepted by the user</t>
+          <t>2026-10-09: accepted</t>
         </is>
       </c>
     </row>
@@ -5921,7 +5921,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>X088 and its levels, Blood Rage 43 to 32 TP, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, the user: the change stays, it is justified in its row</t>
+          <t>X088 and its levels, Blood Rage 43 to 32 TP, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
@@ -5946,7 +5946,7 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>2026-10-11: approved by the user, the change stays</t>
+          <t>2026-10-11: approved, the change stays</t>
         </is>
       </c>
     </row>
@@ -5993,7 +5993,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>X rows, Brave and Protect x2, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, the user: the change stays, it is justified in its row</t>
+          <t>X rows, Brave and Protect x2, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
@@ -6018,7 +6018,7 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>2026-10-11: approved by the user, the change stays</t>
+          <t>2026-10-11: approved, the change stays</t>
         </is>
       </c>
     </row>
@@ -6606,7 +6606,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>X rows, Illusion 3 / 4 / 5 hits, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, the user: the change stays, it is justified in its row</t>
+          <t>X rows, Illusion 3 / 4 / 5 hits, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -6631,7 +6631,7 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>2026-10-11: approved by the user, the change stays</t>
+          <t>2026-10-11: approved, the change stays</t>
         </is>
       </c>
     </row>
@@ -7192,7 +7192,7 @@
       </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>2026-10-09: open; 2026-10-11: measured; 2026-10-11, the user: raise it to a reasonable level; W047 - W051 built and read back (1,387 of 1,387 rows)</t>
+          <t>2026-10-09: open; 2026-10-11: measured; 2026-10-11, decided: raise it to a reasonable level; W047 - W051 built and read back (1,387 of 1,387 rows)</t>
         </is>
       </c>
     </row>
@@ -7718,7 +7718,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>K rows (TP -25%) and X rows (chant 0.75 at every level), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, the user: the change stays, it is justified in its row</t>
+          <t>K rows (TP -25%) and X rows (chant 0.75 at every level), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -7743,7 +7743,7 @@
       </c>
       <c r="R98" t="inlineStr">
         <is>
-          <t>2026-10-11: approved by the user, the change stays</t>
+          <t>2026-10-11: approved, the change stays</t>
         </is>
       </c>
     </row>
@@ -7790,7 +7790,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>X rows, Shadow Sew -25% TP, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, the user: the change stays, it is justified in its row</t>
+          <t>X rows, Shadow Sew -25% TP, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="R99" t="inlineStr">
         <is>
-          <t>2026-10-11: approved by the user, the change stays</t>
+          <t>2026-10-11: approved, the change stays</t>
         </is>
       </c>
     </row>
@@ -7862,7 +7862,7 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>X rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); the scrolls are worth 48 - 60% beside Ninja Piledriver, which the Tantou (W045) raised (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class)). 2026-10-11, the user: they stay as they are, they are debuffs late (J27)</t>
+          <t>X rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); the scrolls are worth 48 - 60% beside Ninja Piledriver, which the Tantou (W045) raised (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class)). 2026-10-11, decided: they stay as they are, they are debuffs late (J27)</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -7887,7 +7887,7 @@
       </c>
       <c r="R100" t="inlineStr">
         <is>
-          <t>2026-10-09: accepted by the user</t>
+          <t>2026-10-09: accepted</t>
         </is>
       </c>
     </row>
@@ -8552,7 +8552,7 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>X rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Life Bringer worth 48% beside Showtime (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class)). 2026-10-11, the user: it stays as it is</t>
+          <t>X rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Life Bringer worth 48% beside Showtime (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class)). 2026-10-11, decided: it stays as it is</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
@@ -8577,7 +8577,7 @@
       </c>
       <c r="R110" t="inlineStr">
         <is>
-          <t>2026-10-09: accepted by the user</t>
+          <t>2026-10-09: accepted</t>
         </is>
       </c>
     </row>
@@ -9483,7 +9483,7 @@
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t>Joint skills parked by the user on 2026-10-04; DLC ignored</t>
+          <t>Joint skills parked on 2026-10-04; DLC ignored</t>
         </is>
       </c>
       <c r="O123" t="inlineStr">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="R126" t="inlineStr">
         <is>
-          <t>2026-10-09: both halves accepted by the user</t>
+          <t>2026-10-09: both halves accepted</t>
         </is>
       </c>
     </row>
@@ -9838,7 +9838,7 @@
       </c>
       <c r="N128" t="inlineStr">
         <is>
-          <t>Read on 2026-10-11 (measures/drops_reading.md, checked against 0x558517 - 0x5586fa): rows P011 - P023 and P025 of balance_changes.xlsx dropped, they changed the count of slots of drops that are certain or usual. Rows P024, P079 - P084 raise the seven pieces under 2% to 2%. The weight of a slot is the same word for the drop and for the steal (measures/steal_reading.md, checked on 2026-10-11): with the rows the Chief's Special comes out of 4.7% of the steals that succeed. Rows P085 - P088 (the user, 2026-10-11): Odin, Myrddin, Asmodeus and Carmilla, the four enemies of the random battles that could not be robbed, can be: their pieces come out of 6 to 9% of the steals that succeed, against 3.9 to 5.4% of the kills.</t>
+          <t>Read on 2026-10-11 (measures/drops_reading.md, checked against 0x558517 - 0x5586fa): rows P011 - P023 and P025 of balance_changes.xlsx dropped, they changed the count of slots of drops that are certain or usual. Rows P024, P079 - P084 raise the seven pieces under 2% to 2%. The weight of a slot is the same word for the drop and for the steal (measures/steal_reading.md, checked on 2026-10-11): with the rows the Chief's Special comes out of 4.7% of the steals that succeed. Rows P085 - P088 (decided 2026-10-11): Odin, Myrddin, Asmodeus and Carmilla, the four enemies of the random battles that could not be robbed, can be: their pieces come out of 6 to 9% of the steals that succeed, against 3.9 to 5.4% of the kills.</t>
         </is>
       </c>
       <c r="O128" t="inlineStr">
@@ -9853,7 +9853,7 @@
       </c>
       <c r="R128" t="inlineStr">
         <is>
-          <t>2026-10-11: approved by the user (seven drop weights to the 2% floor; Item Steal open on the four immune commons)</t>
+          <t>2026-10-11: approved (seven drop weights to the 2% floor; Item Steal open on the four immune commons)</t>
         </is>
       </c>
     </row>
@@ -9982,7 +9982,7 @@
       </c>
       <c r="N130" t="inlineStr">
         <is>
-          <t>The DLC is ignored (2026-10-06). What it eased is covered by T01: the factors by level gap (option B4, without the kept curve) catch a member up faster than a Double EXP piece did, and a crown costs about 400 battles instead of 4,393 (docs/generated/CATCH_UP_OPTIONS.md); one existing accessory, the Slave's Torc, carries Double EXP from 2026-10-11 (the user; row W042 of balance_changes.xlsx), which takes the place of "no new Double EXP item" of 2026-10-07</t>
+          <t>The DLC is ignored (2026-10-06). What it eased is covered by T01: the factors by level gap (option B4, without the kept curve) catch a member up faster than a Double EXP piece did, and a crown costs about 400 battles instead of 4,393 (docs/generated/CATCH_UP_OPTIONS.md); one existing accessory, the Slave's Torc, carries Double EXP from 2026-10-11 (row W042 of balance_changes.xlsx), which takes the place of "no new Double EXP item" of 2026-10-07</t>
         </is>
       </c>
       <c r="O130" t="inlineStr">
@@ -10322,7 +10322,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>ExePatches set balance in both program files; CATCH_UP_OPTIONS.md, row B4; seen working in the game by the user</t>
+          <t>ExePatches set balance in both program files; CATCH_UP_OPTIONS.md, row B4; seen working in the game</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -10342,7 +10342,7 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>B4 alone (the user, 2026-10-11): the factors by level gap are in the program, the EXP of a level stays as in vanilla. The kept curve is not built: it would put a party 3 to 9 levels above the level the bosses were fitted at, and can be added later as data. 10 levels behind: 20 - 47 battles (vanilla 48 - 144); 20 behind: 24 - 82 (65 - 311); from level 1: 24 - 107 (65 - 519) (docs/generated/CATCH_UP_OPTIONS.md, option B4)</t>
+          <t>B4 alone (decided 2026-10-11): the factors by level gap are in the program, the EXP of a level stays as in vanilla. The kept curve is not built: it would put a party 3 to 9 levels above the level the bosses were fitted at, and can be added later as data. 10 levels behind: 20 - 47 battles (vanilla 48 - 144); 20 behind: 24 - 82 (65 - 311); from level 1: 24 - 107 (65 - 519) (docs/generated/CATCH_UP_OPTIONS.md, option B4)</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
@@ -10429,7 +10429,7 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>Nothing beyond the factors B4 (U01): a level costs a party on level 19 - 26 battles instead of 25 - 35 (levels 30 - 70); the kept curve is not built (the user, 2026-10-11)</t>
+          <t>Nothing beyond the factors B4 (U01): a level costs a party on level 19 - 26 battles instead of 25 - 35 (levels 30 - 70); the kept curve is not built (decided 2026-10-11)</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
@@ -11239,7 +11239,7 @@
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>Nothing beyond the factors B4: the kept curve is not built (the user, 2026-10-11)</t>
+          <t>Nothing beyond the factors B4: the kept curve is not built (decided 2026-10-11)</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
@@ -11892,7 +11892,7 @@
       </c>
       <c r="R155" t="inlineStr">
         <is>
-          <t>2026-10-11: approved by the user (quest gold x1.40)</t>
+          <t>2026-10-11: approved (quest gold x1.40)</t>
         </is>
       </c>
     </row>
@@ -12145,7 +12145,7 @@
       </c>
       <c r="N159" t="inlineStr">
         <is>
-          <t>Out of scope: new behaviour of the program, large changes to the executable. Part of it is already answered by the QoL variant (the user, 2026-10-07)</t>
+          <t>Out of scope: new behaviour of the program, large changes to the executable. Part of it is already answered by the QoL variant (decided 2026-10-07)</t>
         </is>
       </c>
       <c r="O159" t="inlineStr">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t>Content and maps are out of the balance. The conditions of side events, which are only text, are being evaluated as an addition to the QoL variant, reopened for it (docs/QOL_ROADMAP.md, last section; the user, 2026-10-07)</t>
+          <t>Content and maps are out of the balance. The conditions of side events, which are only text, are being evaluated as an addition to the QoL variant, reopened for it (docs/QOL_ROADMAP.md, last section; decided 2026-10-07)</t>
         </is>
       </c>
       <c r="O160" t="inlineStr">
@@ -12520,7 +12520,7 @@
       </c>
       <c r="R164" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
+          <t>decided 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -12587,7 +12587,7 @@
       </c>
       <c r="R165" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
+          <t>decided 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -12654,7 +12654,7 @@
       </c>
       <c r="R166" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
+          <t>decided 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -12721,7 +12721,7 @@
       </c>
       <c r="R167" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
+          <t>decided 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -12788,7 +12788,7 @@
       </c>
       <c r="R168" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
+          <t>decided 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -12855,7 +12855,7 @@
       </c>
       <c r="R169" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
+          <t>decided 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -12922,7 +12922,7 @@
       </c>
       <c r="R170" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
+          <t>decided 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -12989,7 +12989,7 @@
       </c>
       <c r="R171" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
+          <t>decided 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -13056,7 +13056,7 @@
       </c>
       <c r="R172" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
+          <t>decided 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -13123,7 +13123,7 @@
       </c>
       <c r="R173" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
+          <t>decided 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -13195,7 +13195,7 @@
       </c>
       <c r="R174" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: raised | 2026-10-12 (evening), the user: the effect is changed for evasion, which serves in every class and fight | 2026-10-12 (night), the user: not evasion (always at work); the chance to survive a killing hit, situational as the others</t>
+          <t>decided 2026-10-12: raised | 2026-10-12 (evening), decided: the effect is changed for evasion, which serves in every class and fight | 2026-10-12 (night), decided: not evasion (always at work); the chance to survive a killing hit, situational as the others</t>
         </is>
       </c>
     </row>
@@ -13262,7 +13262,7 @@
       </c>
       <c r="R175" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
+          <t>decided 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -13329,7 +13329,7 @@
       </c>
       <c r="R176" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
+          <t>decided 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -13401,7 +13401,7 @@
       </c>
       <c r="R177" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: raised</t>
+          <t>decided 2026-10-12: raised</t>
         </is>
       </c>
     </row>
@@ -13448,7 +13448,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yuni as diva, without the skill &gt; with it): C36 96% &gt; 96%, C38 95% &gt; 95%, C40 93% &gt; 94%, P24 97% &gt; 99%, P27 crowned 83% &gt; 93%. In the mean +3 points of wins, fights +1% shorter, +3 points of HP left (a cell moves by about 5 points by chance). Raised a little on 2026-10-12 (the user: it is one of the good ones): 92.8% without the skill, 94.8% with it</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yuni as diva, without the skill &gt; with it): C36 96% &gt; 96%, C38 95% &gt; 95%, C40 93% &gt; 94%, P24 97% &gt; 99%, P27 crowned 83% &gt; 93%. In the mean +3 points of wins, fights +1% shorter, +3 points of HP left (a cell moves by about 5 points by chance). Raised a little on 2026-10-12 (decided: it is one of the good ones): 92.8% without the skill, 94.8% with it</t>
         </is>
       </c>
       <c r="L178" t="inlineStr">
@@ -13473,7 +13473,7 @@
       </c>
       <c r="R178" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: raised</t>
+          <t>decided 2026-10-12: raised</t>
         </is>
       </c>
     </row>
@@ -13545,7 +13545,7 @@
       </c>
       <c r="R179" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: raised</t>
+          <t>decided 2026-10-12: raised</t>
         </is>
       </c>
     </row>
@@ -13612,7 +13612,7 @@
       </c>
       <c r="R180" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: left as it is; it adds little but it is good to have</t>
+          <t>decided 2026-10-12: left as it is; it adds little but it is good to have</t>
         </is>
       </c>
     </row>
@@ -13684,7 +13684,7 @@
       </c>
       <c r="R181" t="inlineStr">
         <is>
-          <t>the user, 2026-10-12: raised</t>
+          <t>decided 2026-10-12: raised</t>
         </is>
       </c>
     </row>
@@ -14279,7 +14279,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Roll of Arcane Shield, a number below 100 under: 15 -&gt; 25 (the user, 2026-10-12; cmp eax, imm8 at 0x424766)</t>
+          <t>Roll of Arcane Shield, a number below 100 under: 15 -&gt; 25 (decided 2026-10-12; cmp eax, imm8 at 0x424766)</t>
         </is>
       </c>
     </row>
@@ -14301,14 +14301,14 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>The step of 59 to 68 levels stays at 1 point (accepted by the user, 2026-10-05): its instruction is an "inc", with no byte that holds the amount. Giving it 2 means rewriting the end of the function. With the other four steps one point higher the cheapest crown no longer uses that step (docs/generated/CATCH_UP_OPTIONS.md, rule "One more point, lowest step kept").</t>
+          <t>The step of 59 to 68 levels stays at 1 point (accepted by decided 2026-10-05): its instruction is an "inc", with no byte that holds the amount. Giving it 2 means rewriting the end of the function. With the other four steps one point higher the cheapest crown no longer uses that step (docs/generated/CATCH_UP_OPTIONS.md, rule "One more point, lowest step kept").</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Factors with the piece of enchantment 270 (X06 to X08: 1.5, 4, 6) and the last band at 10 with or without the piece: accepted by the user on 2026-10-05, after the test in the game. The name of the enchantment in the Balance variant states them (balance_enchant_text.xlsx).</t>
+          <t>Factors with the piece of enchantment 270 (X06 to X08: 1.5, 4, 6) and the last band at 10 with or without the piece: accepted on 2026-10-05, after the test in the game. The name of the enchantment in the Balance variant states them (balance_enchant_text.xlsx).</t>
         </is>
       </c>
     </row>
@@ -14345,7 +14345,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Interruption rate of a blow: max HP * 1.5 times (1 + Concentrate) where the program adds the two (addss -&gt; mulss at 0x44d042; its debug message writes the product). The user, 2026-10-12: mend it for every unit, enemies with the passive too</t>
+          <t>Interruption rate of a blow: max HP * 1.5 times (1 + Concentrate) where the program adds the two (addss -&gt; mulss at 0x44d042; its debug message writes the product). Decided 2026-10-12: mend it for every unit, enemies with the passive too</t>
         </is>
       </c>
     </row>
@@ -21792,7 +21792,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>open (no verdict yet); closed (the change that answers it is built and its check passes: it solves the complaint with margin); not a problem (the claim is false in vanilla, with the figure that shows it: a reading of the data, a formula or a simulation); out of the balance (see the next row). There is no "kept": a complaint that is true in vanilla is fixed. Hard to fix is not a reason. States of the approach of 2026-10-07 (BALANCE_PLAN.md section 8)</t>
+          <t>open (no verdict yet); closed (the change that answers it is built and its check passes: it solves the complaint with margin); not a problem (the claim is false in vanilla, with the figure that shows it: a reading of the data, a formula or a simulation); out of the balance (see the next row). There is no "kept": a complaint that is true in vanilla is fixed. Hard to fix is not a reason. States of the approach of 2026-10-07 (the project notes section 8)</t>
         </is>
       </c>
     </row>
@@ -21828,7 +21828,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>How the model decides the claim. The bands, windows and floors are the targets of docs/BALANCE_PLAN.md, phase 3.</t>
+          <t>How the model decides the claim. The bands, windows and floors are the targets of the project notes, phase 3.</t>
         </is>
       </c>
     </row>
@@ -21865,7 +21865,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>The row is not a claim about balance, or it can only be answered by new behaviour of the program (interface functions, content, crashes), or the user set it aside (joint skills, the DLC). It is kept so that the complaint is on record, with the reason in Why. It is never used for a balance claim that is merely hard to fix</t>
+          <t>The row is not a claim about balance, or it can only be answered by new behaviour of the program (interface functions, content, crashes), or it was set aside (joint skills, the DLC). It is kept so that the complaint is on record, with the reason in Why. It is never used for a balance claim that is merely hard to fix</t>
         </is>
       </c>
     </row>
@@ -21877,7 +21877,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>My proposal on whether the row deserves work, for the rows of JP search 2: yes; yes, small; to decide in the diagnosis; no. The user decides.</t>
+          <t>My proposal on whether the row deserves work, for the rows of JP search 2: yes; yes, small; to decide in the diagnosis; no. the decision is taken on.</t>
         </is>
       </c>
     </row>
@@ -21889,7 +21889,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>A search of Japanese player complaints made by another agent for the user on 2026-10-05 (reviews, boards, wikis, blogs). The user asked to take it with a grain of salt: players exaggerate and do not ask for exactly what they need. A complaint is treated at its root and only if it hurts the game; the mod eases the worst of the game without taking its charm; large changes to the program rank last. Entries that already had a row were added to its Also_Raised_By; the rest are rows S01 to S27 with Worth_It and Why. The text file was deleted after filing.</t>
+          <t>A search of Japanese player complaints made by another agent on 2026-10-05 (reviews, boards, wikis, blogs). It was asked to take it with a grain of salt: players exaggerate and do not ask for exactly what they need. A complaint is treated at its root and only if it hurts the game; the mod eases the worst of the game without taking its charm; large changes to the program rank last. Entries that already had a row were added to its Also_Raised_By; the rest are rows S01 to S27 with Worth_It and Why. The text file was deleted after filing.</t>
         </is>
       </c>
     </row>
@@ -22423,12 +22423,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>The cases each change touches (its check), and every boss of the story and the postgame with the reference parties in the final pass (BALANCE_PLAN.md section 3, approach of 2026-10-07)</t>
+          <t>The cases each change touches (its check), and every boss of the story and the postgame with the reference parties in the final pass (the project notes section 3, approach of 2026-10-07)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PARTY_BATTERY.md: no party wins everywhere more than the best of vanilla did; the weakest party of vanilla (Anti-Meta-Plus, 0 - 14% at eight bosses) reaches 29 - 100%, still the weakest. CLASS_STAGES.md: 74 of 76 rows within the band. Limit: the band has no top, so a class that is too fast is not flagged (the Witch fights at 0.59 of the median attacker at the advanced stage; row J11, left by the user)</t>
+          <t>PARTY_BATTERY.md: no party wins everywhere more than the best of vanilla did; the weakest party of vanilla (Anti-Meta-Plus, 0 - 14% at eight bosses) reaches 29 - 100%, still the weakest. CLASS_STAGES.md: 74 of 76 rows within the band. Limit: the band has no top, so a class that is too fast is not flagged (the Witch fights at 0.59 of the median attacker at the advanced stage; row J11, left)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -22482,7 +22482,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Where vanilla asks for a jump of level (the reference level rises from one checkpoint to the next, or a boss stands above the level of its route), the jump stays in the same place: none is removed and none grows; a large one may be softened. No new jump appears. A change upstream (EXP, enemies, catch-up) moves every level after it, so the whole curve is checked, not each checkpoint alone (the user, 2026-10-07)</t>
+          <t>Where vanilla asks for a jump of level (the reference level rises from one checkpoint to the next, or a boss stands above the level of its route), the jump stays in the same place: none is removed and none grows; a large one may be softened. No new jump appears. A change upstream (EXP, enemies, catch-up) moves every level after it, so the whole curve is checked, not each checkpoint alone (decided 2026-10-07)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -22652,7 +22652,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>DIFFICULTY_CURVE.md: 37 of 44 checkpoints within the windows of vanilla, 7 easier (C14, C26, C29, C30, C32, C37, C38), 0 harder. The user, 2026-10-11: the bosses the variant leaves easier stay as they are. C40, raised as an exception, is within (wins 88% &gt; 95%, length 35.5 &gt; 34.2). Limit found the same day: Heretic Samsara of Demiurge is not played by the model, in vanilla or on the variant</t>
+          <t>DIFFICULTY_CURVE.md: 37 of 44 checkpoints within the windows of vanilla, 7 easier (C14, C26, C29, C30, C32, C37, C38), 0 harder. Decided 2026-10-11: the bosses the variant leaves easier stay as they are. C40, raised as an exception, is within (wins 88% &gt; 95%, length 35.5 &gt; 34.2). Limit found the same day: Heretic Samsara of Demiurge is not played by the model, in vanilla or on the variant</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -22701,7 +22701,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>A fight stays an exchange: the enemy still threatens the party and the party has to answer. No change gives the player an excess of power; options widen because what was broken is fixed, not because the party is stronger (the user, 2026-10-07)</t>
+          <t>A fight stays an exchange: the enemy still threatens the party and the party has to answer. No change gives the player an excess of power; options widen because what was broken is fixed, not because the party is stronger (decided 2026-10-07)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -23257,7 +23257,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The user allows it; the risk is an effect the code does not expect in that kind of skill</t>
+          <t>Allowed; the risk is an effect the code does not expect in that kind of skill</t>
         </is>
       </c>
     </row>
@@ -23659,7 +23659,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Decision of the user: only when it can be confirmed</t>
+          <t>Decision of decided: only when it can be confirmed</t>
         </is>
       </c>
     </row>
@@ -24584,7 +24584,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Data only. EXP per level of the earlier proposal the user asked to keep, through the five steps he gave (level, share of vanilla)</t>
+          <t>Data only. EXP per level of the earlier proposal it was asked to keep, through the five steps he gave (level, share of vanilla)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: stat DOWN enchantments show -10%, Provoke level 1 back to the game's value
The six stat DOWN enchantments take away int(stat / 10), read at 0x4f857e; the text said -5% from a guide. Provoke level 1 was below the game (200 against 250): the row is dropped, the rows of levels 2 to 5 are filed under the complaint about Provoke with what was measured. Two measures added: Provoke by size, and the second enchantment of five grand sealbooks.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -5442,7 +5442,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>not a problem</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
@@ -5457,12 +5457,12 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>S033 - S036: the enmity of Provoke grows with its level (250 at level 1, 1500 at level 5)</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>2026-10-09: not a problem</t>
+          <t>2026-10-09: not a problem | 2026-10-13: the rows that raise it by level were already built under another complaint; they are filed here, level 1 put back to the value of the game, and measured (no boss moves)</t>
         </is>
       </c>
     </row>
@@ -14283,7 +14283,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -21856,7 +21855,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -24218,7 +24216,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
@@ -24784,7 +24781,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -24954,7 +24950,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
balance: two grand sealbooks lose their TP cut, EXP factor near the enemy level 1.15
The second enchantment of the books of Samael and Sukuna-Hikona cut the TP cost of the whole party by a fifth: with the second a long fight went from 36 to 27 turns. Both rows dropped; the other three stay, measured. The EXP factor of a member 1 to 4 levels below the enemy goes from 1.25 to 1.15. The patch tool also finds a program file it patched before when a row has changed since.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -13788,18 +13788,18 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>a4936d00</t>
+          <t>9c936d00</t>
         </is>
       </c>
       <c r="G2" t="n">
         <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>1.25</v>
+        <v>1.15</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>EXP factor by gap (member level - enemy level): 1 to 4 below the enemy, no piece</t>
+          <t>EXP factor by gap (member level - enemy level): 1 to 4 below the enemy, no piece. 1.15 since 2026-10-13 (it was 1.25): a little less grind near the level of the enemies, closer to the game; the float is the one the game holds for the piece of enchantment 270 in this band</t>
         </is>
       </c>
     </row>
@@ -24718,12 +24718,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.85, 0.9, 1, 1.25, 3, 5, 10</t>
+          <t>0.85, 0.9, 1, 1.15, 3, 5, 10</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>What is installed since 2026-10-11: the factors by gap of B4 in the program, the EXP of a level as in vanilla</t>
+          <t>What is installed: the factors by gap of B4 in the program (1.15 from 1 level below the enemy since 2026-10-13, 1.25 before), the EXP of a level as in vanilla</t>
         </is>
       </c>
     </row>
@@ -24781,6 +24781,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
data: the register and the regression sheet brought up to the last pass
Rows closed with no figure get the one read from the data (boss dispels, weaknesses); the 17 that rest on an argument are listed by tools/verdicts.py. The levers seen working are marked so, stale and personal wording is gone, and the results of the regression sheet carry the pass of 2026-10-13.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -1262,7 +1262,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>2026-10-09: no change (the user keeps the early misses)</t>
+          <t>2026-10-09: no change (the early misses are kept)</t>
         </is>
       </c>
     </row>
@@ -1697,6 +1697,11 @@
           <t>P01, P02, P03, P09, P10, P12, P13, P15</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>An attack that removes buffs (effect 74: after the hit lands, a roll under its value) is carried by an enemy of 8 of the 40 boss fights of the story (C22, C26, C29, C31, C33, C34, C39, C40) and of 40 of the 55 of the postgame (the attacks of each enemy, data of the game, counted on 2026-10-13)</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -1704,7 +1709,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Dispel costs the boss an entire turn dealing zero damage; short-term buffs and fast chants remain optimal burst windows.</t>
+          <t>True of the postgame, not of the story. The removal rides on a hit that also deals its damage, so it costs the boss nothing; what keeps a buff worth its turn is its length against how often that attack is picked, and the buffs measured still pay (docs/generated/SKILL_VALUE.md). Left as the game has it: it is what makes the postgame bosses different from the story ones</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1715,6 +1720,11 @@
       <c r="P16" t="inlineStr">
         <is>
           <t>partly true</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>2026-10-13: no change</t>
         </is>
       </c>
     </row>
@@ -8078,7 +8088,7 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>partly true: songs compete for two slots with Carol and March</t>
+          <t>partly true: songs compete for two slots with Carol and March; measured +0% of length and of wins at the bosses of the reference party (docs/generated/SKILL_VALUE.md), where little damage is magic</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -9468,7 +9478,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>Joint skills require specific party rosters and TP/gauge investment; parked by user decision</t>
+          <t>Joint skills ask for specific members in the party and for TP and gauge; parked (decided 2026-10-04)</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -10248,6 +10258,11 @@
           <t>P18</t>
         </is>
       </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>The enemy with most HP of a boss fight has a resistance below 0 in 26 of the 40 fights of the story (down to -75 at C17, -50 at C08, C20 and C22) and in 4 of the 55 of the postgame (P36 -50, P07 and P22 -30, P39 -25): data of the game, counted on 2026-10-13</t>
+        </is>
+      </c>
       <c r="L134" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -10255,7 +10270,7 @@
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>Exploiting enemy elemental affinities with zone synergy is the primary intended combat puzzle for magical and hybrid party setups.</t>
+          <t>A weakness is common early and rare where the claim places it: 4 of the 55 postgame fights. Each point below 0 adds half a percent of damage (docs/FORMULAS.md 2.4), so -50 is a quarter more, not a trivial fight</t>
         </is>
       </c>
       <c r="O134" t="inlineStr">
@@ -10266,6 +10281,11 @@
       <c r="P134" t="inlineStr">
         <is>
           <t>partly true</t>
+        </is>
+      </c>
+      <c r="R134" t="inlineStr">
+        <is>
+          <t>2026-10-13: no change</t>
         </is>
       </c>
     </row>
@@ -12083,7 +12103,7 @@
       </c>
       <c r="N158" t="inlineStr">
         <is>
-          <t>A future idea of the user (2026-10-07): complex, interesting for later. Not evaluated and nothing is opened for it. The QoL variant already shows the speed and chant of every skill</t>
+          <t>An idea for later (2026-10-07): complex and interesting. Not evaluated and nothing is opened for it. The QoL variant already shows the speed and chant of every skill</t>
         </is>
       </c>
       <c r="O158" t="inlineStr">
@@ -12207,7 +12227,7 @@
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t>Content and maps are out of the balance. The conditions of side events, which are only text, are being evaluated as an addition to the QoL variant, reopened for it (docs/QOL_ROADMAP.md, last section; decided 2026-10-07)</t>
+          <t>Content and maps are out of the balance. The conditions of side events, which are only text, were looked at as an addition to the QoL variant and dropped on 2026-10-12</t>
         </is>
       </c>
       <c r="O160" t="inlineStr">
@@ -12269,7 +12289,7 @@
       </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t>Not for now: very specific, and the user has seen almost nobody report it (2026-10-07). Reports from the console versions and early patches; none reproduced here</t>
+          <t>Not for now: very specific, and almost nobody reports it (2026-10-07). Reports from the console versions and early patches; none reproduced here</t>
         </is>
       </c>
       <c r="O161" t="inlineStr">
@@ -21779,7 +21799,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Definition of the user (2026-10-05): every row of Criticisms is "closed" or "not a problem", AND every row of Regression holds on the built variant. Closing the known criticisms is not enough: a fix that makes something else dominant must be caught, and nobody complained about it in vanilla.</t>
+          <t>Defined on 2026-10-05: every row of Criticisms is "closed" or "not a problem", AND every row of Regression holds on the built variant. Closing the known criticisms is not enough: a fix that makes something else dominant must be caught, and nobody complained about it in vanilla.</t>
         </is>
       </c>
     </row>
@@ -22394,7 +22414,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Result (final pass, 2026-10-11)</t>
+          <t>Result (final pass; the date of each row is in it)</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -22426,7 +22446,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PARTY_BATTERY.md: no party wins everywhere more than the best of vanilla did; the weakest party of vanilla (Anti-Meta-Plus, 0 - 14% at eight bosses) reaches 29 - 100%, still the weakest. CLASS_STAGES.md: 74 of 76 rows within the band. Limit: the band has no top, so a class that is too fast is not flagged (the Witch fights at 0.59 of the median attacker at the advanced stage; row J11, left)</t>
+          <t>2026-10-13. measures/WIN_RATES.md (200 battles): the three parties that work in the game end level, Meta 92%, Dual-Support 91%, Mage-Heavy 94% of wins over the 17 bosses of the battery (85%, 89%, 90% in the game); Meta, the one that gains most, was the weakest of the three at C26, C30 and C38 in the game. The weakest party of the game (Anti-Meta-Plus, 0 - 12% at eight bosses) reaches 41 - 100%. CLASS_STAGES.md: 74 of 76 rows within the band. Limit: the band has no top, so a class that is too fast is not flagged (row J11, left)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -22458,7 +22478,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PARTY_BATTERY.md: 64 of 85 pairs at or above the floor in vanilla, 76 of 85 on the variant; no pair that met its floor in vanilla lost it. CLASS_STAGES.md: the two slow rows (Assassin and Treasure Hunter of the treasure hunter role) were slow before the changes (row J26)</t>
+          <t>2026-10-13. PARTY_BATTERY.md: 65 of 85 pairs at or above the floor in vanilla, 74 of 85 on the variant; no pair that met its floor in vanilla lost it. CLASS_STAGES.md: the two slow rows (Assassin and Treasure Hunter of the treasure hunter role) were slow before the changes (row J26)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -22586,7 +22606,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BALANCE_BUILD.md: 1,386 of 1,386 live rows built, and each names the row it serves (column Serves, none empty)</t>
+          <t>2026-10-13. BALANCE_BUILD.md: 1,456 of 1,456 live rows built, and each names the row it serves (column Serves, none empty)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -22650,12 +22670,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>DIFFICULTY_CURVE.md: 37 of 44 checkpoints within the windows of vanilla, 7 easier (C14, C26, C29, C30, C32, C37, C38), 0 harder. Decided 2026-10-11: the bosses the variant leaves easier stay as they are. C40, raised as an exception, is within (wins 88% &gt; 95%, length 35.5 &gt; 34.2). Limit found the same day: Heretic Samsara of Demiurge is not played by the model, in vanilla or on the variant</t>
+          <t>2026-10-13. DIFFICULTY_CURVE.md (40 battles a boss): 33 of 44 checkpoints within the windows of vanilla, 11 easier (C14, C15, C17, C26, C28, C29, C32, C37, C38, C39, C40), 0 harder. Seven of them were accepted on 2026-10-11; C30 is back within with its HP x1.15, and C38 keeps 92% of wins against 70% with the same. C15, C17, C28, C39 and C40 crossed their window since then by one measure each (length, wins or lowest HP), which at 40 battles may be chance (measures/curve_ablation.py settles it with more battles)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>met; 7 bosses easier, accepted</t>
+          <t>met but for 11 bosses easier: 6 accepted, 5 since then not decided</t>
         </is>
       </c>
     </row>
@@ -22677,12 +22697,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>VERDICTS.md: of 162 rows, 72 closed with the figure before and after, 77 not a problem with their figure, 12 out of the balance, 1 open (J02, left for the postgame)</t>
+          <t>2026-10-13. VERDICTS.md: of 180 rows, 80 closed, 88 not a problem, 12 out of the balance, 0 open. 17 of them are closed on an argument with no figure (listed at the end of VERDICTS.md)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>met</t>
+          <t>met; 17 rows rest on an argument</t>
         </is>
       </c>
     </row>
@@ -22709,7 +22729,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>DIFFICULTY_CURVE.md, columns Lowest HP and Pressure: inside the window of vanilla at 37 of 44 checkpoints; where they leave it the party stands higher (lowest HP 11 - 31% &gt; 22 - 53% at C29, C30, C38), never lower. SIM_ANCHORS.md: 6 of 6 anchors met</t>
+          <t>2026-10-13. DIFFICULTY_CURVE.md, columns Lowest HP and Pressure: where a checkpoint leaves the window of vanilla the party stands higher (lowest HP 31 - 48% &gt; 49 - 61% at C32, C38, C39, C40), never lower; pressure is above the window at C26 alone (0.07 &gt; 0.10). SIM_ANCHORS.md: 6 of 6 anchors met</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -23657,7 +23677,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Decision of decided: only when it can be confirmed</t>
+          <t>Decided: only when it can be confirmed</t>
         </is>
       </c>
     </row>
@@ -24383,7 +24403,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>tools/text_checks.py PARTY_EFFECT; the bonus of each effect is worked out at 0x4f9000 - 0x4f94e6. Not seen working in the game yet</t>
+          <t>tools/text_checks.py PARTY_EFFECT; the bonus of each effect is worked out at 0x4f9000 - 0x4f94e6. Seen working in the game (play-tested, 2026-10-12)</t>
         </is>
       </c>
     </row>
@@ -24420,7 +24440,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 12.19; the unique skills are looked up as any status (0x47e340 on the lists of the blow function). Not seen working in the game yet</t>
+          <t>docs/FORMULAS.md 12.19; the unique skills are looked up as any status (0x47e340 on the lists of the blow function). Seen working in the game (play-tested, 2026-10-12)</t>
         </is>
       </c>
     </row>
@@ -24457,7 +24477,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>tools/npc_data.py (the stats are read at 0x4fed59 - 0x4fee27). Not seen working in the game yet</t>
+          <t>tools/npc_data.py (the stats are read at 0x4fed59 - 0x4fee27). Seen working in the game (play-tested, 2026-10-12)</t>
         </is>
       </c>
     </row>
@@ -24494,7 +24514,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 2.5: the only reader of effect 264 as a status is 0x44cfad. Not seen working in the game yet</t>
+          <t>docs/FORMULAS.md 2.5: the only reader of effect 264 as a status is 0x44cfad. Seen working in the game (play-tested, 2026-10-12)</t>
         </is>
       </c>
     </row>
@@ -24781,7 +24801,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
data: seven rows closed on an argument get their measure
Area spikes, forging, forged against unique, harmful zones, the early economy and the anti-magic bosses carry the figure their test asks for (measures/design_rows.py); meals stay unmeasured. Five bosses that crossed their window are checked with 200 battles: three were chance.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -1836,6 +1836,11 @@
           <t>P03, P04, P07, P09, P10, P13</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>The reference party at the 40 boss fights of the story, 30 battles each: the largest damage of one enemy action on one member is above the whole HP of the frailest member in the median battle of 12 fights (C26, C29, C30, C31, C32, C34 to C40; 119% to 201% of her HP) and at least once in 18. Before C26 it stays below (40% to 94%) (measures/DESIGN_ROWS.md, 2026-10-13)</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -1843,7 +1848,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Cover (Valkyrie) and Phalanx (Paladin) are designed precisely to protect fragile backline casters from lethal AoE spikes.</t>
+          <t>From C26 on one enemy action can fell the frailest member from full HP in most battles, with Cover and the guards played. It is what makes the Valkyrie and the Paladin worth their place (rows J04, F07); nothing was changed for it</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -1853,7 +1858,12 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>partly true</t>
+          <t>true from C26 on</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>2026-10-13: measured; the claim holds. No change so far: the state waits for a decision</t>
         </is>
       </c>
     </row>
@@ -3227,6 +3237,11 @@
           <t>P04, P07, P10, P15, P19</t>
         </is>
       </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Each upgrade level adds int(level * rate) to every stat of the piece: for the 17 weapons that take levels, 5.4% to 9.7% of base ATK a level (median 6.3%), not one percent. Only 29 of the 551 pieces take levels at all. What a level costs in gold is in the program and was not read (measures/DESIGN_ROWS.md, 2026-10-13)</t>
+        </is>
+      </c>
       <c r="L36" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -3234,7 +3249,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Forging costs scale quadratically as an endgame gold sink; S16 complains of the opposite (forged gear being too strong). Progression functions as intended.</t>
+          <t>A level is worth about 6% of the base ATK of the weapon, and the levels add up (a Claymore goes from 37 to 312 ATK at the top level). The half of the claim about the price is not answered</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -3244,7 +3259,12 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>false on the size of the bonus; its cost not measured</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>2026-10-13: no change</t>
         </is>
       </c>
     </row>
@@ -3289,6 +3309,11 @@
           <t>P10, P13</t>
         </is>
       </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Of the 16 meals, 4 only restore HP or TP or cure, at once, and 12 also give a buff (a skill at a fixed level). How many steps that buff lasts is in the program and was not read, so the test of this row is not answered (measures/DESIGN_ROWS.md, 2026-10-13)</t>
+        </is>
+      </c>
       <c r="L37" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -3296,7 +3321,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Meals provide pre-dungeon or mid-dungeon prep; cooking and eating items near boss rooms or utilizing long-duration food recipes addresses boss preparation.</t>
+          <t>A quarter of the meals have nothing that could run out. For the other twelve the length of the buff is not known here</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -3306,7 +3331,12 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>not measured</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>2026-10-13: left; it needs a reading of the program</t>
         </is>
       </c>
     </row>
@@ -10196,6 +10226,11 @@
           <t>P04, P07, P10, P11, P13</t>
         </is>
       </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Boss fights on a cell that forbids magic: C29a in the story, P07, P13, P25 and P47 in the postgame. C29a is won without her (Dual-Support 100%). In the postgame the same party with and without the Treasure Hunter, 100 battles: Meta 57% &gt; 18% at P13 and 96% &gt; 76% at P25; Dual-Support with her in the place of the shooter 14% &gt; 43% and 52% &gt; 75%; at P07 she changes nothing (97% &gt; 95%, 3% &gt; 3%) and nobody wins P47 (measures/DESIGN_ROWS.md, 2026-10-13)</t>
+        </is>
+      </c>
       <c r="L133" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -10203,7 +10238,7 @@
       </c>
       <c r="N133" t="inlineStr">
         <is>
-          <t>Non-magic healing through Bard/Diva songs, Maid cooking, and consumables prevents Treasure Hunter from being mandatory.</t>
+          <t>She helps where magic is shut, as the guide says, but a party wins P07 and P25 without her (Meta 95% and 76%)</t>
         </is>
       </c>
       <c r="O133" t="inlineStr">
@@ -10213,7 +10248,12 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>partly true</t>
+          <t>partly true: she adds 20 to 40 points of wins at two of the four postgame fights, and is not needed in the story</t>
+        </is>
+      </c>
+      <c r="R133" t="inlineStr">
+        <is>
+          <t>2026-10-13: no change</t>
         </is>
       </c>
     </row>
@@ -11463,6 +11503,11 @@
           <t>P18</t>
         </is>
       </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Of the 103 floors, 20 have cells that forbid magic and 26 cells that lower physical or magic attack; where a floor has them they cover a median of 10% and 16% of the cells of its map (walls counted), at most 36% and 44%. A lowering zone multiplies attack by 0.5 to 0.75, for both sides (measures/DESIGN_ROWS.md, 2026-10-13)</t>
+        </is>
+      </c>
       <c r="L149" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -11475,7 +11520,7 @@
       </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t>Anti-magic, darkness, and damage tiles are core dungeon crawling hazards with dedicated counterplay (Light spell, levitate/cushion items, Grand Sealbook Sahohime).</t>
+          <t>The zones weigh on both sides alike and cover a small part of the floors that have them. Maps are out of what the variant changes</t>
         </is>
       </c>
       <c r="O149" t="inlineStr">
@@ -11485,7 +11530,12 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>a matter of taste; the figure: a fifth to a quarter of the floors, a tenth to a sixth of their cells</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>2026-10-13: no change</t>
         </is>
       </c>
     </row>
@@ -11597,6 +11647,11 @@
           <t>P15, P19</t>
         </is>
       </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>The best weapon that takes levels, at the highest level a zone gives (99), has less ATK than the best fixed piece in each of the 10 weapon types (Claymore 312 against Amenomurakumo 433, Heavy Axe 361 against Adamas Greatscythe 462, Kukri 137 against Kali Kukri 279). The fixed pieces carry 1 to 4 enchantments of their own; the chosen enchantments of a forged piece are not weighed here (measures/DESIGN_ROWS.md, 2026-10-13)</t>
+        </is>
+      </c>
       <c r="L151" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -11609,7 +11664,7 @@
       </c>
       <c r="N151" t="inlineStr">
         <is>
-          <t>Contradicts J35. Unique postgame weapons feature distinct innates and higher base stats; forged gear provides customization flexibility without invalidating unique top-tier drops.</t>
+          <t>On attack the unique pieces stay ahead to the end, by 20% to 140%. Whether three or four chosen enchantments make up for it is not measured</t>
         </is>
       </c>
       <c r="O151" t="inlineStr">
@@ -11619,7 +11674,12 @@
       </c>
       <c r="P151" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>false on ATK; the enchantments not compared</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>2026-10-13: no change</t>
         </is>
       </c>
     </row>
@@ -11813,6 +11873,11 @@
           <t>P13</t>
         </is>
       </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>A random battle of the first two dungeons gives 5 to 18 gold and of the next two 27 to 88, against 90 for the cheapest healing item (Croissant), 180 for an Egg Sandwich and 450 for a Danish; a piece sells for a third of its price. The prices of equipment are not decoded (measures/DESIGN_ROWS.md, 2026-10-13)</t>
+        </is>
+      </c>
       <c r="L154" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -11825,7 +11890,7 @@
       </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t>Early game resource scarcity is intentional survival tension in dungeon crawlers; early story quests and enemy drops provide adequate funds for baseline gear.</t>
+          <t>Battles pay little at the start; quests are where the early gold comes from, and the variant raises the gold of every quest by 40% (row S20)</t>
         </is>
       </c>
       <c r="O154" t="inlineStr">
@@ -11835,7 +11900,12 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>partly true: five to eighteen battles pay one basic heal at the start</t>
+        </is>
+      </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>2026-10-13: answered in part by the rows of S20; nothing more</t>
         </is>
       </c>
     </row>
@@ -22670,12 +22740,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-10-13. DIFFICULTY_CURVE.md (40 battles a boss): 33 of 44 checkpoints within the windows of vanilla, 11 easier (C14, C15, C17, C26, C28, C29, C32, C37, C38, C39, C40), 0 harder. Seven of them were accepted on 2026-10-11; C30 is back within with its HP x1.15, and C38 keeps 92% of wins against 70% with the same. C15, C17, C28, C39 and C40 crossed their window since then by one measure each (length, wins or lowest HP), which at 40 battles may be chance (measures/curve_ablation.py settles it with more battles)</t>
+          <t>2026-10-13. DIFFICULTY_CURVE.md (40 battles a boss): 33 of 44 checkpoints within the windows of vanilla, 11 easier, 0 harder. Six were accepted on 2026-10-11 (C14, C26, C29, C32, C37, C38); C30 is back within with its HP x1.15. The five that crossed since then, with 200 battles (measures/curve_recheck.py): C15, C28 and C39 are within, it was chance; C17 is 28% shorter (49.1 &gt; 35.4, wins 100% both) and C40 is won more (85% &gt; 97%)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>met but for 11 bosses easier: 6 accepted, 5 since then not decided</t>
+          <t>met but for 8 bosses easier: 6 accepted, C17 and C40 not decided</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: the wandering shops of a zone read; Sacred Hymn and Ecstasy measured
The five special chances of a zone are the peddler, the blacksmith, the ice cream and ramen shops and the dark peddler, with the conditions under which each is rolled. Ecstasy adds nothing that can be measured; Sacred Hymn serves at the last boss. C17 and C40 are accepted as easier.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -3321,7 +3321,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>A quarter of the meals have nothing that could run out. For the other twelve the length of the buff is not known here</t>
+          <t>A quarter of the meals have nothing that could run out. For the other twelve the buff is the skill itself, performed at a fixed level by the ordinary skill action (0x50b030, 0x41d2b0); what ends it outside a battle was looked for on 2026-10-13 and not found (the list emptied every 100 steps at 0x4b92ed holds the shops that appeared, not the buffs)</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>2026-10-13: left; it needs a reading of the program</t>
+          <t>2026-10-13: read in part; the length of the buff is still not known</t>
         </is>
       </c>
     </row>
@@ -8106,11 +8106,21 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>The Maid of the reference party without the song and with it at its top level: wins 84% &gt; 91% and HP left 82% &gt; 88% at C40, 93% &gt; 95% at C26, no change at C30, C36 and C38; the length of the fights does not move (measures/one_skill_trial.py, 150 battles, 2026-10-13)</t>
+        </is>
+      </c>
       <c r="L103" t="inlineStr">
         <is>
           <t>not a problem</t>
         </is>
       </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>A song of RES is worth its slot where the boss casts: the last one. Elsewhere Carol and March are better uses of the two slots</t>
+        </is>
+      </c>
       <c r="O103" t="inlineStr">
         <is>
           <t>T06 Skills</t>
@@ -8118,7 +8128,7 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>partly true: songs compete for two slots with Carol and March; measured +0% of length and of wins at the bosses of the reference party (docs/generated/SKILL_VALUE.md), where little damage is magic</t>
+          <t>partly true: it serves at the last boss alone</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -8128,7 +8138,7 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>2026-10-09: not a problem</t>
+          <t>2026-10-13: measured; no change</t>
         </is>
       </c>
     </row>
@@ -8451,11 +8461,21 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>The passive gives ATK and DEX +10% to +15% for 3 turns, once a battle, the first time its bearer falls below half her HP (EffectRules 312); its statuses (41, 45) are not those of War Cry (161), so they add. The Mistress without it and with it at its top level: wins within 2 points and length within 2% at C26, C30, C36, C38 and C40 (measures/one_skill_trial.py, 150 battles, 2026-10-13)</t>
+        </is>
+      </c>
       <c r="L108" t="inlineStr">
         <is>
           <t>not a problem</t>
         </is>
       </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>Three turns once a battle are too little at that size. At 30% to 50% the fights of C30 and C40 are 5% to 8% shorter; at 60% to 100%, 8% to 10% (the same measure with the values changed)</t>
+        </is>
+      </c>
       <c r="O108" t="inlineStr">
         <is>
           <t>T06 Skills</t>
@@ -8463,7 +8483,7 @@
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>false in the model: Ecstasy raises its own ATK and DEX statuses, which stack with War Cry</t>
+          <t>true, for another reason: it stacks with War Cry but adds nothing that can be measured</t>
         </is>
       </c>
       <c r="Q108" t="inlineStr">
@@ -8473,7 +8493,7 @@
       </c>
       <c r="R108" t="inlineStr">
         <is>
-          <t>2026-10-09: not a problem</t>
+          <t>2026-10-13: measured; a dead passive as the game has it. Whether to raise it waits for a decision</t>
         </is>
       </c>
     </row>
@@ -22740,12 +22760,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-10-13. DIFFICULTY_CURVE.md (40 battles a boss): 33 of 44 checkpoints within the windows of vanilla, 11 easier, 0 harder. Six were accepted on 2026-10-11 (C14, C26, C29, C32, C37, C38); C30 is back within with its HP x1.15. The five that crossed since then, with 200 battles (measures/curve_recheck.py): C15, C28 and C39 are within, it was chance; C17 is 28% shorter (49.1 &gt; 35.4, wins 100% both) and C40 is won more (85% &gt; 97%)</t>
+          <t>2026-10-13. DIFFICULTY_CURVE.md (40 battles a boss): 33 of 44 checkpoints within the windows of vanilla, 11 easier, 0 harder. Six were accepted on 2026-10-11 (C14, C26, C29, C32, C37, C38); C30 is back within with its HP x1.15. The five that crossed since then, with 200 battles (measures/curve_recheck.py): C15, C28 and C39 are within, it was chance; C17 is 28% shorter (49.1 &gt; 35.4, wins 100% both) and C40 is won more (85% &gt; 97%). Both accepted on 2026-10-13</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>met but for 8 bosses easier: 6 accepted, C17 and C40 not decided</t>
+          <t>met; 8 bosses easier, accepted</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: the blacksmith appears half again as often, Ecstasy gives twice as much
The chance of the wandering blacksmith is an int of each zone of the floor files: 166 rows of a new table zones, written in place into the packs of the dungeons and put back the same way (tools/floor_patch.py), since those packs are too large to copy. The player installer does the same from the lines poke of its list. Ecstasy goes from 10 - 15% to 20 - 30%.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R181"/>
+  <dimension ref="A1:R182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8466,9 +8466,14 @@
           <t>The passive gives ATK and DEX +10% to +15% for 3 turns, once a battle, the first time its bearer falls below half her HP (EffectRules 312); its statuses (41, 45) are not those of War Cry (161), so they add. The Mistress without it and with it at its top level: wins within 2 points and length within 2% at C26, C30, C36, C38 and C40 (measures/one_skill_trial.py, 150 battles, 2026-10-13)</t>
         </is>
       </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>5 Y rows, ATK and DEX +20% to +30%: the fights of C30 and C40 a little shorter (measures/one_skill_trial.py)</t>
+        </is>
+      </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>not a problem</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -8493,7 +8498,7 @@
       </c>
       <c r="R108" t="inlineStr">
         <is>
-          <t>2026-10-13: measured; a dead passive as the game has it. Whether to raise it waits for a decision</t>
+          <t>2026-10-13: raised to 30% at its top level</t>
         </is>
       </c>
     </row>
@@ -13795,6 +13800,93 @@
       <c r="R181" t="inlineStr">
         <is>
           <t>decided 2026-10-12: raised</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>S28</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Play test</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Blacksmith</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>The wandering blacksmith shows up too seldom to count on her</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Tedium</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Chance that the blacksmith is the next shop to appear in a zone, and the steps it takes</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>Floor files, zone 0x24 (docs/FORMULAS.md 14)</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>Her chance a step is 2 to 10 in the 166 zones that have her (5 to 7 in most), rolled after the battle and after the peddler (3 to 10), only after 5 battles and 50 steps since the last shop, once until the counters of the dungeon are cleared. In a zone at 5 with a peddler at 6 she is the next shop 44% of the times</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>166 Z rows of the table zones, her chance x1.5 rounded (3 to 15): in the same zone she is the next shop 56% of the times. The waits of 5 battles and 50 steps are the program's and stay</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>yes, small</t>
+        </is>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>More often everywhere, and not much: the peddler keeps his turn and the waits stay</t>
+        </is>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>T10 Forge, enchantments and sealbooks</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>Her chance x1.5 in every zone (L46)</t>
+        </is>
+      </c>
+      <c r="R182" t="inlineStr">
+        <is>
+          <t>2026-10-13: approved (more often in general, not too high)</t>
         </is>
       </c>
     </row>
@@ -22839,7 +22931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -24326,6 +24418,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
@@ -24605,6 +24698,43 @@
       <c r="G52" t="inlineStr">
         <is>
           <t>docs/FORMULAS.md 2.5: the only reader of effect 264 as a status is 0x44cfad. Seen working in the game (play-tested, 2026-10-12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>L46</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Chance a step of a wandering shop of a zone (peddler, blacksmith, ice cream, ramen, dark peddler)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Dungeon/stNN/Data.pck floor file</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>zone 0x20 - 0x30, five ints</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>A whole number from 1 to 100; a zone with 0 keeps 0. Written in place and put back the same way (tools/floor_patch.py): the packs are not copied</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 14: each is rolled against a number below 100 on a step (0x4bc8a1 - 0x4bcb77), as the chance of a battle (L29)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: a meal lasts 15 to 50 steps, the row of the register measured
The buff of a meal is the status of a skill at a fixed level and a turn of a status is five steps on the map, so the ten meals that give one last about one battle.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -3311,7 +3311,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Of the 16 meals, 4 only restore HP or TP or cure, at once, and 12 also give a buff (a skill at a fixed level). How many steps that buff lasts is in the program and was not read, so the test of this row is not answered (measures/DESIGN_ROWS.md, 2026-10-13)</t>
+          <t>Of the 16 meals, 10 give a buff: the status of a skill at a fixed level, with the turns of that skill (3 to 10). On the map a turn of a status is 5 steps (docs/FORMULAS.md 12.18), so a meal lasts 15 to 50 steps, and in a battle each action of its bearer takes a turn off it. The mean walk between two random battles is 18 to 28 steps (measures/DESIGN_ROWS.md, 2026-10-13)</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>A quarter of the meals have nothing that could run out. For the other twelve the buff is the skill itself, performed at a fixed level by the ordinary skill action (0x50b030, 0x41d2b0); what ends it outside a battle was looked for on 2026-10-13 and not found (the list emptied every 100 steps at 0x4b92ed holds the shops that appeared, not the buffs)</t>
+          <t>The shop appears where the roll of a step puts it, and its buff is gone a battle later: it reaches a boss only when the shop appears at its door. The turns are those of the skills themselves, and the five steps a turn are one byte of the program that every status of the map shares (ailments too)</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>not measured</t>
+          <t>true: a meal lasts 15 to 50 steps, about one battle</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>2026-10-13: read in part; the length of the buff is still not known</t>
+          <t>2026-10-13: measured; the claim holds. No change so far: the state waits for a decision</t>
         </is>
       </c>
     </row>
@@ -24418,7 +24418,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
balance: a turn of a status takes 20 steps of the map, so a meal lasts
One byte of the program (row X15, lever L47): the count of steps of the statuses with a number of turns, used only outside a battle. A meal goes from 15 - 50 steps to 60 - 200. The ailments that end on a roll and petrification have their own counts and are left.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -3314,14 +3314,19 @@
           <t>Of the 16 meals, 10 give a buff: the status of a skill at a fixed level, with the turns of that skill (3 to 10). On the map a turn of a status is 5 steps (docs/FORMULAS.md 12.18), so a meal lasts 15 to 50 steps, and in a battle each action of its bearer takes a turn off it. The mean walk between two random battles is 18 to 28 steps (measures/DESIGN_ROWS.md, 2026-10-13)</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Row X15 of the sheet ExePatches: a turn of a status takes 20 steps of the map in the place of 5, so a meal lasts 60 to 200 steps, two to eight random battles of walking. Battles count turns as before</t>
+        </is>
+      </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>not a problem</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>The shop appears where the roll of a step puts it, and its buff is gone a battle later: it reaches a boss only when the shop appears at its door. The turns are those of the skills themselves, and the five steps a turn are one byte of the program that every status of the map shares (ailments too)</t>
+          <t>The buff of a meal was gone a battle later. The count of steps is one byte that only the map uses; with it the buffs and the lowered stats a member carries out of a battle last four times as long on the map too, while poison and the other ailments that end on a roll keep their own count</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -3336,7 +3341,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>2026-10-13: measured; the claim holds. No change so far: the state waits for a decision</t>
+          <t>2026-10-13: approved, 20 steps a turn: a buff with its drawback</t>
         </is>
       </c>
     </row>
@@ -13901,7 +13906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14485,6 +14490,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -14547,6 +14553,43 @@
       <c r="I20" t="inlineStr">
         <is>
           <t>Interruption rate of a blow: max HP * 1.5 times (1 + Concentrate) where the program adds the two (addss -&gt; mulss at 0x44d042; its debug message writes the product). Decided 2026-10-12: mend it for every unit, enemies with the passive too</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>X15</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>L47</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>0x48d5f3</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Steps of the map that count as one turn of a status with a number of turns (cmp dword ptr [esi + 0x2c], 5 at 0x48d5f0, reached only when the tick is not of a battle: the word at +0x40 of its second argument is 0). 5 -&gt; 20: a meal lasts 60 to 200 steps in the place of 15 to 50. Decided 2026-10-13</t>
         </is>
       </c>
     </row>
@@ -22931,7 +22974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -24418,6 +24461,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
@@ -24734,6 +24778,43 @@
       <c r="G53" t="inlineStr">
         <is>
           <t>docs/FORMULAS.md 14: each is rolled against a number below 100 on a step (0x4bc8a1 - 0x4bcb77), as the chance of a battle (L29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>L47</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Steps of the map that count as one turn of a status with a number of turns</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>executable, 0x48d5f3</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>one byte</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Executable</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>A byte from 1 to 127; the same instruction, the same length</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>docs/FORMULAS.md 12.18: the tick of the 97 effects of the class CCommandTurnBase (0x48d590). The ailments that end on a roll (0x48d180, its own count at 0x48d202) and petrification (0x483010) have theirs and are left</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: a turn of a status takes 12 steps of the map, not 20
20 carried the buffs a member walks out of a battle with too far. At 12 a meal lasts 36 to 120 steps.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -3316,7 +3316,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Row X15 of the sheet ExePatches: a turn of a status takes 20 steps of the map in the place of 5, so a meal lasts 60 to 200 steps, two to eight random battles of walking. Battles count turns as before</t>
+          <t>Row X15 of the sheet ExePatches: a turn of a status takes 12 steps of the map in the place of 5, so a meal lasts 36 to 120 steps, one to five random battles of walking. Battles count turns as before</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>The buff of a meal was gone a battle later. The count of steps is one byte that only the map uses; with it the buffs and the lowered stats a member carries out of a battle last four times as long on the map too, while poison and the other ailments that end on a roll keep their own count</t>
+          <t>The buff of a meal was gone a battle later. The count of steps is one byte that only the map uses; with it the buffs and the lowered stats a member carries out of a battle last 2.4 times as long on the map too, which is why it is 12 and not more, while poison and the other ailments that end on a roll keep their own count</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -3341,7 +3341,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>2026-10-13: approved, 20 steps a turn: a buff with its drawback</t>
+          <t>2026-10-13: approved at 12 steps a turn (20 was too strong for the buffs kept out of a battle)</t>
         </is>
       </c>
     </row>
@@ -14584,12 +14584,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>0c</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Steps of the map that count as one turn of a status with a number of turns (cmp dword ptr [esi + 0x2c], 5 at 0x48d5f0, reached only when the tick is not of a battle: the word at +0x40 of its second argument is 0). 5 -&gt; 20: a meal lasts 60 to 200 steps in the place of 15 to 50. Decided 2026-10-13</t>
+          <t>Steps of the map that count as one turn of a status with a number of turns (cmp dword ptr [esi + 0x2c], 5 at 0x48d5f0, reached only when the tick is not of a battle: the word at +0x40 of its second argument is 0). 5 -&gt; 12: a meal lasts 36 to 120 steps in the place of 15 to 50. Decided 2026-10-13 (20 at first, lowered the same day: the buffs a member walks out of a battle with last as much longer)</t>
         </is>
       </c>
     </row>
@@ -24461,7 +24461,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
data: what the audit left open in the workbooks, the player README, the .bat
Rows that named a row of the register that is not theirs name the right one. First Grid keeps its chance and loses the higher SP cost: it adds nothing that can be measured. The opening of Samael is measured (21% to 34% of wins at P23). Rows S07, S08, S20, S22, J32 and S17 say what was measured and decided. The player README lists what it left out, and the .bat files end their lines as Windows wants.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -3021,6 +3021,11 @@
           <t>not a problem</t>
         </is>
       </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Trump Card multiplies her damage (+60% to +150%) and takes her DEF away while it lasts: any hit fells her unless someone covers her. It is the trade the class is built on (docs/CLASS_IDENTITY.md)</t>
+        </is>
+      </c>
       <c r="O33" t="inlineStr">
         <is>
           <t>T05 Classes and mercenaries</t>
@@ -3033,7 +3038,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>2026-10-09: no change; the fragility is the Joker's identity (docs/CLASS_IDENTITY.md)</t>
+          <t>2026-10-09: no change; the fragility is what the Joker is</t>
         </is>
       </c>
     </row>
@@ -10986,7 +10991,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>Witch excels in story (length 0.63, 46 - 68% damage) due to elemental AoE coverage; normalizes in postgame (length 0.98, 39 - 52% damage) where boss elemental resistances rise (CLASS_STAGES.md)</t>
+          <t>CLASS_STAGES.md (2026-10-13): at the advanced stage her fights last 0.61 of those of the median attacker with 46 - 67% of the damage of the party. The peak is one boss: 0.34 at C30, Heartless Avenger, who resists slash, stab and bash at 90, 100 and 90 and the elements at 50 to 100. At C22, C34 and C40 she stands at 0.67 to 0.72; late (P08 - P24) at 0.98</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -11001,7 +11006,7 @@
       </c>
       <c r="N142" t="inlineStr">
         <is>
-          <t>Strong in story by elemental coverage, balanced against physical burst in postgame</t>
+          <t>She is far ahead where the boss shuts physical damage out, which is what a mage is for; elsewhere she is the fastest attacker by a third, and level with the others in the postgame</t>
         </is>
       </c>
       <c r="O142" t="inlineStr">
@@ -11021,7 +11026,7 @@
       </c>
       <c r="R142" t="inlineStr">
         <is>
-          <t>2026-10-10: no change; class identity preserved</t>
+          <t>2026-10-13: not a problem where the boss is the weak one to magic; no change</t>
         </is>
       </c>
     </row>
@@ -11083,7 +11088,7 @@
       </c>
       <c r="N143" t="inlineStr">
         <is>
-          <t>Data: the weapon rank each form names sets its weight, and its six factors its stats (tools/summon_data.py)</t>
+          <t>Its wait is that of the slowest member (median 0.42 at level 90), still sooner than most bosses (0.42 - 0.55): late for a party, not too late to act. Its weight is data of each form (tools/summon_data.py)</t>
         </is>
       </c>
       <c r="O143" t="inlineStr">
@@ -11093,7 +11098,7 @@
       </c>
       <c r="P143" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>partly true: a summon acts like the slowest member of the party</t>
         </is>
       </c>
       <c r="Q143" t="inlineStr">
@@ -11103,7 +11108,7 @@
       </c>
       <c r="R143" t="inlineStr">
         <is>
-          <t>2026-10-09: no change (summons are not of the doll line; they already act like the slowest member)</t>
+          <t>2026-10-09: no change of its speed</t>
         </is>
       </c>
     </row>
@@ -11771,7 +11776,7 @@
       </c>
       <c r="N152" t="inlineStr">
         <is>
-          <t>Executable constant; defensive viability is provided through skills and stats</t>
+          <t>The pieces that cut damage add up to a quarter at most (docs/FORMULAS.md 2.4: never below 0.75); the claim compares it with the half of the first game. It is a constant of the program, and a party defends itself with DEF, guards and Cover, which the cap does not touch</t>
         </is>
       </c>
       <c r="O152" t="inlineStr">
@@ -11791,7 +11796,7 @@
       </c>
       <c r="R152" t="inlineStr">
         <is>
-          <t>2026-10-10: no change; defenses operate via stats and guard skills</t>
+          <t>2026-10-10: no change; raising it would be a patch of the program for a build nobody is missing</t>
         </is>
       </c>
     </row>
@@ -11982,12 +11987,12 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>41 P rows of the table quests, gold reward x1.40, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); EXP for the members behind comes from the factors B4 (U01)</t>
+          <t>The EXP of a quest is not changed. What the variant changes beside it: the gold of the 41 quests that pay gold x1.40 (P rows of the table quests), and the EXP of a member below the level of the enemies (the factors by level gap, sheet ExePatches)</t>
         </is>
       </c>
       <c r="L155" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="M155" t="inlineStr">
@@ -11997,7 +12002,7 @@
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t>Reopened on 2026-10-11: rows P026 - P030 of balance_changes.xlsx, which this verdict leaned on, cannot be written (the figure they took for gold is the id of the item or piece the quest gives; QuestData 0x38 is the kind of the reward) and are blocked; the B4 factors it also names are not built. Quest gold rewards increased by +30% to +50% in QuestData, allowing players to purchase better gear and seals, while underleveled party members catch up rapidly via the B4 EXP curve on quest monsters.</t>
+          <t>Of the 471 quests none pays EXP as its reward in a field the variant writes: the reward is an item, a piece, EXP or gold by its kind (QuestData 0x38), and only gold was raised. The claim stands as the game has it; the members who are behind catch up in battles, not through quests</t>
         </is>
       </c>
       <c r="O155" t="inlineStr">
@@ -12007,12 +12012,12 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>partly true</t>
+          <t>true as stated; not answered by a change of quests</t>
         </is>
       </c>
       <c r="R155" t="inlineStr">
         <is>
-          <t>2026-10-11: approved (quest gold x1.40)</t>
+          <t>2026-10-11: quest gold x1.40 approved; 2026-10-13: the row says that this is not EXP</t>
         </is>
       </c>
     </row>
@@ -12124,6 +12129,16 @@
           <t>P13; which fixed battle it is</t>
         </is>
       </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>The reference party at its level (64), 200 battles: 85% of wins in 33.2 turns in the game, the lowest HP of the party 33% (measures/curve_recheck.py, 2026-10-13). Of the parties of the battery, Mage-Heavy wins 62%, Juggernaut-Plus 19% and the two without a healer none (measures/WIN_RATES.md)</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>On the variant the reference party wins 97% in 31.1 turns: easier, accepted on 2026-10-13 (Regression R08)</t>
+        </is>
+      </c>
       <c r="L157" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -12136,7 +12151,7 @@
       </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t>C40 final story boss Demiurge calibrated to 85% win rate at Lv64 across 41 turns, maintaining intended narrative climax challenge.</t>
+          <t>A wall for a party without a Diva or a healer, not for one built for it: the fight asks for a heal every turn, as the guides say</t>
         </is>
       </c>
       <c r="O157" t="inlineStr">
@@ -12146,7 +12161,12 @@
       </c>
       <c r="P157" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>partly true: won 85% by a prepared party, never by one with no healer</t>
+        </is>
+      </c>
+      <c r="R157" t="inlineStr">
+        <is>
+          <t>2026-10-13: no change of its own; easier on the variant, accepted</t>
         </is>
       </c>
     </row>
@@ -14490,7 +14510,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -22671,7 +22690,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-13. measures/WIN_RATES.md (200 battles): the three parties that work in the game end level, Meta 92%, Dual-Support 91%, Mage-Heavy 94% of wins over the 17 bosses of the battery (85%, 89%, 90% in the game); Meta, the one that gains most, was the weakest of the three at C26, C30 and C38 in the game. The weakest party of the game (Anti-Meta-Plus, 0 - 12% at eight bosses) reaches 41 - 100%. CLASS_STAGES.md: 74 of 76 rows within the band. Limit: the band has no top, so a class that is too fast is not flagged (row J11, left)</t>
+          <t>2026-10-13. measures/WIN_RATES.md (200 battles): the three parties that work in the game end level, Meta 92%, Dual-Support 91%, Mage-Heavy 94% of wins over the 17 bosses of the battery (85%, 89%, 90% in the game); Meta, the one that gains most, was the weakest of the three at C26, C30 and C38 in the game. The weakest party of the game (Anti-Meta-Plus, 0 - 12% at eight bosses) reaches 41 - 100%. CLASS_STAGES.md: 74 of 76 rows within the band. Limit: the band has no top, so a class that is too fast is not flagged (row J11, left). The Witch is the case: 0.61 of the median attacker at the advanced stage, 0.34 at C30 alone, a boss that resists physical damage at 90 - 100 (row S07, decided 2026-10-13: not a problem there)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>

<commit_message>
data: why Samael opens another way is written in its rows
The opening of the postgame Samael was unfair: a spell on the whole party before any guard could be up. Row F86 and row P038 say so, with the measure.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -3038,7 +3038,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>2026-10-09: no change; the fragility is what the Joker is</t>
+          <t>2026-10-09: no change; 2026-10-13, confirmed: the fragility is the flavour of the class</t>
         </is>
       </c>
     </row>
@@ -9618,6 +9618,16 @@
           <t>P03, P04, P07, P08, P09, P10, P13</t>
         </is>
       </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>The Samael of the postgame (P23) casts Dark Blast on the whole party on its first turn, every time (the weights of its first set of attacks: slot 6 alone). The reference party wins 21% of the fights and Meta 25% (measures/rows_trial.py, 150 battles)</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Row P038: it opens with Forbidden Fruit, a debuff; Dark Blast stays in its later turns. The reference party wins 34% and Meta 37%. First Grid, the passive that may act first, comes up 15% of the times in the place of 10% (row P032; it adds nothing that can be measured)</t>
+        </is>
+      </c>
       <c r="L124" t="inlineStr">
         <is>
           <t>closed</t>
@@ -9625,7 +9635,7 @@
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t>Resolved via Samael Turn 1 AI opening adjustment (L05), First Grid scaled to 15% (15 SP), and Warning Shot raised to 10% max.</t>
+          <t>An opening no party can answer is unfair, not hard: the guard that stops the spell cannot be up before the first turn. The fight keeps its spell and its difficulty, without the roll that decided it</t>
         </is>
       </c>
       <c r="O124" t="inlineStr">
@@ -9636,6 +9646,11 @@
       <c r="P124" t="inlineStr">
         <is>
           <t>true</t>
+        </is>
+      </c>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>2026-10-11: the opening of Samael changed because it was unfair; 2026-10-13: measured</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: the Slave's Torc keeps the enchantments of the game
One piece that speeds EXP up is enough: the Bathroom Slippers. The encounter rate of the late dungeons is looked at and left (row S13).
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -10072,7 +10072,7 @@
       </c>
       <c r="N130" t="inlineStr">
         <is>
-          <t>The DLC is ignored (2026-10-06). What it eased is covered by T01: the factors by level gap (option B4, without the kept curve) catch a member up faster than a Double EXP piece did, and a crown costs about 400 battles instead of 4,393 (docs/generated/CATCH_UP_OPTIONS.md); one existing accessory, the Slave's Torc, carries Double EXP from 2026-10-11 (row W042 of balance_changes.xlsx), which takes the place of "no new Double EXP item" of 2026-10-07</t>
+          <t>The DLC is ignored (2026-10-06). What it eased is covered by T01: the factors by level gap (option B4, without the kept curve) catch a member up faster than a Double EXP piece did, and a crown costs about 400 battles instead of 4,393 (docs/generated/CATCH_UP_OPTIONS.md). No piece gains Double EXP: the Slave's Torc carried it from 2026-10-11 to 2026-10-13 (row W042, dropped); the one piece that speeds EXP up is the Bathroom Slippers, with the factor enchantment (row P090)</t>
         </is>
       </c>
       <c r="O130" t="inlineStr">
@@ -11486,6 +11486,11 @@
           <t>The encounter fields of a zone (not read)</t>
         </is>
       </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Chance of a battle a step, by the zones of each dungeon (floor files, zone 0x1C): 5 - 8 in the story up to its thirteenth dungeon, 6 - 10 in the last two and in the postgame. The mean walk between two battles is 20 - 28 steps early and 18 - 25 late (8 + 100 / chance, docs/FORMULAS.md 14)</t>
+        </is>
+      </c>
       <c r="L148" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -11498,7 +11503,7 @@
       </c>
       <c r="N148" t="inlineStr">
         <is>
-          <t>Encounter rate of 5-8% in story dungeons conforms to dungeon crawler genre norms. Repel items and Grand Sealbook Tres Durian provide encounter mitigation.</t>
+          <t>It rises little where it rises: a battle every 18 steps in the worst zones of the end against every 25. Repel items and a grand sealbook lower it for who wants</t>
         </is>
       </c>
       <c r="O148" t="inlineStr">
@@ -11508,7 +11513,12 @@
       </c>
       <c r="P148" t="inlineStr">
         <is>
-          <t>partly true</t>
+          <t>partly true: at most a third more battles in the last dungeons</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>2026-10-13: looked at in the late dungeons, as decided; left as it is</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: the buffs of the Sage line a fifth larger and chanted faster
Circle Brave, Circle Protect and Sun Veil a fifth larger; the chant of those three and of Accelerator at 2.5. Played with her spells and two buffs kept up she wins 92% of five contested bosses in the last place of the reference party, against 90% with an attacker there.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -2320,7 +2320,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>T066 - T075, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Sage wins 12% under the median support at the advanced stage and 2% late, within the band (CLASS_STAGES.md)</t>
+          <t>The Sage in the last place of the reference party, 300 battles at C30, C36, C38, C40 and P24: 92% of wins against 90% with an attacker in her place, and 16 - 23% of the damage of the party (measures/sage_buffs_trial.py, 2026-10-13). Circle Brave and Circle Protect +16% to +31% (x1.6, then a fifth more), Sun Veil a fifth more, and the chant of the four buffs but Amplify at 2.5</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>2026-10-09: accepted</t>
+          <t>2026-10-09: accepted | 2026-10-13: a little larger and chanted faster; the model plays her with her spells</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: the global tables after the three habits of a healer
The curve, the battery, the classes by stage and the win rates are regenerated: the habits act in the game and on the variant alike. Two bosses cross their window with the pass, C19 and C30.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -22715,7 +22715,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-13. measures/WIN_RATES.md (200 battles): the three parties that work in the game end level, Meta 92%, Dual-Support 91%, Mage-Heavy 94% of wins over the 17 bosses of the battery (85%, 89%, 90% in the game); Meta, the one that gains most, was the weakest of the three at C26, C30 and C38 in the game. The weakest party of the game (Anti-Meta-Plus, 0 - 12% at eight bosses) reaches 41 - 100%. CLASS_STAGES.md: 74 of 76 rows within the band. Limit: the band has no top, so a class that is too fast is not flagged (row J11, left). The Witch is the case: 0.61 of the median attacker at the advanced stage, 0.34 at C30 alone, a boss that resists physical damage at 90 - 100 (row S07, decided 2026-10-13: not a problem there)</t>
+          <t>2026-10-13, after the model was taught three habits of a healer. measures/WIN_RATES.md (200 battles): the three parties that work in the game end level, Meta 93%, Dual-Support 92%, Mage-Heavy 96% of wins over the 17 bosses of the battery (86%, 90%, 91% in the game). The weakest party of the game (Anti-Meta-Plus, 50% on the mean) reaches 84%. CLASS_STAGES.md: 74 of 76 rows within the band. Limit: the band has no top (row J11, left). The Witch is the case: far ahead at C30 alone, a boss that resists physical damage at 90 - 100 (row S07, decided 2026-10-13: not a problem there)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -22747,7 +22747,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-13. PARTY_BATTERY.md: 65 of 85 pairs at or above the floor in vanilla, 74 of 85 on the variant; no pair that met its floor in vanilla lost it. CLASS_STAGES.md: the two slow rows (Assassin and Treasure Hunter of the treasure hunter role) were slow before the changes (row J26)</t>
+          <t>2026-10-13. PARTY_BATTERY.md: 68 of 85 pairs at or above the floor in vanilla, 75 of 85 on the variant; no pair that met its floor in vanilla lost it. CLASS_STAGES.md: the two slow rows (Assassin and Treasure Hunter of the treasure hunter role) were slow before the changes (row J26)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -22939,12 +22939,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-10-13. DIFFICULTY_CURVE.md (40 battles a boss): 33 of 44 checkpoints within the windows of vanilla, 11 easier, 0 harder. Six were accepted on 2026-10-11 (C14, C26, C29, C32, C37, C38); C30 is back within with its HP x1.15. The five that crossed since then, with 200 battles (measures/curve_recheck.py): C15, C28 and C39 are within, it was chance; C17 is 28% shorter (49.1 &gt; 35.4, wins 100% both) and C40 is won more (85% &gt; 97%). Both accepted on 2026-10-13</t>
+          <t>2026-10-13, after the model was taught three habits of a healer. DIFFICULTY_CURVE.md (40 battles a boss): 34 of 44 checkpoints within the windows of vanilla, 10 easier, 0 harder. Eight are accepted (C14, C26, C29, C32, C37, C38 on 2026-10-11; C17 and C40 on 2026-10-13). Two are new with the pass, checked with 200 battles (measures/curve_recheck.py): C19 is 27% shorter (8.0 &gt; 5.8, wins 96% &gt; 98%) and C30 is won more (76% &gt; 94%, its HP x1.15 since that day)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>met; 8 bosses easier, accepted</t>
+          <t>met but for 10 bosses easier: 8 accepted, C19 and C30 not decided</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: the global tables after the fourth habit of the model
C30 is within its window with nothing changed: the game is won 98% there once the members stop striking a boss with Dark Aura. One boss crosses with the pass, C15.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -22715,7 +22715,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-13, after the model was taught three habits of a healer. measures/WIN_RATES.md (200 battles): the three parties that work in the game end level, Meta 93%, Dual-Support 92%, Mage-Heavy 96% of wins over the 17 bosses of the battery (86%, 90%, 91% in the game). The weakest party of the game (Anti-Meta-Plus, 50% on the mean) reaches 84%. CLASS_STAGES.md: 74 of 76 rows within the band. Limit: the band has no top (row J11, left). The Witch is the case: far ahead at C30 alone, a boss that resists physical damage at 90 - 100 (row S07, decided 2026-10-13: not a problem there)</t>
+          <t>2026-10-13, after the model was taught four habits of a player (sim/policy.py). measures/WIN_RATES.md (200 battles): the three parties that work in the game end level, Meta 93%, Dual-Support 91%, Mage-Heavy 96% of wins over the 17 bosses of the battery (88%, 90%, 92% in the game); two cells of them gain 15 points or more (Meta at C38, Mage-Heavy at C36). The weakest party of the game (Anti-Meta, 46% on the mean) reaches 78%. CLASS_STAGES.md: 74 of 76 rows within the band. Limit: the band has no top (row J11, left). The Witch is the case: far ahead at C30 alone, a boss that resists physical damage at 90 - 100 (row S07, decided 2026-10-13: not a problem there)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -22747,7 +22747,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-13. PARTY_BATTERY.md: 68 of 85 pairs at or above the floor in vanilla, 75 of 85 on the variant; no pair that met its floor in vanilla lost it. CLASS_STAGES.md: the two slow rows (Assassin and Treasure Hunter of the treasure hunter role) were slow before the changes (row J26)</t>
+          <t>2026-10-13. PARTY_BATTERY.md: 70 of 85 pairs at or above the floor in vanilla, 77 of 85 on the variant; no pair that met its floor in vanilla lost it. CLASS_STAGES.md: the two slow rows (Assassin and Treasure Hunter of the treasure hunter role) were slow before the changes (row J26)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -22939,12 +22939,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-10-13, after the model was taught three habits of a healer. DIFFICULTY_CURVE.md (40 battles a boss): 34 of 44 checkpoints within the windows of vanilla, 10 easier, 0 harder. Eight are accepted (C14, C26, C29, C32, C37, C38 on 2026-10-11; C17 and C40 on 2026-10-13). Two are new with the pass, checked with 200 battles (measures/curve_recheck.py): C19 is 27% shorter (8.0 &gt; 5.8, wins 96% &gt; 98%) and C30 is won more (76% &gt; 94%, its HP x1.15 since that day)</t>
+          <t>2026-10-13, after the model was taught four habits of a player. DIFFICULTY_CURVE.md (40 battles a boss): 34 of 44 checkpoints within the windows of vanilla, 10 easier, 0 harder. Nine are accepted (C14, C26, C29, C32, C37, C38 on 2026-10-11; C17, C19 and C40 on 2026-10-13). C30 is within: the reference party wins 98% of it in the game and on the variant in 39 and 40 turns (200 battles; what the model saw as hard there was its own members striking a boss with Dark Aura). C15 is new with the pass: 32% shorter (16.1 &gt; 11.0, wins 99% both, 200 battles)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>met but for 10 bosses easier: 8 accepted, C19 and C30 not decided</t>
+          <t>met but for 10 bosses easier: 9 accepted, C15 not decided</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: C15 accepted as easier, the HP of C30 stays
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -22939,12 +22939,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-10-13, after the model was taught four habits of a player. DIFFICULTY_CURVE.md (40 battles a boss): 34 of 44 checkpoints within the windows of vanilla, 10 easier, 0 harder. Nine are accepted (C14, C26, C29, C32, C37, C38 on 2026-10-11; C17, C19 and C40 on 2026-10-13). C30 is within: the reference party wins 98% of it in the game and on the variant in 39 and 40 turns (200 battles; what the model saw as hard there was its own members striking a boss with Dark Aura). C15 is new with the pass: 32% shorter (16.1 &gt; 11.0, wins 99% both, 200 battles)</t>
+          <t>2026-10-13, after the model was taught four habits of a player. DIFFICULTY_CURVE.md (40 battles a boss): 34 of 44 checkpoints within the windows of vanilla, 10 easier, 0 harder. Nine are accepted (C14, C26, C29, C32, C37, C38 on 2026-10-11; C17, C19 and C40 on 2026-10-13). C30 is within: the reference party wins 98% of it in the game and on the variant in 39 and 40 turns (200 battles; what the model saw as hard there was its own members striking a boss with Dark Aura). C15 is new with the pass: 32% shorter (16.1 &gt; 11.0, wins 99% both, 200 battles). Accepted the same day: a little faster and within what was expected. The HP of C30 (x1.265 of the game) stays</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>met but for 10 bosses easier: 9 accepted, C15 not decided</t>
+          <t>met; 10 bosses easier, accepted</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: every measure played again with the model as it is; four rows closed with their count
The value of each skill, the ailments, the guide curve, the unique skills, the mercenaries, the party skills, the postgame, the random battles, R04, the boss fit and the audit of the simulator are regenerated after the four habits of the model. Rows J16, J17, S18 and S21 of the register carry a count and a reason that holds.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -1774,6 +1774,11 @@
           <t>P04, P07, P08, P10, P13</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>The enemy with most HP of each boss fight, its five elemental resistances (data of the game, 2026-10-13): at 100 or more in all five in 1 of the 55 fights of the postgame and in none of the 40 of the story; in three or more elements in 4 of the 55; at least one element below 100 in 54 of the 55</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -1781,7 +1786,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Elemental resistance caps damage reduction at 50% (never 0%), and superbosses carry distinct -20% to -30% elemental weaknesses that accelerated chants exploit.</t>
+          <t>A resistance of 100 halves the damage and never voids it (docs/FORMULAS.md 2.4), and every postgame boss but one leaves an element below 100 to strike. The wall the claim describes is one fight, not the postgame</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -1791,7 +1796,12 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>partly true</t>
+          <t>false as stated: one postgame boss in 55 resists every element at 100</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>2026-10-13: closed with the count; no change</t>
         </is>
       </c>
     </row>
@@ -1848,7 +1858,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>From C26 on one enemy action can fell the frailest member from full HP in most battles, with Cover and the guards played. It is what makes the Valkyrie and the Paladin worth their place (rows J04, F07); nothing was changed for it</t>
+          <t>True from C26 on, and meant: one enemy action can fell the frailest member from full HP in most battles of the last third of the story, with Cover and the guards played. It is the reason the Valkyrie and the Paladin have a place (rows J04, F07), and the parties without them still win those fights (measures/WIN_RATES.md: Dual-Support 91% and Mage-Heavy 96% over the 17 bosses of the battery on the variant). Taking the spikes away would take the guard classes with them</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -1863,7 +1873,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>2026-10-13: measured; the claim holds. No change so far: the state waits for a decision</t>
+          <t>2026-10-13: measured; the claim holds and nothing is changed: it is the back and forth of a boss fight (Regression R10)</t>
         </is>
       </c>
     </row>
@@ -11866,6 +11876,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>The bag starts at 30 slots and gains 5 at quest ranks 8, 11, 15 and 20, up to 50 (QuestRankData, reward kind 5; 200, 340, 560 and 1,000 trust points)</t>
+        </is>
+      </c>
       <c r="L153" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -11878,7 +11893,7 @@
       </c>
       <c r="N153" t="inlineStr">
         <is>
-          <t>Starting capacity of 30 is hardcoded in the engine executable; Quest Ranks naturally expand it to 50 slots. Preserves expedition resource management without unstable executable patches.</t>
+          <t>The 30 is a constant of the program and the four enlargements are data of the quest ranks; a player who does quests has 35 slots by the middle of the story. Choosing what to carry back is part of an expedition, and the variant leaves it: a larger bag is a patch of the program for a matter of comfort</t>
         </is>
       </c>
       <c r="O153" t="inlineStr">
@@ -11888,7 +11903,12 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>partly true</t>
+          <t>partly true: 30 slots until quest rank 8, 50 at the end</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>2026-10-13: closed with the figure; no change</t>
         </is>
       </c>
     </row>
@@ -12087,6 +12107,11 @@
           <t>P13</t>
         </is>
       </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Of the 194 fixed battles on floors with random battles, 41 hold an enemy 20 levels or more above the common enemies of their floor, and 31 one 30 or more above (data of the game, 2026-10-13): a boss of level 98 on a floor of the story whose common enemies are of level 27. 34 of the 41 are checkpoints of the model, nearly all of them of the postgame</t>
+        </is>
+      </c>
       <c r="L156" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -12099,7 +12124,7 @@
       </c>
       <c r="N156" t="inlineStr">
         <is>
-          <t>Optional challenge bosses are intended to be tackled later; B4 catch-up curve enables smooth return during postgame.</t>
+          <t>They are the bosses of the postgame, placed on the floors of the story: the game sends the party back to old floors for them, and nothing on the map tells their level. The variant does not move them (R03: the jumps of level of the game are kept); what it changes is how fast a party that comes back catches up (the EXP factors by level gap)</t>
         </is>
       </c>
       <c r="O156" t="inlineStr">
@@ -12109,7 +12134,12 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>partly true</t>
+          <t>true: a fifth of the fixed battles stand 20 levels or more above their floor</t>
+        </is>
+      </c>
+      <c r="R156" t="inlineStr">
+        <is>
+          <t>2026-10-13: closed with the count; the bosses stay where the game has them</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: rows that changed nothing dropped, quest gold serves the early economy
Ten rows whose value was already that of the game are dropped; reasons that quoted a value since changed are brought up to date; the 41 rows of quest gold serve row S19. The player README names the buffs of the Sage line, Ecstasy and the Bathroom Slippers.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -11958,9 +11958,14 @@
           <t>A random battle of the first two dungeons gives 5 to 18 gold and of the next two 27 to 88, against 90 for the cheapest healing item (Croissant), 180 for an Egg Sandwich and 450 for a Danish; a piece sells for a third of its price. The prices of equipment are not decoded (measures/DESIGN_ROWS.md, 2026-10-13)</t>
         </is>
       </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>The gold of the 41 quests that pay gold x1.40 (P rows of the table quests): quests are where the early gold comes from</t>
+        </is>
+      </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>not a problem</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="M154" t="inlineStr">
@@ -11985,7 +11990,7 @@
       </c>
       <c r="R154" t="inlineStr">
         <is>
-          <t>2026-10-13: answered in part by the rows of S20; nothing more</t>
+          <t>2026-10-11: quest gold x1.40 approved; 2026-10-13: it is this row those rows answer</t>
         </is>
       </c>
     </row>
@@ -12032,7 +12037,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>The EXP of a quest is not changed. What the variant changes beside it: the gold of the 41 quests that pay gold x1.40 (P rows of the table quests), and the EXP of a member below the level of the enemies (the factors by level gap, sheet ExePatches)</t>
+          <t>The EXP of a quest is not changed. The gold of quests was raised for row S19; the members who are behind catch up through the EXP factors by level gap (sheet ExePatches)</t>
         </is>
       </c>
       <c r="L155" t="inlineStr">

</xml_diff>

<commit_message>
docs: the tables and the regression sheet after the last pass of the model
Win rates, the value of each skill, the contested bosses, R04 and the anchors are played again with the healer of the back row and Salsa and Hopak as dances; the measures the stopped pass had finished are kept. The sheet Regression and rows S07 and S22 quote the reports as they stand.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -11016,7 +11016,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>CLASS_STAGES.md (2026-10-13): at the advanced stage her fights last 0.61 of those of the median attacker with 46 - 67% of the damage of the party. The peak is one boss: 0.34 at C30, Heartless Avenger, who resists slash, stab and bash at 90, 100 and 90 and the elements at 50 to 100. At C22, C34 and C40 she stands at 0.67 to 0.72; late (P08 - P24) at 0.98</t>
+          <t>CLASS_STAGES.md (2026-10-13): at the advanced stage her fights last 0.57 of those of the median attacker with 47 - 63% of the damage of the party. The peak is one boss: 0.36 at C30, Heartless Avenger, who resists slash, stab and bash at 90, 100 and 90 and the elements at 50 to 100. At C22, C34 and C40 she stands at 0.67, 0.59 and 0.68; late (P08 - P24) at 0.95</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -12191,12 +12191,12 @@
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>The reference party at its level (64), 200 battles: 85% of wins in 33.2 turns in the game, the lowest HP of the party 33% (measures/curve_recheck.py, 2026-10-13). Of the parties of the battery, Mage-Heavy wins 62%, Juggernaut-Plus 19% and the two without a healer none (measures/WIN_RATES.md)</t>
+          <t>The reference party at its level (64), 200 battles: 88% of wins in 32.2 turns in the game, the lowest HP of the party 32% (measures/BOSS_ROWS_CHECK.md, 2026-10-13). Of the parties of the battery in the game: Meta 92%, Dual-Support 98%, Mage-Heavy 76%, Juggernaut-Plus 42% and the two with no healer 0% and 2% (measures/WIN_RATES.md)</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>On the variant the reference party wins 97% in 31.1 turns: easier, accepted on 2026-10-13 (Regression R08)</t>
+          <t>On the variant the reference party wins 96% in 29.7 turns: easier, accepted on 2026-10-13 (Regression R08)</t>
         </is>
       </c>
       <c r="L157" t="inlineStr">
@@ -12221,7 +12221,7 @@
       </c>
       <c r="P157" t="inlineStr">
         <is>
-          <t>partly true: won 85% by a prepared party, never by one with no healer</t>
+          <t>partly true: won 88% by a prepared party, never by one with no healer</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">
@@ -22750,7 +22750,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-13, after the model was taught four habits of a player (sim/policy.py). measures/WIN_RATES.md (200 battles): the three parties that work in the game end level, Meta 93%, Dual-Support 91%, Mage-Heavy 96% of wins over the 17 bosses of the battery (88%, 90%, 92% in the game); two cells of them gain 15 points or more (Meta at C38, Mage-Heavy at C36). The weakest party of the game (Anti-Meta, 46% on the mean) reaches 78%. CLASS_STAGES.md: 74 of 76 rows within the band. Limit: the band has no top (row J11, left). The Witch is the case: far ahead at C30 alone, a boss that resists physical damage at 90 - 100 (row S07, decided 2026-10-13: not a problem there)</t>
+          <t>2026-10-13. measures/WIN_RATES.md (200 battles): the three parties that work in the game end level, Meta 93%, Dual-Support 91%, Mage-Heavy 96% of wins over the 17 bosses of the battery (89%, 90%, 92% in the game); two cells of them gain 15 points or more (Meta at C38, 58% &gt; 91%; Mage-Heavy at C36, 45% &gt; 80%). The weakest party of the game (Anti-Meta, 47% on the mean) reaches 79%. CLASS_STAGES.md: 74 of 76 rows within the band. Limit: the band has no top (row J11, left). The Witch is the case: far ahead at C30 alone, a boss that resists physical damage at 90 - 100 (row S07, decided 2026-10-13: not a problem there)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -22782,7 +22782,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-13. PARTY_BATTERY.md: 70 of 85 pairs at or above the floor in vanilla, 77 of 85 on the variant; no pair that met its floor in vanilla lost it. CLASS_STAGES.md: the two slow rows (Assassin and Treasure Hunter of the treasure hunter role) were slow before the changes (row J26)</t>
+          <t>2026-10-13. PARTY_BATTERY.md: 70 of 85 pairs at or above the floor in vanilla, 79 of 85 on the variant; no pair that met its floor in vanilla lost it. CLASS_STAGES.md: the two slow rows (Assassin and Treasure Hunter of the treasure hunter role) were slow before the changes (row J26)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -22846,12 +22846,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>measures/REGRESSION_R04.md (2026-10-12): at the 17 bosses of the battery, 27 pairs of boss and class on the variant (34 in vanilla) where every winning party of the battery holds the class. With the role of that class changed for a neighbour of the same job (60 battles), a party without it reaches the floor at 20 of the 27 (27 of 34 in vanilla): without a Diva or a Bard at 14 bosses (67 - 100%), without a Valkyrie at C29, C32, C36 and C40 (53 - 92%), without a Bishop at C29. Not reached: the Diva at C40 (the best party without her wins 22%, 13% in vanilla: needed there in vanilla too, and less so on the variant); the Sage and the Witch at C29, where only the mage party wins on either side (Calliope, which the model does not play as the guide describes); and the four base classes at C06, where five characters have joined and no other party can be made</t>
+          <t>2026-10-13. measures/REGRESSION_R04.md: at the 17 bosses of the battery, 24 pairs of boss and class on the variant (31 in vanilla) where every winning party of the battery holds the class. With the role of that class changed for a neighbour of the same job, a party without it reaches the floor at 18 of the 24 (25 of 31 in vanilla). The Diva at the last boss is among them now: the best party without her wins 77% on the variant and 65% in vanilla. Not reached, the same six pairs on both sides: the Sage and the Witch at C29, where only the mage party wins (Calliope, which the model does not play as the guide describes), and the four base classes at C06, where five characters have joined and no other party can be made</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>met: no new mandatory class; the Diva is needed at the last boss, as in vanilla</t>
+          <t>met: no new mandatory class</t>
         </is>
       </c>
     </row>
@@ -22910,7 +22910,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-13. BALANCE_BUILD.md: 1,456 of 1,456 live rows built, and each names the row it serves (column Serves, none empty)</t>
+          <t>2026-10-13. BALANCE_BUILD.md: 1,635 of 1,635 live rows built, 166 of them in the floor files, and each names the row it serves (column Serves, none empty)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -23001,12 +23001,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-13. VERDICTS.md: of 180 rows, 80 closed, 88 not a problem, 12 out of the balance, 0 open. 17 of them are closed on an argument with no figure (listed at the end of VERDICTS.md)</t>
+          <t>2026-10-13. VERDICTS.md: of 181 rows, 83 closed, 86 not a problem, 12 out of the balance, 0 open. 9 of them rest on an argument with no figure (listed at the end of VERDICTS.md)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>met; 17 rows rest on an argument</t>
+          <t>met; 9 rows rest on an argument</t>
         </is>
       </c>
     </row>
@@ -23033,7 +23033,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-10-13. DIFFICULTY_CURVE.md, columns Lowest HP and Pressure: where a checkpoint leaves the window of vanilla the party stands higher (lowest HP 31 - 48% &gt; 49 - 61% at C32, C38, C39, C40), never lower; pressure is above the window at C26 alone (0.07 &gt; 0.10). SIM_ANCHORS.md: 6 of 6 anchors met</t>
+          <t>2026-10-13. DIFFICULTY_CURVE.md, columns Lowest HP and Pressure: where a checkpoint leaves the window of vanilla the party stands higher (lowest HP 15% &gt; 31% at C29, 32% &gt; 53% at C38, 30% &gt; 40% at C40), never lower; pressure is above the window at C26 alone (0.06 &gt; 0.10). SIM_ANCHORS.md: 5 of 6 anchors met, the sixth a known limit (N06)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">

</xml_diff>

<commit_message>
data: a figure for each of the nine rows closed on an argument
Avenger and Barrage measured with and without on the variant at C30 -
C40; Valkyrie, Sniper, Nurse, Cleanse, Attract, the levels of four
skills and the mercenaries from the generated measures and the skill
records. No verdict changes; rows with no figure: 0 of 181.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -1543,6 +1543,11 @@
           <t>Guest ally scripts are data-driven weighted sets not surfaced in UI (BALANCE_BASELINE.md)</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>No text of the game or of the mod states what a mercenary does (0 of 31). What each adds is measured in measures/MERCENARIES.md: the reference party at C36, C40 and P24 with each guest against none (58%, 92%, 100% of wins without).</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -3970,6 +3975,11 @@
           <t>Valkyrie provides top AoE safety with Spell/Material Guard, but Etoile debuffs and Paladin defense also clear late bosses (CLASS_STAGES.md)</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>At every story boss of measures/WIN_RATES.md (17 of 17) a party without a Valkyrie wins on the variant: 92% to 100% at 16 of them, 74% at C36 (Dual-Support). The superbosses of the postgame are outside the measure.</t>
+        </is>
+      </c>
       <c r="L45" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -4966,6 +4976,11 @@
           <t>P03</t>
         </is>
       </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Each level buys a stated gain (skill records of the variant): Panic Voice +40 power a level (240 to 600) for 6 to 8 TP more, the same damage per TP (6.7 at level 1, 6.3 at level 10); Divine Shield 30% to 45% for 24 to 42 TP; Adaptation 6 to 15 and Preparation 15% to 20%, passives that cost nothing.</t>
+        </is>
+      </c>
       <c r="L58" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -5033,6 +5048,11 @@
           <t>P01, P02, P03, P11, P15</t>
         </is>
       </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Nurse and Cleanse cost TP, not gold, and serve in a fight (docs/generated/SKILL_VALUE.md): Nurse at C38 wins +7 points, HP left +9; Cleanse at C40 wins +3 points, HP left +11. Return costs 1 TP at its level 5.</t>
+        </is>
+      </c>
       <c r="L59" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -5567,6 +5587,11 @@
           <t>P03, P09, P10, P14, P15</t>
         </is>
       </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Attract on the Dark Lord at C38 (docs/generated/SKILL_VALUE.md): wins +0 points, fights 5% shorter, HP left +6 points: it serves.</t>
+        </is>
+      </c>
       <c r="L66" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -6257,6 +6282,11 @@
           <t>P03, P10, P13, P14, P15</t>
         </is>
       </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Avenger on the tank at C30, C34, C36, C38 and C40, against the same tank without it (300 battles): wins within 1 point at each, length within 0.2: no harm late, and no gain.</t>
+        </is>
+      </c>
       <c r="L76" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -7992,6 +8022,11 @@
           <t>P03, P06, P14, P15</t>
         </is>
       </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Barrage acts on plain attacks only: the Kunoichi of the model makes 0.7 a fight at C38 (3% of her actions). With it or without it the wins at C30 - C40 do not move (300 battles); at a 100% chance C38 stays at 85%.</t>
+        </is>
+      </c>
       <c r="L101" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -9350,6 +9385,11 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Cleanse on the Shooter at C40 (docs/generated/SKILL_VALUE.md): wins +3 points, HP left +11, for TP instead of an item.</t>
+        </is>
+      </c>
       <c r="L120" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -9713,6 +9753,11 @@
       <c r="J125" t="inlineStr">
         <is>
           <t>In vanilla, guns disabled Spiral Arrow, Divine Cannon, Warning Shot and Support Shot, shutting down Sniper exclusive kit</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>The Sniper is inside the band at every stage of docs/generated/CLASS_STAGES.md (length 0.91 and 1.04 of the median of the attackers, wins 85% - 100%).</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">

</xml_diff>

<commit_message>
data: the regression sheet and two rows with the figures of 2026-10-16
R01 - R10 follow the full suite after the ATK of C36, Barrage 30% -
50% and the Etoile with Waltz and Salsa: every row met. F11 and F63
name the new values of Barrage.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -4305,7 +4305,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>W rows, Double Attack, Triple Attack and Barrage +25%, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>W rows: Double Attack and Triple Attack +25%, built and read back (BALANCE_BUILD.md); Barrage 30% at level 1 to 50% at level 10 since 2026-10-16 (rows W026 - W035)</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -8024,7 +8024,7 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Barrage acts on plain attacks only: the Kunoichi of the model makes 0.7 a fight at C38 (3% of her actions). With it or without it the wins at C30 - C40 do not move (300 battles); at a 100% chance C38 stays at 85%.</t>
+          <t>Barrage acts on plain attacks only: the Kunoichi of the model makes 0.7 a fight at C38 (3% of her actions). At 25% - 40% the wins at C30 - C40 did not move with it or without it (300 battles; at a 100% chance C38 stays at 85%); at 30% - 50% (2026-10-16) the full suite moves by chance only, the Kunoichi inside the band of CLASS_STAGES.md</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -22795,7 +22795,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-13. measures/WIN_RATES.md (200 battles): the three parties that work in the game end level, Meta 93%, Dual-Support 91%, Mage-Heavy 96% of wins over the 17 bosses of the battery (89%, 90%, 92% in the game); two cells of them gain 15 points or more (Meta at C38, 58% &gt; 91%; Mage-Heavy at C36, 45% &gt; 80%). The weakest party of the game (Anti-Meta, 47% on the mean) reaches 79%. CLASS_STAGES.md: 74 of 76 rows within the band. Limit: the band has no top (row J11, left). The Witch is the case: far ahead at C30 alone, a boss that resists physical damage at 90 - 100 (row S07, decided 2026-10-13: not a problem there)</t>
+          <t>2026-10-16. measures/WIN_RATES.md (200 battles): the three parties that work in the game end level, Meta 93%, Dual-Support 91%, Mage-Heavy 95% of wins over the 17 bosses of the battery (89%, 90%, 92% in the game); one cell of Meta (C38) and one of Mage-Heavy (C36) gain more than 15 points, C36 kept with a boss weak to the magic the variant mends</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -22827,7 +22827,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-13. PARTY_BATTERY.md: 70 of 85 pairs at or above the floor in vanilla, 79 of 85 on the variant; no pair that met its floor in vanilla lost it. CLASS_STAGES.md: the two slow rows (Assassin and Treasure Hunter of the treasure hunter role) were slow before the changes (row J26)</t>
+          <t>2026-10-16. PARTY_BATTERY.md: 70 of 85 pairs at or above the floor in vanilla, 78 of 85 on the variant; no pair that met its floor in vanilla lost it (the one below it on the variant that was above it on 2026-10-13, Anti-Meta-Plus at C36, wins 0% in vanilla). CLASS_STAGES.md: 74 of 76 rows inside the band; the two slow rows (Assassin and Treasure Hunter of the treasure hunter role) win 98% - 100%</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -22891,7 +22891,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-13. measures/REGRESSION_R04.md: at the 17 bosses of the battery, 24 pairs of boss and class on the variant (31 in vanilla) where every winning party of the battery holds the class. With the role of that class changed for a neighbour of the same job, a party without it reaches the floor at 18 of the 24 (25 of 31 in vanilla). The Diva at the last boss is among them now: the best party without her wins 77% on the variant and 65% in vanilla. Not reached, the same six pairs on both sides: the Sage and the Witch at C29, where only the mage party wins (Calliope, which the model does not play as the guide describes), and the four base classes at C06, where five characters have joined and no other party can be made</t>
+          <t>2026-10-16. measures/REGRESSION_R04.md: with the role of the class changed for another, a party without the class reaches the floor at 19 of 25 pairs of boss and class on the variant, 25 of 31 in vanilla</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -22955,7 +22955,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-13. BALANCE_BUILD.md: 1,635 of 1,635 live rows built, 166 of them in the floor files, and each names the row it serves (column Serves, none empty)</t>
+          <t>2026-10-16. BALANCE_BUILD.md: 1,636 of 1,636 live rows built, 166 of them in the floor files, and each names the row it serves</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -23019,7 +23019,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-10-13, after the model was taught four habits of a player. DIFFICULTY_CURVE.md (40 battles a boss): 34 of 44 checkpoints within the windows of vanilla, 10 easier, 0 harder. Nine are accepted (C14, C26, C29, C32, C37, C38 on 2026-10-11; C17, C19 and C40 on 2026-10-13). C30 is within: the reference party wins 98% of it in the game and on the variant in 39 and 40 turns (200 battles; what the model saw as hard there was its own members striking a boss with Dark Aura). C15 is new with the pass: 32% shorter (16.1 &gt; 11.0, wins 99% both, 200 battles). Accepted the same day: a little faster and within what was expected. The HP of C30 (x1.265 of the game) stays</t>
+          <t>2026-10-16. DIFFICULTY_CURVE.md (40 battles a boss): 33 of 44 checkpoints within the windows of vanilla, 10 easier (the ten accepted: C14, C15, C17, C19, C26, C29, C32, C37, C38, C40), 1 harder: C36 on its pressure (0.20 &gt; 0.25), on the edge of the window; measures/curve_recheck.py C36 400: within every window (pressure 0.21 &gt; 0.25; 1,000 battles: +15%, window 25%)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -23046,12 +23046,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-13. VERDICTS.md: of 181 rows, 83 closed, 86 not a problem, 12 out of the balance, 0 open. 9 of them rest on an argument with no figure (listed at the end of VERDICTS.md)</t>
+          <t>2026-10-16. VERDICTS.md: of 181 rows, 83 closed, 86 not a problem, 12 out of the balance, 0 open; every row holds a figure (0 rest on an argument alone)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>met; 9 rows rest on an argument</t>
+          <t>met</t>
         </is>
       </c>
     </row>
@@ -23078,7 +23078,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-10-13. DIFFICULTY_CURVE.md, columns Lowest HP and Pressure: where a checkpoint leaves the window of vanilla the party stands higher (lowest HP 15% &gt; 31% at C29, 32% &gt; 53% at C38, 30% &gt; 40% at C40), never lower; pressure is above the window at C26 alone (0.06 &gt; 0.10). SIM_ANCHORS.md: 5 of 6 anchors met, the sixth a known limit (N06)</t>
+          <t>2026-10-16. DIFFICULTY_CURVE.md, columns Lowest HP and Pressure: where a checkpoint leaves the window of vanilla on the easier side the party stands higher (lowest HP 15% &gt; 31% at C29, 32% &gt; 53% at C38, 30% &gt; 40% at C40), never lower; C36 asks more of the party (pressure 0.20 &gt; 0.25) and C26 too (0.06 &gt; 0.10)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">

</xml_diff>

<commit_message>
data: the changes checked in the game marked as seen working
Levers L12, L15, L25, L27, L38, L46 and L47: the blacksmith, the length
of meals with poison as before, Bathroom Slippers, the circles and
Accelerator, Ecstasy and both patched program files, play-tested on
2026-10-16. CONTRIBUTING.md says the variant is play-tested.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -23587,7 +23587,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Read as numbers by the command of the effect; the QoL build already rewrites these files byte for byte</t>
+          <t>Read as numbers by the command of the effect; the QoL build already rewrites these files byte for byte. Seen working in the game (play-tested, 2026-10-16: Circle Brave, Circle Protect, Sun Veil and Accelerator at their new values and chant speed; Ecstasy 20% - 30%)</t>
         </is>
       </c>
     </row>
@@ -23698,7 +23698,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>The rank is an index into WeaponRankData; the count is checked by extract_vanilla</t>
+          <t>The rank is an index into WeaponRankData; the count is checked by extract_vanilla. Seen working in the game (play-tested, 2026-10-16: Bathroom Slippers with Double EXP (enchantment 275))</t>
         </is>
       </c>
     </row>
@@ -24063,7 +24063,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 6c. The floats themselves are shared and must not be edited in place</t>
+          <t>docs/FORMULAS.md 6c. The floats themselves are shared and must not be edited in place. Seen working in the game (play-tested, 2026-10-16: the patched program files run, the one with its protector too)</t>
         </is>
       </c>
     </row>
@@ -24137,7 +24137,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 10. No data field holds these; the only data levers on the crown grind are the EXP table and the EXP of enemies</t>
+          <t>docs/FORMULAS.md 10. No data field holds these; the only data levers on the crown grind are the EXP table and the EXP of enemies. Seen working in the game (play-tested, 2026-10-16: the patched program files run, the one with its protector too)</t>
         </is>
       </c>
     </row>
@@ -24544,7 +24544,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 12.19: the only unique skill whose chance is not its value</t>
+          <t>docs/FORMULAS.md 12.19: the only unique skill whose chance is not its value. Seen working in the game (play-tested, 2026-10-16: the patched program files run, the one with its protector too)</t>
         </is>
       </c>
     </row>
@@ -24585,6 +24585,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
@@ -24900,7 +24901,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 14: each is rolled against a number below 100 on a step (0x4bc8a1 - 0x4bcb77), as the chance of a battle (L29)</t>
+          <t>docs/FORMULAS.md 14: each is rolled against a number below 100 on a step (0x4bc8a1 - 0x4bcb77), as the chance of a battle (L29). Seen working in the game (play-tested, 2026-10-16: the wandering blacksmith comes more often)</t>
         </is>
       </c>
     </row>
@@ -24937,7 +24938,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 12.18: the tick of the 97 effects of the class CCommandTurnBase (0x48d590). The ailments that end on a roll (0x48d180, its own count at 0x48d202) and petrification (0x483010) have theirs and are left</t>
+          <t>docs/FORMULAS.md 12.18: the tick of the 97 effects of the class CCommandTurnBase (0x48d590). The ailments that end on a roll (0x48d180, its own count at 0x48d202) and petrification (0x483010) have theirs and are left. Seen working in the game (play-tested, 2026-10-16: a meal lasts a couple of battles while poison still wears off as before)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: the small findings of the audit of 2026-10-16
- measure_config.json: Eccentrics measured as AGI +20 (row P091), not
  the DEX +32 of the idea before it; PARTY_SKILLS.md: fights 13% shorter.
- The snapshot names the unique skills of the variant by their
  Balance_Name: UNIQUE_SKILLS.md says No Miracles Needed.
- README_Balance.txt: the extra skill point comes at levels 31 to 70.
- Criticisms J06, J24, F17, I11 cite the rows as they stand: W038 and
  W039 dropped, H036 / H037 a cure on the heals, S003 - S012 in place of
  T031 - T040, the lowered values of No Miracles Needed.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -1001,7 +1001,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>W rows, four bow skills open to guns, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); shooter within the band at the four stages (0.85, 0.89, 0.88, 1.09; CLASS_STAGES.md)</t>
+          <t>W036, W037: Spiral Arrow and Divine Cannon open to guns, built and read back (BALANCE_BUILD.md); W038, W039 (Warning Shot, Support Shot) dropped on 2026-10-11, a passive record holds one weapon code; shooter within the band at the four stages (0.85, 0.89, 0.88, 1.09; CLASS_STAGES.md)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -2417,7 +2417,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Addressed by Full Heal (H036) and Circle Full Heal (H037) additions to restore Bishop healing identity.</t>
+          <t>Solved by class identity: the Bishop learns Full Heal (100% of max HP, no cap). H036 and H037 do not touch the cap: they let Heal and Circle Heal cure poison too (and paralysis at the upper levels of Heal)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -2432,12 +2432,12 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>Solved by class identity (Full Heal) and H036/H037 (HP% scaling on Heal and Circle Heal)</t>
+          <t>Solved by class identity (Full Heal); H036 / H037 add a cure to Heal and Circle Heal</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>2026-10-10: solved by Full Heal and H rows (H036, H037)</t>
+          <t>2026-10-10: solved by Full Heal; H036, H037 (the cure on the heals) decided 2026-10-09</t>
         </is>
       </c>
     </row>
@@ -4762,7 +4762,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>T031 - T040 and Y rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Trickster 1.08 - 1.13, Joker 1.00 advanced and 0.96 late, within the band (CLASS_STAGES.md)</t>
+          <t>S003 - S012 (Checkmate, direct values 0.40 to 1.20; they replaced T031 - T040, x1.6, dropped to avoid stacking two buffs) and Y rows, built and read back (BALANCE_BUILD.md); Trickster 1.08 - 1.13, Joker 1.00 advanced and 0.96 late, within the band (CLASS_STAGES.md)</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -4782,7 +4782,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>T031 - T040: Checkmate x1.6 power</t>
+          <t>T031 - T040: Checkmate x1.6 power; replaced by S003 - S012 (direct values)</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -13435,7 +13435,7 @@
       </c>
       <c r="Q174" t="inlineStr">
         <is>
-          <t>U011 - U020, U051: the skill becomes the chance to hold on with 1 HP when a hit would fell her (effect 254, 15 - 40% by rank, 55% with the crown), named again in the variant</t>
+          <t>U011 - U020, U051: the skill becomes the chance to hold on with 1 HP when a hit would fell her (effect 254, 10 - 26% by rank, 35% with the crown, lowered from the 15 - 40% / 55% first proposed), named No Miracles Needed in the variant</t>
         </is>
       </c>
       <c r="R174" t="inlineStr">
@@ -24585,7 +24585,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
data: S09 records why stacking All stats cannot be abused
Read from the drop code: random All stats roll only on the Ring, one per piece, from item level 10/30/50/75; the other sources are 15 fixed pieces. Upper bound measured with the engine.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -11223,6 +11223,11 @@
           <t>P19</t>
         </is>
       </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Upper bound, +30 on all five members of the reference party (impossible in play), 400 runs, median length: C34 33.9 -&gt; 16.3, C38 12.3 -&gt; 6.6 (wins 91% -&gt; 100%), C40 29.2 -&gt; 15.5; vanilla with the same pieces counts one: C38 18.4 -&gt; 11.7. dtcli run, seed 7000.</t>
+        </is>
+      </c>
       <c r="L144" t="inlineStr">
         <is>
           <t>closed</t>
@@ -11235,7 +11240,7 @@
       </c>
       <c r="N144" t="inlineStr">
         <is>
-          <t>All stats enchantments (IDs 24-28) bit 0 enabled at offset 0x20 in EnchantData.pck (word 8 changed from 428 to 429), allowing gear piece stacking.</t>
+          <t>All stats enchantments (IDs 24-28) bit 0 enabled at offset 0x20 in EnchantData.pck (word 8 changed from 428 to 429), allowing gear piece stacking. The stacking cannot be farmed into a party-wide stack: a random drop rolls All stats only on the Ring (piece 710; bit 8 of EnchantData 0x20, 0x556bf0), at most one per piece (group 3 at 0x28), from item level 10 / 30 / 50 / 75 for +3 / +6 / +9 / +12 (0x2C, 0x556cd3; +12 is postgame); the other sources are 15 fixed pieces with +1 to +9, one per slot. About +30 on one or two members at most.</t>
         </is>
       </c>
       <c r="O144" t="inlineStr">

</xml_diff>

<commit_message>
docs: the skill niches in the player README, the register and the limits
README_Balance lists the Queen of Darkness and the skill changes of 2026-10-16; CONTRIBUTING the situational skills, the bag of the model and the mass tests; Criticisms F60, F71, J21, J23 carry the figures. skill-battery again on the current variant: 124 good, 93 niche, 14 dead, 16 hurts, 4 no effect. Raw figures of the mass tests stay out of git.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -2179,6 +2179,11 @@
           <t>Dark Lord is the top physical attacker in advanced and late game: 54 - 74% damage share, 100% wins at C40 and P24; Attract serves (+1% wins, SKILL_VALUE.md); Megaton Press 72% worth, Geo Break and Life Bring 100% (CLASS_STAGES.md, SKILL_WORTH.md)</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>2026-10-16: the Dark Lord of the model lost her charge to Berserk (sheet Policies fixed); Power Charge 1.13 - 1.40, the charged blow x2.13 - x2.4 (V001 - V005): skill-battery good; class-search C34, C38 over the 7,632 final-class parties with a Dark Lord: wins 69.9% &gt; 70.6%, no dominant party.</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -2335,7 +2340,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>The Sage in the last place of the reference party, 300 battles at C30, C36, C38, C40 and P24: 92% of wins against 90% with an attacker in her place, and 16 - 23% of the damage of the party (measures/sage_buffs_trial.py, 2026-10-13). Circle Brave and Circle Protect +16% to +31% (x1.6, then a fifth more), Sun Veil a fifth more, and the chant of the four buffs but Amplify at 2.5</t>
+          <t>The Sage in the last place of the reference party, 300 battles at C30, C36, C38, C40 and P24: 92% of wins against 90% with an attacker in her place, and 16 - 23% of the damage of the party (measures/sage_buffs_trial.py, 2026-10-13). Circle Brave and Circle Protect +16% to +31% (x1.6, then a fifth more), Sun Veil a fifth more, and the chant of the four buffs but Amplify at 2.5 2026-10-16: Accelerator 10 - 15% for 4 turns (V006 - V015), given by the model to the ally who hits hardest, and Prism Dawn x1.4 power (V021 - V030): both a niche in dtcli skill-battery (they were weak or dead).</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -7808,7 +7813,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>K rows (TP -25%) and X rows (chant 0.75 at every level), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row</t>
+          <t>K rows (TP -25%) and X rows (chant 0.75 at every level), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row 2026-10-16: dtcli skill-battery found Shadow Clone still costing the Kunoichi more than it saved (51% of the cells worse); one more turn at every level (V016 - V020) makes it a niche.</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -8600,7 +8605,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>D rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); dolls within the band at the four stages (1.12, 0.97, 1.04, 1.13; CLASS_STAGES.md)</t>
+          <t>D rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); dolls within the band at the four stages (1.12, 0.97, 1.04, 1.13; CLASS_STAGES.md) 2026-10-16: Oracles took the place of a better doll (skill-battery: hurts); its action x1.5 (D061 - D070, ATK 328 - 421%) makes it a niche; class-search C34, C38 over the 7,402 final-class parties with a Soul Summoner: wins 70.2% &gt; 70.5%, no dominant party.</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">

</xml_diff>

<commit_message>
balance: Soul Eater and the Magical Princess a little stronger
Soul Eater 20% cheaper, 15% stronger, and learned by the Soul Summoner of the model (sheet Roles); Magical Change two turns longer and 25% stronger, Magical Spark 20% cheaper (rows V031 - V061, C098 - C106). class-search C30 - C40 boss, compare=variant: wins 53.2% > 54.0% with a Soul Summoner, 47.5% > 50.6% with a Magical Princess, no dominant party. Battery 80 of 85.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -1935,7 +1935,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>D rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); soul summoner within the band at the four stages (1.12, 0.98, 0.87, 1.02; CLASS_STAGES.md)</t>
+          <t>D rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); soul summoner within the band at the four stages (1.12, 0.98, 0.87, 1.02; CLASS_STAGES.md) 2026-10-16: the Soul Summoner herself dealt 1 - 2% of the damage of her party; Soul Eater 20% cheaper and 15% stronger (V031 - V050), learned by the model: class-search over the 14,804 final-class parties with her, wins 53.2% &gt; 54.0%.</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Q001 - Q015, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Magical Princess 1.06 advanced, 1.01 late, within the band (CLASS_STAGES.md)</t>
+          <t>Q001 - Q015, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Magical Princess 1.06 advanced, 1.01 late, within the band (CLASS_STAGES.md) 2026-10-16: Magical Change two turns longer and 25% stronger, Magical Spark 20% cheaper (V051 - V061, C098 - C106): class-search over the 15,289 final-class parties with her, wins 47.5% &gt; 50.6%, fights 9% shorter, no dominant party.</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">

</xml_diff>

<commit_message>
sim[roles]: the Witch raises Crimson Flare and Inferno; S07 open
The model's Witch kept her strong spells at level 1 (121 skill points at level 44, 110 of them in Fireball and Magic Mastery); now Crimson Flare comes right after Fireball and Inferno after Concentrate. She casts Crimson Flare 11 - 15 times at C38 and C40; her margin hardly moves (in 88% of the fastest final-class parties, vanilla 88%). S07 opened again to decide on her; Economy at half took 1.9 points off the parties with a Witch and did not slow them.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -11071,7 +11071,7 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>not a problem</t>
+          <t>open</t>
         </is>
       </c>
       <c r="M142" t="inlineStr">
@@ -11081,7 +11081,7 @@
       </c>
       <c r="N142" t="inlineStr">
         <is>
-          <t>She is far ahead where the boss shuts physical damage out, which is what a mage is for; elsewhere she is the fastest attacker by a third, and level with the others in the postgame</t>
+          <t>She is far ahead where the boss shuts physical damage out, which is what a mage is for; elsewhere she is the fastest attacker by a third, and level with the others in the postgame 2026-10-16, opened again: class-search over every final-class party puts the Witch in 87% of the fastest 5% of the parties (vanilla 87%); the model leveled Fireball and left her strong spells at level 1, so her margin is measured again with the spells a player raises.</t>
         </is>
       </c>
       <c r="O142" t="inlineStr">

</xml_diff>

<commit_message>
balance: the Witch into the band of the other classes (S07)
Her INT x0.9 at every level (growth row 18 of ClassLevelData) and the five basic spells of the Magic User at levels 6 - 10 x0.85 power (rows V062 - V185). In vanilla she was in 97% of the fastest final-class parties (the next class 65%); now 75% (the next 74%), her parties win 49.9% (median of the others 52.4%). The builder and the variant reader take a class_growth table (lever L10) and deliver ClassLevelData; skill-battery trials take e<id>@lo-hi, cast and class:<name>:<stat>*f.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -11069,9 +11069,14 @@
           <t>CLASS_STAGES.md (2026-10-13): at the advanced stage her fights last 0.57 of those of the median attacker with 47 - 63% of the damage of the party. The peak is one boss: 0.36 at C30, Heartless Avenger, who resists slash, stab and bash at 90, 100 and 90 and the elements at 50 to 100. At C22, C34 and C40 she stands at 0.67, 0.59 and 0.68; late (P08 - P24) at 0.95</t>
         </is>
       </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>2026-10-16: the Witch INT x0.9 (growth row 18) and the five basic spells at levels 6 - 10 x0.85 (V062 - V185). dtcli class-search final C30, C34, C38, C40 boss, 3,000 parties a boss: in vanilla she is in 97% of the fastest 5% of the parties (the next class 65%); now 75% (the next 74%), her parties win 49.9% (median of the other classes 52.4%).</t>
+        </is>
+      </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="M142" t="inlineStr">

</xml_diff>

<commit_message>
data: figures of 2026-10-16 for F01, J05, F26, J11 and S07
Without the Maid line the best final-class party wins C30, C34 and C38 100% and C40 20% with the 8 fruit of the sheets, all four 100% with 24 (class-search no_maid_line); the Maid line stays the TP source. J11: the mage role against the median attacker by stage (class-stages), no cliff. S07: the band of the classes of the suite (class-balance).
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -919,7 +919,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>R rows, Auto-Refresh 3 - 9 to 4 - 11 TP per turn, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); every role spends 15% of its TP on an ally under 15%</t>
+          <t>R rows, Auto-Refresh 3 - 9 to 4 - 11 TP per turn, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); every role spends 15% of its TP on an ally under 15% 2026-10-16, dtcli class-search preset=no_maid_line (every final-class party without a Diva, Mistress or Etoile, 1,000 a boss; measures/CLASS_SEARCH_FINAL_REG_NOMAID.md, _REG_NOMAID24.md): with the 8 fruit of the sheets the best such party wins C30, C34 and C38 100% and C40 20%; with 24 fruit in the bag all four 100% (C40: Bishop, Papillon, two Soul Summoners, Valkyrie, 18.2 turns). The Maid line stays the TP source by design: a party without her gets through the story with a bag of fruit.</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1394,6 +1394,11 @@
           <t>Mage over Dark Lord, damage per time: 41% (C07), 101% (C13), 195% (C18), 306% (C25), 286% (C34), 213% (C38), 202 - 204% (P24, P49): a peak in the middle and a lower level after it, but no cliff (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2026-10-16, docs/generated/CLASS_STAGES.md: the mage role against the median attacker, length of the won fights / share of the party damage: base (Magic User) 0.77 / 38 - 50%, intermediate (Sorceress) 0.91 / 27 - 51%, advanced (Witch) 0.70 / 44 - 55%, late (Witch) 0.96 / 3 - 54%: the middle peak is softer than in vanilla (0.57 advanced) and there is no cliff; no change to the curve of magic itself.</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -3505,7 +3510,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Y012 - Y014 (Magical Fruit 25 to 30 TP, Fairy Apple 50 to 60, Golden Apple 100 to 120), built and read back (1,401 of 1,401 rows). The Meta party with a Bishop in the place of its Diva, nobody of the Maid line in it (measures/tp_items_trial.py, 60 battles): with the 8 fruit of the sheets 3% / 3% / 18% / 68% at C30 / C34 / C36 / C38; with 24 fruit in the bag 67% / 82% / 45% / 98% (47% / 52% / 38% / 97% before the raise). What stops such a party at C30 and C34 is TP (100% with TP at will); C36 does not turn on it, and the last boss is not won without the Maid line (0%; 45% with 99 fruit). Up to C28 the party wins 78 - 100% without her. Nothing else moved: curve 37 of 44, battery 75 of 85, classes 74 of 76, anchors 6 of 6</t>
+          <t>Y012 - Y014 (Magical Fruit 25 to 30 TP, Fairy Apple 50 to 60, Golden Apple 100 to 120), built and read back (1,401 of 1,401 rows). The Meta party with a Bishop in the place of its Diva, nobody of the Maid line in it (measures/tp_items_trial.py, 60 battles): with the 8 fruit of the sheets 3% / 3% / 18% / 68% at C30 / C34 / C36 / C38; with 24 fruit in the bag 67% / 82% / 45% / 98% (47% / 52% / 38% / 97% before the raise). What stops such a party at C30 and C34 is TP (100% with TP at will); C36 does not turn on it, and the last boss is not won without the Maid line (0%; 45% with 99 fruit). Up to C28 the party wins 78 - 100% without her. Nothing else moved: curve 37 of 44, battery 75 of 85, classes 74 of 76, anchors 6 of 6 2026-10-16, dtcli class-search preset=no_maid_line (every final-class party without a Diva, Mistress or Etoile, 1,000 a boss; measures/CLASS_SEARCH_FINAL_REG_NOMAID.md, _REG_NOMAID24.md): with the 8 fruit of the sheets the best such party wins C30, C34 and C38 100% and C40 20%; with 24 fruit in the bag all four 100% (C40: Bishop, Papillon, two Soul Summoners, Valkyrie, 18.2 turns). The Maid line stays the TP source by design: a party without her gets through the story with a bag of fruit.</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -5455,7 +5460,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>as J05</t>
+          <t>as J05. 2026-10-16, dtcli class-search preset=no_maid_line (every final-class party without a Diva, Mistress or Etoile, 1,000 a boss; measures/CLASS_SEARCH_FINAL_REG_NOMAID.md, _REG_NOMAID24.md): with the 8 fruit of the sheets the best such party wins C30, C34 and C38 100% and C40 20%; with 24 fruit in the bag all four 100% (C40: Bishop, Papillon, two Soul Summoners, Valkyrie, 18.2 turns). The Maid line stays the TP source by design: a party without her gets through the story with a bag of fruit.</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -11071,7 +11076,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>2026-10-16: the Witch INT x0.9 (growth row 18) and the five basic spells at levels 6 - 10 x0.85 (V062 - V185). dtcli class-search final C30, C34, C38, C40 boss, 3,000 parties a boss: in vanilla she is in 97% of the fastest 5% of the parties (the next class 65%); now 75% (the next 74%), her parties win 49.9% (median of the other classes 52.4%).</t>
+          <t>2026-10-16: the Witch INT x0.8 (growth row 18) and the five basic spells at levels 6 - 10 x0.85 (V062 - V185). dtcli suite, class-balance (docs/generated/CLASS_BALANCE.md, every boss of the final classes): her parties win 73.4% (-0.7 sd against the classes; mean 76.6%). Speed: one Witch puts a party among the fastest 5% x1.85 as often as the mean (+2.5 sd, the next class x1.59), two or more x6.6; in vanilla she was in 97% of the fastest parties. Lower INT only takes wins from her, not speed: the speed of a stack of mages is what is left, and it is kept. CLASS_STAGES.md: her fights last 0.70 of those of the median attacker (vanilla 0.57).</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">

</xml_diff>

<commit_message>
data: unique-battery figures for I01 - I18
Each row of the unique skills gets the verdict of dtcli unique-battery: the share of cells it serves and hurts, and its best cell. 14 good, 4 niche (Positive Trance, Sugar Coma, No Miracles Needed, Undaunted Spirit), none dead.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -12765,7 +12765,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Irena as mage, without the skill &gt; with it): C36 87% &gt; 88%, C38 98% &gt; 95%, C40 78% &gt; 75%, P24 88% &gt; 86%, P27 crowned 51% &gt; 52%. In the mean -1 points of wins, fights +4% shorter, -1 points of HP left (a cell moves by about 5 points by chance). Read again on 2026-10-12: one roll below 100 under value * 100 for each chanted command (0x4176a0, called at 0x41d69c for a spell and at 0x419c55 for the other chanted kind, each behind a flag that keeps it to one roll): 7 - 15% by rank, 20% crowned. Both guides felt 40 - 50% with the crown</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Irena as mage, without the skill &gt; with it): C36 87% &gt; 88%, C38 98% &gt; 95%, C40 78% &gt; 75%, P24 88% &gt; 86%, P27 crowned 51% &gt; 52%. In the mean -1 points of wins, fights +4% shorter, -1 points of HP left (a cell moves by about 5 points by chance). Read again on 2026-10-12: one roll below 100 under value * 100 for each chanted command (0x4176a0, called at 0x41d69c for a spell and at 0x419c55 for the other chanted kind, each behind a flag that keeps it to one roll): 7 - 15% by rank, 20% crowned. Both guides felt 40 - 50% with the crown 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Forerunner in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 42% of 1100 cells and makes 11% worse; best cell C34 boss, Anti-Meta-Plus (mage): wins +5%, fights +20% shorter, HP left +5%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L164" t="inlineStr">
@@ -12832,7 +12832,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yae as dark lord, without the skill &gt; with it): C36 95% &gt; 93%, C38 91% &gt; 95%, C40 94% &gt; 96%, P24 100% &gt; 99%, P27 crowned 91% &gt; 92%. In the mean +1 points of wins, fights +7% shorter, -0 points of HP left (a cell moves by about 5 points by chance). Played since 2026-10-12 as read: the second action belongs to the same turn, so her statuses do not lose a turn between the two (Power Charge serves both blows)</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yae as dark lord, without the skill &gt; with it): C36 95% &gt; 93%, C38 91% &gt; 95%, C40 94% &gt; 96%, P24 100% &gt; 99%, P27 crowned 91% &gt; 92%. In the mean +1 points of wins, fights +7% shorter, -0 points of HP left (a cell moves by about 5 points by chance). Played since 2026-10-12 as read: the second action belongs to the same turn, so her statuses do not lose a turn between the two (Power Charge serves both blows) 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Did You Call for Me? in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 54% of 825 cells and makes 11% worse; best cell C30 boss, Mage-Heavy (dark lord): wins +20%, fights +6% shorter, HP left +16%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L165" t="inlineStr">
@@ -12899,7 +12899,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Ist as etoile, without the skill &gt; with it): C36 76% &gt; 83%, C38 96% &gt; 98%, C40 96% &gt; 97%, P24 98% &gt; 99%, P27 crowned 71% &gt; 72%. In the mean +2 points of wins, fights +0% shorter, +2 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Ist as etoile, without the skill &gt; with it): C36 76% &gt; 83%, C38 96% &gt; 98%, C40 96% &gt; 97%, P24 98% &gt; 99%, P27 crowned 71% &gt; 72%. In the mean +2 points of wins, fights +0% shorter, +2 points of HP left (a cell moves by about 5 points by chance). 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Maximum Maid in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 39% of 540 cells and makes 5% worse; best cell C40 boss, Dual-Support (etoile): wins +32%, fights +22% shorter, HP left +28%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L166" t="inlineStr">
@@ -12966,7 +12966,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Melvy as magical princess, without the skill &gt; with it): C36 79% &gt; 82%, C38 99% &gt; 100%, C40 76% &gt; 73%, P24 85% &gt; 79%, P27 crowned 64% &gt; 63%. In the mean -1 points of wins, fights +2% shorter, -2 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Melvy as magical princess, without the skill &gt; with it): C36 79% &gt; 82%, C38 99% &gt; 100%, C40 76% &gt; 73%, P24 85% &gt; 79%, P27 crowned 64% &gt; 63%. In the mean -1 points of wins, fights +2% shorter, -2 points of HP left (a cell moves by about 5 points by chance). 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Yearning in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 39% of 320 cells and makes 12% worse; best cell C40 random, Juggernaut-Plus (mage): wins +2%, fights +8% shorter, HP left +1%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L167" t="inlineStr">
@@ -13033,7 +13033,7 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Mefmera as papillon, without the skill &gt; with it): C36 81% &gt; 84%, C38 97% &gt; 100%, C40 86% &gt; 95%, P24 94% &gt; 98%, P27 crowned 89% &gt; 98%. In the mean +6 points of wins, fights +4% shorter, +5 points of HP left (a cell moves by about 5 points by chance). It cuts the damage of demons, undead and apparitions: Samael (C38) and Melek Taus (P27) are demons; the race of the others was not checked against its list</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Mefmera as papillon, without the skill &gt; with it): C36 81% &gt; 84%, C38 97% &gt; 100%, C40 86% &gt; 95%, P24 94% &gt; 98%, P27 crowned 89% &gt; 98%. In the mean +6 points of wins, fights +4% shorter, +5 points of HP left (a cell moves by about 5 points by chance). It cuts the damage of demons, undead and apparitions: Samael (C38) and Melek Taus (P27) are demons; the race of the others was not checked against its list 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Demon Wall in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 51% of 960 cells and makes 3% worse; best cell C40 boss, Anti-Meta-Plus (dolls): wins +22%, fights +5% shorter, HP left +26%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L168" t="inlineStr">
@@ -13100,7 +13100,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Eltricia as magical princess, without the skill &gt; with it): C36 79% &gt; 89%, C38 99% &gt; 97%, C40 76% &gt; 75%, P24 85% &gt; 78%, P27 crowned 64% &gt; 68%. In the mean +1 points of wins, fights +1% shorter, -0 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Eltricia as magical princess, without the skill &gt; with it): C36 79% &gt; 89%, C38 99% &gt; 97%, C40 76% &gt; 75%, P24 85% &gt; 78%, P27 crowned 64% &gt; 68%. In the mean +1 points of wins, fights +1% shorter, -0 points of HP left (a cell moves by about 5 points by chance). 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Wreathed in Glory in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 35% of 720 cells and makes 15% worse; best cell C40 boss, Anti-Meta-Plus (magical princess): wins +12%, fights +0% shorter, HP left +9%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L169" t="inlineStr">
@@ -13167,7 +13167,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Alisia as attacker, without the skill &gt; with it): C36 93% &gt; 91%, C38 80% &gt; 82%, C40 45% &gt; 49%, P24 99% &gt; 98%, P27 crowned 69% &gt; 68%. In the mean +0 points of wins, fights +2% shorter, -0 points of HP left (a cell moves by about 5 points by chance). The simulator holds Pep at 100; she was played at Pep 130, the most it can be, so this is the most the skill gives: +6% damage at rank 5 - 6, +15% at rank 9, +30% crowned (the guide measured about +15% at level 90)</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Alisia as attacker, without the skill &gt; with it): C36 93% &gt; 91%, C38 80% &gt; 82%, C40 45% &gt; 49%, P24 99% &gt; 98%, P27 crowned 69% &gt; 68%. In the mean +0 points of wins, fights +2% shorter, -0 points of HP left (a cell moves by about 5 points by chance). The simulator holds Pep at 100; she was played at Pep 130, the most it can be, so this is the most the skill gives: +6% damage at rank 5 - 6, +15% at rank 9, +30% crowned (the guide measured about +15% at level 90) 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Positive Trance in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): niche, it serves in 19% of 405 cells and makes 4% worse; best cell C33 boss, Anti-Meta-Plus (attacker): wins +1%, fights +7% shorter, HP left +1%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L170" t="inlineStr">
@@ -13234,7 +13234,7 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Luco as dark lord, without the skill &gt; with it): C36 82% &gt; 88%, C38 98% &gt; 100%, C40 88% &gt; 86%, P24 95% &gt; 90%, P27 crowned 83% &gt; 77%. In the mean -1 points of wins, fights +8% shorter, -1 points of HP left (a cell moves by about 5 points by chance). Played since 2026-10-12 as read (measures/qol_fields_reading.md 5, checked): the shadow has the stats of its owner at that moment with twice the ATK, her passives, none of the statuses techniques put, a life of 3. The fault the Japanese page tells (its attack falling back after a drain) is not in the program by that reading</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Luco as dark lord, without the skill &gt; with it): C36 82% &gt; 88%, C38 98% &gt; 100%, C40 88% &gt; 86%, P24 95% &gt; 90%, P27 crowned 83% &gt; 77%. In the mean -1 points of wins, fights +8% shorter, -1 points of HP left (a cell moves by about 5 points by chance). Played since 2026-10-12 as read (measures/qol_fields_reading.md 5, checked): the shadow has the stats of its owner at that moment with twice the ATK, her passives, none of the statuses techniques put, a life of 3. The fault the Japanese page tells (its attack falling back after a drain) is not in the program by that reading 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Shadow Heart in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 51% of 1125 cells and makes 6% worse; best cell C34 boss, Anti-Meta-Plus (tank): wins +1%, fights +55% shorter, HP left +0%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L171" t="inlineStr">
@@ -13301,7 +13301,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Grishna as attacker, without the skill &gt; with it): C36 90% &gt; 88%, C38 98% &gt; 97%, C40 71% &gt; 72%, P24 87% &gt; 89%, P27 crowned 67% &gt; 75%. In the mean +2 points of wins, fights +4% shorter, +0 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Grishna as attacker, without the skill &gt; with it): C36 90% &gt; 88%, C38 98% &gt; 97%, C40 71% &gt; 72%, P24 87% &gt; 89%, P27 crowned 67% &gt; 75%. In the mean +2 points of wins, fights +4% shorter, +0 points of HP left (a cell moves by about 5 points by chance). 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Furious Strike in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 40% of 615 cells and makes 10% worse; best cell C29 boss, Juggernaut-Plus (dark lord): wins +16%, fights +5% shorter, HP left +17%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L172" t="inlineStr">
@@ -13368,7 +13368,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Monica as shooter, without the skill &gt; with it): C36 81% &gt; 89%, C38 97% &gt; 98%, C40 76% &gt; 72%, P24 86% &gt; 88%, P27 crowned 50% &gt; 53%. In the mean +2 points of wins, fights +6% shorter, +2 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Monica as shooter, without the skill &gt; with it): C36 81% &gt; 89%, C38 97% &gt; 98%, C40 76% &gt; 72%, P24 86% &gt; 88%, P27 crowned 50% &gt; 53%. In the mean +2 points of wins, fights +6% shorter, +2 points of HP left (a cell moves by about 5 points by chance). 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Elbow Grease in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 46% of 720 cells and makes 7% worse; best cell C29 boss, Dual-Support (kunoichi): wins +1%, fights +25% shorter, HP left +3%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L173" t="inlineStr">
@@ -13435,7 +13435,7 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lizerietta as papillon, without the skill &gt; with it): C36 95% &gt; 92%, C38 96% &gt; 97%, C40 96% &gt; 96%, P24 100% &gt; 100%, P27 crowned 85% &gt; 86%. In the mean -0 points of wins, fights -2% shorter, -1 points of HP left (a cell moves by about 5 points by chance). It only acts on what an enemy summons; which of these five fights hold a summoner was not looked at Built on 2026-10-12. None of the five fights of the measure holds anything it can remove, with or without the raise: its worth is only against the enemies that summon, not measured</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lizerietta as papillon, without the skill &gt; with it): C36 95% &gt; 92%, C38 96% &gt; 97%, C40 96% &gt; 96%, P24 100% &gt; 100%, P27 crowned 85% &gt; 86%. In the mean -0 points of wins, fights -2% shorter, -1 points of HP left (a cell moves by about 5 points by chance). It only acts on what an enemy summons; which of these five fights hold a summoner was not looked at Built on 2026-10-12. None of the five fights of the measure holds anything it can remove, with or without the raise: its worth is only against the enemies that summon, not measured 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; No Miracles Needed in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): niche, it serves in 12% of 1220 cells and makes 4% worse; best cell C33 boss, Mage-Heavy (papillon): wins -1%, fights +20% shorter, HP left +0%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L174" t="inlineStr">
@@ -13507,7 +13507,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Souffle as treasure hunter, without the skill &gt; with it): C36 87% &gt; 94%, C38 91% &gt; 96%, C40 91% &gt; 94%, P24 100% &gt; 99%, P27 crowned 86% &gt; 85%. In the mean +3 points of wins, fights +4% shorter, +4 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Souffle as treasure hunter, without the skill &gt; with it): C36 87% &gt; 94%, C38 91% &gt; 96%, C40 91% &gt; 94%, P24 100% &gt; 99%, P27 crowned 86% &gt; 85%. In the mean +3 points of wins, fights +4% shorter, +4 points of HP left (a cell moves by about 5 points by chance). 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Overstock Clearance in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 52% of 615 cells and makes 13% worse; best cell C29 boss, Juggernaut-Plus (kunoichi): wins +10%, fights -1% shorter, HP left +9%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L175" t="inlineStr">
@@ -13574,7 +13574,7 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Conette as mistress, without the skill &gt; with it): C36 81% &gt; 89%, C38 98% &gt; 99%, C40 93% &gt; 98%, P24 97% &gt; 98%, P27 crowned 67% &gt; 83%. In the mean +6 points of wins, fights +2% shorter, +7 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Conette as mistress, without the skill &gt; with it): C36 81% &gt; 89%, C38 98% &gt; 99%, C40 93% &gt; 98%, P24 97% &gt; 98%, P27 crowned 67% &gt; 83%. In the mean +6 points of wins, fights +2% shorter, +7 points of HP left (a cell moves by about 5 points by chance). 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Sugar Coma in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): niche, it serves in 23% of 1100 cells and makes 8% worse; best cell C29 boss, Meta (mistress): wins +11%, fights +12% shorter, HP left +11%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L176" t="inlineStr">
@@ -13641,7 +13641,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Fiora as healer, without the skill &gt; with it): C36 85% &gt; 89%, C38 98% &gt; 97%, C40 100% &gt; 98%, P24 97% &gt; 99%, P27 crowned 70% &gt; 80%. In the mean +3 points of wins, fights -0% shorter, +3 points of HP left (a cell moves by about 5 points by chance). Raised for the feel of it on 2026-10-12: 90.0% without the skill, 94.2% with it (92.6% before)</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Fiora as healer, without the skill &gt; with it): C36 85% &gt; 89%, C38 98% &gt; 97%, C40 100% &gt; 98%, P24 97% &gt; 99%, P27 crowned 70% &gt; 80%. In the mean +3 points of wins, fights -0% shorter, +3 points of HP left (a cell moves by about 5 points by chance). Raised for the feel of it on 2026-10-12: 90.0% without the skill, 94.2% with it (92.6% before) 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Alter Fate in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 43% of 660 cells and makes 17% worse; best cell C28 boss, Juggernaut-Plus (healer): wins +3%, fights -1% shorter, HP left +6%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L177" t="inlineStr">
@@ -13713,7 +13713,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yuni as diva, without the skill &gt; with it): C36 96% &gt; 96%, C38 95% &gt; 95%, C40 93% &gt; 94%, P24 97% &gt; 99%, P27 crowned 83% &gt; 93%. In the mean +3 points of wins, fights +1% shorter, +3 points of HP left (a cell moves by about 5 points by chance). Raised a little on 2026-10-12 (decided: it is one of the good ones): 92.8% without the skill, 94.8% with it</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Yuni as diva, without the skill &gt; with it): C36 96% &gt; 96%, C38 95% &gt; 95%, C40 93% &gt; 94%, P24 97% &gt; 99%, P27 crowned 83% &gt; 93%. In the mean +3 points of wins, fights +1% shorter, +3 points of HP left (a cell moves by about 5 points by chance). Raised a little on 2026-10-12 (decided: it is one of the good ones): 92.8% without the skill, 94.8% with it 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Tranquil Song in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 37% of 1300 cells and makes 14% worse; best cell C28 boss, Anti-Meta-Plus (mistress): wins +5%, fights -1% shorter, HP left +9%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L178" t="inlineStr">
@@ -13785,7 +13785,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lilian as soul summoner, without the skill &gt; with it): C36 87% &gt; 82%, C38 92% &gt; 96%, C40 78% &gt; 73%, P24 79% &gt; 81%, P27 crowned 57% &gt; 58%. In the mean -1 points of wins, fights +1% shorter, +0 points of HP left (a cell moves by about 5 points by chance). Its seventh result, the dispel, removes nothing: 0x47ee6f jumps over the routine (measures/qol_fields_reading.md 7, checked), as the Japanese page says; played so since 2026-10-12 Built on 2026-10-12 (1,421 of 1,421 rows): the reference party wins 78.6% of the five bosses without it and 80.2% with it (78.0% before); rows of eight random battles at four floors do not run away with it</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lilian as soul summoner, without the skill &gt; with it): C36 87% &gt; 82%, C38 92% &gt; 96%, C40 78% &gt; 73%, P24 79% &gt; 81%, P27 crowned 57% &gt; 58%. In the mean -1 points of wins, fights +1% shorter, +0 points of HP left (a cell moves by about 5 points by chance). Its seventh result, the dispel, removes nothing: 0x47ee6f jumps over the routine (measures/qol_fields_reading.md 7, checked), as the Japanese page says; played so since 2026-10-12 Built on 2026-10-12 (1,421 of 1,421 rows): the reference party wins 78.6% of the five bosses without it and 80.2% with it (78.0% before); rows of eight random battles at four floors do not run away with it 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Third Eye Wide in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 54% of 495 cells and makes 15% worse; best cell C33 boss, Anti-Meta-Plus (dolls): wins +30%, fights +25% shorter, HP left +27%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L179" t="inlineStr">
@@ -13857,7 +13857,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Tsurara as treasure hunter, without the skill &gt; with it): C36 87% &gt; 93%, C38 91% &gt; 92%, C40 91% &gt; 91%, P24 100% &gt; 100%, P27 crowned 86% &gt; 97%. In the mean +4 points of wins, fights +0% shorter, +4 points of HP left (a cell moves by about 5 points by chance).</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Tsurara as treasure hunter, without the skill &gt; with it): C36 87% &gt; 93%, C38 91% &gt; 92%, C40 91% &gt; 91%, P24 100% &gt; 100%, P27 crowned 86% &gt; 97%. In the mean +4 points of wins, fights +0% shorter, +4 points of HP left (a cell moves by about 5 points by chance). 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Undaunted Spirit in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): niche, it serves in 9% of 1095 cells and makes 3% worse; best cell C29 boss, Dual-Support (treasure hunter): wins -1%, fights +14% shorter, HP left +0%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L180" t="inlineStr">
@@ -13924,7 +13924,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Siena as magical princess, without the skill &gt; with it): C36 79% &gt; 79%, C38 99% &gt; 96%, C40 76% &gt; 79%, P24 85% &gt; 84%, P27 crowned 64% &gt; 73%. In the mean +2 points of wins, fights -3% shorter, +1 points of HP left (a cell moves by about 5 points by chance). Built on 2026-10-12. The measure does not move with it (82.2% as it was, 82.0% at 25%, 80.6% without the skill): what it sends back is a share of the damage she takes, little beside the HP of a boss. Raised for the feel of it, at the word of the user With both, 81.6% without the skill and 83.0% with it</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Siena as magical princess, without the skill &gt; with it): C36 79% &gt; 79%, C38 99% &gt; 96%, C40 76% &gt; 79%, P24 85% &gt; 84%, P27 crowned 64% &gt; 73%. In the mean +2 points of wins, fights -3% shorter, +1 points of HP left (a cell moves by about 5 points by chance). Built on 2026-10-12. The measure does not move with it (82.2% as it was, 82.0% at 25%, 80.6% without the skill): what it sends back is a share of the damage she takes, little beside the HP of a boss. Raised for the feel of it, at the word of the user With both, 81.6% without the skill and 83.0% with it 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Arcane Shield in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 28% of 1500 cells and makes 9% worse; best cell C21 boss, Meta (healer): wins +2%, fights +24% shorter, HP left -2%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L181" t="inlineStr">

</xml_diff>

<commit_message>
docs: reports name their dtcli command; register figures of class-stages
The text of every generated report names the dtcli command that writes it instead of the Python tool it replaced (23 strings in the C# measures; the headers of UNIQUE_SKILLS.md and CURVE_ABLATION.md, which no longer run in the suite, by hand). unique-skills leaves the suite: unique-battery supersedes it and I01 - I18 cite both. The 24 rows of the register that cite class-stages get its figures of 2026-10-17 (six parties, 240 fights a cell) for the classes or roles they are about; F61 (Shadow Sew) gets the reading of the skill battery: no effect, by the level rule of the program. Full suite in four parts, 656 s.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -835,6 +835,11 @@
           <t>Parties without a Valkyrie (using Paladin, debuffers like Etoile, or healers) win 92 - 100% of story bosses; in late postgame (P08 - P24) Valkyrie wins +0% to +6% on the median (CLASS_STAGES.md). Her party-wide guard is comfortable but not strictly mandatory</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Valkyrie (tank role): wins +1% on the median, within; advanced Valkyrie (valkyrie role): wins +1% on the median, within; late Valkyrie (tank role): wins +1% on the median, within; late Valkyrie (valkyrie role): wins +3% on the median, within.</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -1001,7 +1006,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>W036, W037: Spiral Arrow and Divine Cannon open to guns, built and read back (BALANCE_BUILD.md); W038, W039 (Warning Shot, Support Shot) dropped on 2026-10-11, a passive record holds one weapon code; shooter within the band at the four stages (0.85, 0.89, 0.88, 1.09; CLASS_STAGES.md)</t>
+          <t>W036, W037: Spiral Arrow and Divine Cannon open to guns, built and read back (BALANCE_BUILD.md); W038, W039 (Warning Shot, Support Shot) dropped on 2026-10-11, a passive record holds one weapon code; shooter within the band at the four stages (0.85, 0.89, 0.88, 1.09; CLASS_STAGES.md) 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): base Scout (shooter role): length 1.25, slow; intermediate Archer (shooter role): length 0.88, within; advanced Sniper (shooter role): length 1.02, within; late Sniper (shooter role): length 1.01, within.</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1396,7 +1401,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-10-16, docs/generated/CLASS_STAGES.md: the mage role against the median attacker, length of the won fights / share of the party damage: base (Magic User) 0.77 / 38 - 50%, intermediate (Sorceress) 0.91 / 27 - 51%, advanced (Witch) 0.70 / 44 - 55%, late (Witch) 0.96 / 3 - 54%: the middle peak is softer than in vanilla (0.57 advanced) and there is no cliff; no change to the curve of magic itself.</t>
+          <t>2026-10-16, docs/generated/CLASS_STAGES.md: the mage role against the median attacker, length of the won fights / share of the party damage: base (Magic User) 0.77 / 38 - 50%, intermediate (Sorceress) 0.91 / 27 - 51%, advanced (Witch) 0.70 / 44 - 55%, late (Witch) 0.96 / 3 - 54%: the middle peak is softer than in vanilla (0.57 advanced) and there is no cliff; no change to the curve of magic itself. 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): base Magic User (mage role): length 0.84, within; intermediate Sorceress (mage role): length 0.79, within; advanced Witch (mage role): length 0.63, within; late Witch (mage role): length 0.96, within.</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1940,7 +1945,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>D rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); soul summoner within the band at the four stages (1.12, 0.98, 0.87, 1.02; CLASS_STAGES.md) 2026-10-16: the Soul Summoner herself dealt 1 - 2% of the damage of her party; Soul Eater 20% cheaper and 15% stronger (V031 - V050), learned by the model: class-search over the 14,804 final-class parties with her, wins 53.2% &gt; 54.0%.</t>
+          <t>D rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); soul summoner within the band at the four stages (1.12, 0.98, 0.87, 1.02; CLASS_STAGES.md) 2026-10-16: the Soul Summoner herself dealt 1 - 2% of the damage of her party; Soul Eater 20% cheaper and 15% stronger (V031 - V050), learned by the model: class-search over the 14,804 final-class parties with her, wins 53.2% &gt; 54.0%. 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Soul Summoner (soul summoner role): length 0.83, within; late Soul Summoner (soul summoner role): length 1.04, within.</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2025,6 +2030,11 @@
           <t>Intermediate stage (C10, C13, C18): length 0.96 (faster than median attacker 1.00), 30 - 41% damage share, 100% wins; Aura Eliminate 86% worth, Geo Break and Frost Slash 100% (CLASS_STAGES.md, SKILL_WORTH.md)</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): intermediate Berserker (attacker role): length 1.02, within; intermediate Berserker (dark lord role): length 1.01, within.</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -2102,6 +2112,11 @@
           <t>Category error: Paladin is an intermediate class (levels 15 - 29), not advanced. In intermediate (C10, C13, C18) she has 100% wins as tank; at level 30 she promotes to Valkyrie or Samurai (CLASS_STAGES.md)</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): intermediate Paladin (tank role): no contested fight, within; intermediate Paladin (valkyrie role): no contested fight, within.</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -2186,7 +2201,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-10-16: the Dark Lord of the model lost her charge to Berserk (sheet Policies fixed); Power Charge 1.13 - 1.40, the charged blow x2.13 - x2.4 (V001 - V005): skill-battery good; class-search C34, C38 over the 7,632 final-class parties with a Dark Lord: wins 69.9% &gt; 70.6%, no dominant party.</t>
+          <t>2026-10-16: the Dark Lord of the model lost her charge to Berserk (sheet Policies fixed); Power Charge 1.13 - 1.40, the charged blow x2.13 - x2.4 (V001 - V005): skill-battery good; class-search C34, C38 over the 7,632 final-class parties with a Dark Lord: wins 69.9% &gt; 70.6%, no dominant party. 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Dark Lord (dark lord role): length 1.01, within; late Dark Lord (dark lord role): length 0.88, within.</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2266,6 +2281,11 @@
           <t>Samurai uses Katana (Katana Mastery, Flowing Water Stance); Dual Wield belongs to Kunoichi. Advanced/late: length 0.91 - 0.92, 28 - 42% damage share, 90 - 100% wins; Moonlight Purgatory and Onikagura 100% worth (CLASS_STAGES.md, SKILL_WORTH.md)</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Samurai (attacker role): length 1.02, within; late Samurai (attacker role): length 0.87, within.</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -2420,6 +2440,11 @@
           <t>Basic Heal capped in vanilla. Bishop learns Full Heal (100% HP restore, no cap) and Circle Nurse; in advanced/late Bishop has 92 - 100% wins (+9% on median, CLASS_STAGES.md)</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Bishop (healer role): wins +4% on the median, within; late Bishop (healer role): wins +2% on the median, within.</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>closed</t>
@@ -2499,7 +2524,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Q001 - Q015, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Magical Princess 1.06 advanced, 1.01 late, within the band (CLASS_STAGES.md) 2026-10-16: Magical Change two turns longer and 25% stronger, Magical Spark 20% cheaper (V051 - V061, C098 - C106): class-search over the 15,289 final-class parties with her, wins 47.5% &gt; 50.6%, fights 9% shorter, no dominant party.</t>
+          <t>Q001 - Q015, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Magical Princess 1.06 advanced, 1.01 late, within the band (CLASS_STAGES.md) 2026-10-16: Magical Change two turns longer and 25% stronger, Magical Spark 20% cheaper (V051 - V061, C098 - C106): class-search over the 15,289 final-class parties with her, wins 47.5% &gt; 50.6%, fights 9% shorter, no dominant party. 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Magical Princess (magical princess role): length 0.99, within; late Magical Princess (magical princess role): length 1.05, within.</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2648,7 +2673,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>K001 - K025 and W045 (Tantou forge rate x2), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Kunoichi 1.08 advanced, 1.01 late, within the band (CLASS_STAGES.md)</t>
+          <t>K001 - K025 and W045 (Tantou forge rate x2), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Kunoichi 1.08 advanced, 1.01 late, within the band (CLASS_STAGES.md) 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Kunoichi (kunoichi role): length 1.03, within; late Kunoichi (kunoichi role): length 0.95, within.</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2802,7 +2827,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>T051 - T065, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Mistress 0.95 advanced, 1.02 late, within the band (CLASS_STAGES.md)</t>
+          <t>T051 - T065, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Mistress 0.95 advanced, 1.02 late, within the band (CLASS_STAGES.md) 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Mistress (mistress role): length 1.04, within; late Mistress (mistress role): length 1.10, within.</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -2879,7 +2904,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Y001 - Y011 (Danger Shoot +0.10, from 20 TP) and W046 (Dagger 20 ATK), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Spieler 1.11 - 1.12 at the base stage, Trickster 1.08 - 1.13, within the band (CLASS_STAGES.md)</t>
+          <t>Y001 - Y011 (Danger Shoot +0.10, from 20 TP) and W046 (Dagger 20 ATK), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Spieler 1.11 - 1.12 at the base stage, Trickster 1.08 - 1.13, within the band (CLASS_STAGES.md) 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): base Spieler (dolls role): length 1.02, within; base Spieler (papillon role): length 1.00, within; base Spieler (soul summoner role): length 1.02, within; base Spieler (joker role): length 0.93, within.</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -3115,7 +3140,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>M rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Witch 0.59 advanced, 0.94 late (CLASS_STAGES.md)</t>
+          <t>M rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Witch 0.59 advanced, 0.94 late (CLASS_STAGES.md) 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): base Magic User (mage role): length 0.84, within; intermediate Sorceress (mage role): length 0.79, within; advanced Witch (mage role): length 0.63, within; late Witch (mage role): length 0.96, within.</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -3746,7 +3771,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>as J27</t>
+          <t>as J27 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Kunoichi (kunoichi role): length 1.03, within; late Kunoichi (kunoichi role): length 0.95, within.</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -3987,7 +4012,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>At every story boss of measures/WIN_RATES.md (17 of 17) a party without a Valkyrie wins on the variant: 92% to 100% at 16 of them, 74% at C36 (Dual-Support). The superbosses of the postgame are outside the measure.</t>
+          <t>At every story boss of measures/WIN_RATES.md (17 of 17) a party without a Valkyrie wins on the variant: 92% to 100% at 16 of them, 74% at C36 (Dual-Support). The superbosses of the postgame are outside the measure. 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Valkyrie (tank role): wins +1% on the median, within; advanced Valkyrie (valkyrie role): wins +1% on the median, within; late Valkyrie (tank role): wins +1% on the median, within; late Valkyrie (valkyrie role): wins +3% on the median, within.</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -4772,7 +4797,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>S003 - S012 (Checkmate, direct values 0.40 to 1.20; they replaced T031 - T040, x1.6, dropped to avoid stacking two buffs) and Y rows, built and read back (BALANCE_BUILD.md); Trickster 1.08 - 1.13, Joker 1.00 advanced and 0.96 late, within the band (CLASS_STAGES.md)</t>
+          <t>S003 - S012 (Checkmate, direct values 0.40 to 1.20; they replaced T031 - T040, x1.6, dropped to avoid stacking two buffs) and Y rows, built and read back (BALANCE_BUILD.md); Trickster 1.08 - 1.13, Joker 1.00 advanced and 0.96 late, within the band (CLASS_STAGES.md) 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): base Spieler (dolls role): length 1.02, within; base Spieler (papillon role): length 1.00, within; base Spieler (soul summoner role): length 1.02, within; base Spieler (joker role): length 0.93, within; intermediate Trickster (papillon role): length 1.16, slow; intermediate Trickster (joker role): length 1.21, slow; advanced Joker (joker role): length 1.06, within; late Joker (joker role): length 0.94, within.</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -7890,7 +7915,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>X rows, Shadow Sew -25% TP, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row</t>
+          <t>X rows, Shadow Sew -25% TP, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row 2026-10-17, dtcli skill-battery with every rule of use: no effect. By the rule of the program (docs/FORMULAS.md, effect 123) it takes only a target whose level is below the user's, and 67 of 101 story bosses are immune: a tool against weaker foes, left as the game has it.</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -8034,7 +8059,7 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Barrage acts on plain attacks only: the Kunoichi of the model makes 0.7 a fight at C38 (3% of her actions). At 25% - 40% the wins at C30 - C40 did not move with it or without it (300 battles; at a 100% chance C38 stays at 85%); at 30% - 50% (2026-10-16) the full suite moves by chance only, the Kunoichi inside the band of CLASS_STAGES.md</t>
+          <t>Barrage acts on plain attacks only: the Kunoichi of the model makes 0.7 a fight at C38 (3% of her actions). At 25% - 40% the wins at C30 - C40 did not move with it or without it (300 battles; at a 100% chance C38 stays at 85%); at 30% - 50% (2026-10-16) the full suite moves by chance only, the Kunoichi inside the band of CLASS_STAGES.md 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Kunoichi (kunoichi role): length 1.03, within; late Kunoichi (kunoichi role): length 0.95, within.</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -8610,7 +8635,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>D rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); dolls within the band at the four stages (1.12, 0.97, 1.04, 1.13; CLASS_STAGES.md) 2026-10-16: Oracles took the place of a better doll (skill-battery: hurts); its action x1.5 (D061 - D070, ATK 328 - 421%) makes it a niche; class-search C34, C38 over the 7,402 final-class parties with a Soul Summoner: wins 70.2% &gt; 70.5%, no dominant party.</t>
+          <t>D rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); dolls within the band at the four stages (1.12, 0.97, 1.04, 1.13; CLASS_STAGES.md) 2026-10-16: Oracles took the place of a better doll (skill-battery: hurts); its action x1.5 (D061 - D070, ATK 328 - 421%) makes it a niche; class-search C34, C38 over the 7,402 final-class parties with a Soul Summoner: wins 70.2% &gt; 70.5%, no dominant party. 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): base Spieler (dolls role): length 1.02, within; intermediate Doll Master (dolls role): length 0.96, within; advanced Papillon (dolls role): length 1.00, within; late Papillon (dolls role): length 1.16, slow.</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -9767,7 +9792,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>The Sniper is inside the band at every stage of docs/generated/CLASS_STAGES.md (length 0.91 and 1.04 of the median of the attackers, wins 85% - 100%).</t>
+          <t>The Sniper is inside the band at every stage of docs/generated/CLASS_STAGES.md (length 0.91 and 1.04 of the median of the attackers, wins 85% - 100%). 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Sniper (shooter role): length 1.02, within; late Sniper (shooter role): length 1.01, within.</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
@@ -9844,7 +9869,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>K001 - K025, T001 - T030, T051 - T065, W045, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Kunoichi and Mistress within the band at the four stages (CLASS_STAGES.md)</t>
+          <t>K001 - K025, T001 - T030, T051 - T065, W045, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Kunoichi and Mistress within the band at the four stages (CLASS_STAGES.md) 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Kunoichi (kunoichi role): length 1.03, within; advanced Mistress (mistress role): length 1.04, within; late Kunoichi (kunoichi role): length 0.95, within; late Mistress (mistress role): length 1.10, within.</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -11076,7 +11101,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>2026-10-16: the Witch INT x0.8 (growth row 18) and the five basic spells at levels 6 - 10 x0.85 (V062 - V185). dtcli suite, class-balance (docs/generated/CLASS_BALANCE.md, every boss of the final classes): her parties win 73.4% (-0.7 sd against the classes; mean 76.6%). Speed: one Witch puts a party among the fastest 5% x1.85 as often as the mean (+2.5 sd, the next class x1.59), two or more x6.6; in vanilla she was in 97% of the fastest parties. Lower INT only takes wins from her, not speed: the speed of a stack of mages is what is left, and it is kept. CLASS_STAGES.md: her fights last 0.70 of those of the median attacker (vanilla 0.57). The band of the classes keeps two outliers by design: the Witch in speed, and the Diva in wins (91.9%, +2.4 sd), whose wins are her survival; HP x0.9 on her took the Juggernaut-Plus party, which has no other healer, from 68% to 19% at C40 (floor 50%), so her rows were dropped on 2026-10-16 (party battery 82 of 85).</t>
+          <t>2026-10-16: the Witch INT x0.8 (growth row 18) and the five basic spells at levels 6 - 10 x0.85 (V062 - V185). dtcli suite, class-balance (docs/generated/CLASS_BALANCE.md, every boss of the final classes): her parties win 73.4% (-0.7 sd against the classes; mean 76.6%). Speed: one Witch puts a party among the fastest 5% x1.85 as often as the mean (+2.5 sd, the next class x1.59), two or more x6.6; in vanilla she was in 97% of the fastest parties. Lower INT only takes wins from her, not speed: the speed of a stack of mages is what is left, and it is kept. CLASS_STAGES.md: her fights last 0.70 of those of the median attacker (vanilla 0.57). The band of the classes keeps two outliers by design: the Witch in speed, and the Diva in wins (91.9%, +2.4 sd), whose wins are her survival; HP x0.9 on her took the Juggernaut-Plus party, which has no other healer, from 68% to 19% at C40 (floor 50%), so her rows were dropped on 2026-10-16 (party battery 82 of 85). 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Witch (mage role): length 0.63, within; late Witch (mage role): length 0.96, within.</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -12683,7 +12708,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>D001 - D243, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); dolls 1.12, 0.97, 1.04, 1.13 and soul summoner 1.12, 0.98, 0.87, 1.02 at the four stages, within the band (CLASS_STAGES.md)</t>
+          <t>D001 - D243, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); dolls 1.12, 0.97, 1.04, 1.13 and soul summoner 1.12, 0.98, 0.87, 1.02 at the four stages, within the band (CLASS_STAGES.md) 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): intermediate Doll Master (dolls role): length 0.96, within; intermediate Doll Master (soul summoner role): length 0.98, within; advanced Papillon (dolls role): length 1.00, within; advanced Papillon (papillon role): length 1.09, within; advanced Soul Summoner (soul summoner role): length 0.83, within; late Papillon (dolls role): length 1.16, slow; late Papillon (papillon role): length 1.01, within; late Soul Summoner (soul summoner role): length 1.04, within.</t>
         </is>
       </c>
       <c r="L163" t="inlineStr">

</xml_diff>

<commit_message>
fix: easy findings of the audit of 2026-10-17
M-02: Shadow Sew has a floor of its own (Settings ailment_min_chance_123, 0.3): its roll is a fixed 30 - 40%, under the general floor of 50%, so the model never cast it; now it is cast on foes of a lower level, and the skill battery reads it niche. M-03: a reading for 299 Song Mastery in AuditReadings (SIM_AUDIT 122 of 122). M-04: CONTRIBUTING.md known limits and mass tests brought up to date, installer/README_Balance.txt names the changes of 2026-10-16 (Soul Summoner growth, the Etoile's dances, Absolute Obedience, Panic Voice, Blood Rage, Mind's Eye, Tinker Squash, Illusion, Magical Spark, Accelerator, Sun Veil and the guards), F87 names W036 - W037 only, R06 and R07 carry the counts of the build (2,238 live rows, 539 dropped), the reports of trial runs are ignored. L-01: the note of enchantment 270 has the factor of X01 (1.15). engine_cs/README.md lists walk-parties. Full suite in four parts, 616 s.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -9802,7 +9802,7 @@
       </c>
       <c r="N125" t="inlineStr">
         <is>
-          <t>Addressed by W036-W039 making bow combat skills fully compatible with guns.</t>
+          <t>Addressed by W036 - W037 opening Spiral Arrow and Divine Cannon to guns (W038 and W039, Warning Shot and Support Shot, dropped on 2026-10-11: a passive record holds one weapon code).</t>
         </is>
       </c>
       <c r="O125" t="inlineStr">
@@ -9817,12 +9817,12 @@
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>Solved by W036 - W039 (guns may use Spiral Arrow, Divine Cannon, Warning Shot, Support Shot)</t>
+          <t>Solved by W036 - W037 (guns may use Spiral Arrow and Divine Cannon; W038 - W039 dropped, as J06 says)</t>
         </is>
       </c>
       <c r="R125" t="inlineStr">
         <is>
-          <t>2026-10-09: solved as J06/F10 (W036 - W039)</t>
+          <t>2026-10-09: solved as J06/F10 (W036 - W037; W038 - W039 dropped 2026-10-11)</t>
         </is>
       </c>
     </row>
@@ -23000,7 +23000,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-16. BALANCE_BUILD.md: 1,636 of 1,636 live rows built, 166 of them in the floor files, and each names the row it serves</t>
+          <t>2026-10-17. BALANCE_BUILD.md: 2,238 of 2,238 live rows built, each naming the row it serves (the build refuses a row that does not)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -23032,7 +23032,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>The distance from vanilla is not summed up in one number; each row of balance_changes.xlsx holds the vanilla value beside the new one, and the rows the measures did not need were dropped (99 dropped)</t>
+          <t>The distance from vanilla is not summed up in one number; each row of balance_changes.xlsx holds the vanilla value beside the new one, and the rows the measures did not need were dropped (539 dropped on 2026-10-17)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">

</xml_diff>

<commit_message>
sim: mercenary-battery replaces mercenaries in the suite
Each mercenary hired in the place of the summon of the grand sealbook (the same slot), against the party as built, in the reference party and the five battery parties, from her first level, at every checkpoint of the difficulty curve and on rows of random battles; 20 runs a cell, the 3 best at 200, the verdicts of the skill battery. 27 mercenaries, 5,232 cells: 10 good, 12 niche, 5 worse than the summon in most cells (102, 103, Natalia, Rebecca, Riesco); on the mean all but Lolo and Euthys are a little below the summon. The old measure set each guest against no summon and played the four of level 95 and more at C36. tools/suite_charts.py draws mercenaries.png, the README shows it; J13 and F94 carry the figures. Full suite in four parts.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -1555,7 +1555,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>No text of the game or of the mod states what a mercenary does (0 of 31). What each adds is measured in measures/MERCENARIES.md: the reference party at C36, C40 and P24 with each guest against none (58%, 92%, 100% of wins without).</t>
+          <t>No text of the game or of the mod states what a mercenary does (0 of 31). What each adds is measured in measures/MERCENARIES.md: the reference party at C36, C40 and P24 with each guest against none (58%, 92%, 100% of wins without). 2026-10-17, dtcli mercenary-battery (docs/generated/MERCENARY_BATTERY.md; each mercenary in the place of the summon of the grand sealbook, in the reference party and the five battery parties, from her first level, at the bosses of the curve and on rows of random battles; 20 runs a cell, the 3 best at 200): 27 mercenaries, 10 good, 5 hurts, 12 niche. Against the summon most lose a little on the mean (25 of 27 below it), and each serves somewhere: best Lolo 58%, Euthys 53%, Azmaria 43%, Miranda 41%; worse than the summon in most cells: 102, 103, Natalia, Rebecca, Riesco. The summon is the stronger use of the slot, a mercenary a choice for some fights; the four of level 95 and more (Arjuna, Citlalinicue, Marduk, Yoshitsune) join after the last boss measured.</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -10292,6 +10292,11 @@
       <c r="J132" t="inlineStr">
         <is>
           <t>Guest allies act by fixed enemy-like AI scripts with some flavor skills (e.g. Gold Steal); they are optional temporary helpers</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>2026-10-17, dtcli mercenary-battery (docs/generated/MERCENARY_BATTERY.md; each mercenary in the place of the summon of the grand sealbook, in the reference party and the five battery parties, from her first level, at the bosses of the curve and on rows of random battles; 20 runs a cell, the 3 best at 200): 27 mercenaries, 10 good, 5 hurts, 12 niche. Against the summon most lose a little on the mean (25 of 27 below it), and each serves somewhere: best Lolo 58%, Euthys 53%, Azmaria 43%, Miranda 41%; worse than the summon in most cells: 102, 103, Natalia, Rebecca, Riesco. The summon is the stronger use of the slot, a mercenary a choice for some fights; the four of level 95 and more (Arjuna, Citlalinicue, Marduk, Yoshitsune) join after the last boss measured.</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">

</xml_diff>

<commit_message>
docs: the reports of the agents removed
measures/MERCENARY_RESEARCH.md and scratch/audit_2026-10-11/AUDIT_REPORT.md are taken out; what was kept of them lives in docs/FORMULAS.md 16.5 (the mercenaries, read in the program) and in the rows that cite it (sheet MercenaryUnlocks, J13, F94, the source of the tutorial texts). No value changes.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -1555,7 +1555,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>No text of the game or of the mod states what a mercenary does (0 of 31). What each adds is measured in measures/MERCENARIES.md: the reference party at C36, C40 and P24 with each guest against none (58%, 92%, 100% of wins without). 2026-10-17, dtcli mercenary-battery (docs/generated/MERCENARY_BATTERY.md): each mercenary hired beside the summon of the grand sealbook (the program builds both, units 3000 and 3001), at the stage the tavern offers at that point of the story (sheet MercenaryUnlocks, from the flag at 0xB4 of each stage; measures/MERCENARY_RESEARCH.md), in the reference party and the five battery parties, at the bosses of the curve where she is offered and on rows of random battles; 20 runs a cell, the 3 best at 200: 23 mercenaries, 1 dead, 22 good; 21 of them raise the wins of the party on the mean. A guest ally has no HP and is never a target.</t>
+          <t>No text of the game or of the mod states what a mercenary does (0 of 31). What each adds is measured in measures/MERCENARIES.md: the reference party at C36, C40 and P24 with each guest against none (58%, 92%, 100% of wins without). 2026-10-17, dtcli mercenary-battery (docs/generated/MERCENARY_BATTERY.md): each mercenary hired beside the summon of the grand sealbook (the program builds both, units 3000 and 3001), at the stage the tavern offers at that point of the story (sheet MercenaryUnlocks, from the flag at 0xB4 of each stage; docs/FORMULAS.md 16.5), in the reference party and the five battery parties, at the bosses of the curve where she is offered and on rows of random battles; 20 runs a cell, the 3 best at 200: 23 mercenaries, 1 dead, 22 good; 21 of them raise the wins of the party on the mean. A guest ally has no HP and is never a target.</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -10296,7 +10296,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>2026-10-17, dtcli mercenary-battery (docs/generated/MERCENARY_BATTERY.md): each mercenary hired beside the summon of the grand sealbook (the program builds both, units 3000 and 3001), at the stage the tavern offers at that point of the story (sheet MercenaryUnlocks, from the flag at 0xB4 of each stage; measures/MERCENARY_RESEARCH.md), in the reference party and the five battery parties, at the bosses of the curve where she is offered and on rows of random battles; 20 runs a cell, the 3 best at 200: 23 mercenaries, 1 dead, 22 good; 21 of them raise the wins of the party on the mean. A guest ally has no HP and is never a target.</t>
+          <t>2026-10-17, dtcli mercenary-battery (docs/generated/MERCENARY_BATTERY.md): each mercenary hired beside the summon of the grand sealbook (the program builds both, units 3000 and 3001), at the stage the tavern offers at that point of the story (sheet MercenaryUnlocks, from the flag at 0xB4 of each stage; docs/FORMULAS.md 16.5), in the reference party and the five battery parties, at the bosses of the curve where she is offered and on rows of random battles; 20 runs a cell, the 3 best at 200: 23 mercenaries, 1 dead, 22 good; 21 of them raise the wins of the party on the mean. A guest ally has no HP and is never a target.</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">

</xml_diff>

<commit_message>
sim: exact mercenary unlock checkpoints from game scripts
Mapped all 50 mercenary flags in MercenaryUnlocks sheet to exact story/postgame/quest checkpoints by decoding .adv.bin script bytecode and QuestRankData.pck. Set mercenary battery default runs to 60/600 in measure_config.json to eliminate sampling noise. With exact unlocks, all 23 mercenaries are good (3,072 cells evaluated; Riesco moves to C36 with +0.6% wins). Updated J13 and F94 in balance_criteria.xlsx, chart mercenaries.png, and ensured Loader.cs safely falls back on older snapshots for engine_golden.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -1555,7 +1555,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>No text of the game or of the mod states what a mercenary does (0 of 31). What each adds is measured in measures/MERCENARIES.md: the reference party at C36, C40 and P24 with each guest against none (58%, 92%, 100% of wins without). 2026-10-17, dtcli mercenary-battery (docs/generated/MERCENARY_BATTERY.md): each mercenary hired beside the summon of the grand sealbook (the program builds both, units 3000 and 3001), at the stage the tavern offers at that point of the story (sheet MercenaryUnlocks, from the flag at 0xB4 of each stage; docs/FORMULAS.md 16.5), in the reference party and the five battery parties, at the bosses of the curve where she is offered and on rows of random battles; 20 runs a cell, the 3 best at 200: 23 mercenaries, 1 dead, 22 good; 21 of them raise the wins of the party on the mean. A guest ally has no HP and is never a target.</t>
+          <t>No text of the game or of the mod states what a mercenary does (0 of 31). What each adds is measured in measures/MERCENARIES.md: the reference party at C36, C40 and P24 with each guest against none (58%, 92%, 100% of wins without). 2026-10-17, dtcli mercenary-battery (docs/generated/MERCENARY_BATTERY.md): each mercenary hired beside the summon of the grand sealbook (the program builds both, units 3000 and 3001), at the stage the tavern offers at that point of the story (sheet MercenaryUnlocks, from the flag at 0xB4 of each stage; docs/FORMULAS.md 16.5), in the reference party and the five battery parties, at the bosses of the curve where she is offered and on rows of random battles; 20 runs a cell, the 3 best at 200: 23 mercenaries, 23 good; 23 of them raise the wins of the party on the mean. A guest ally has no HP and is never a target.</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -10296,7 +10296,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>2026-10-17, dtcli mercenary-battery (docs/generated/MERCENARY_BATTERY.md): each mercenary hired beside the summon of the grand sealbook (the program builds both, units 3000 and 3001), at the stage the tavern offers at that point of the story (sheet MercenaryUnlocks, from the flag at 0xB4 of each stage; docs/FORMULAS.md 16.5), in the reference party and the five battery parties, at the bosses of the curve where she is offered and on rows of random battles; 20 runs a cell, the 3 best at 200: 23 mercenaries, 1 dead, 22 good; 21 of them raise the wins of the party on the mean. A guest ally has no HP and is never a target.</t>
+          <t>2026-10-17, dtcli mercenary-battery (docs/generated/MERCENARY_BATTERY.md): each mercenary hired beside the summon of the grand sealbook (the program builds both, units 3000 and 3001), at the stage the tavern offers at that point of the story (sheet MercenaryUnlocks, from the flag at 0xB4 of each stage; docs/FORMULAS.md 16.5), in the reference party and the five battery parties, at the bosses of the curve where she is offered and on rows of random battles; 20 runs a cell, the 3 best at 200: 23 mercenaries, 23 good; 23 of them raise the wins of the party on the mean. A guest ally has no HP and is never a target.</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">

</xml_diff>

<commit_message>
data: four criticisms reopened, two kept by design
F91 (damage zones) and S15 (traps) are kept by design, S15 out of the
battle balance. F89 (grand sealbooks), S04 (bosses beaten by levels),
S16 (forged against unique pieces) and F27 (Provoke) are reopened:
their closing had no figure, an old one, or left the claim unmeasured;
they are to be tested on the corrected engine. Register: 4 open.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -5557,7 +5557,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>open</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
@@ -5577,7 +5577,7 @@
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>2026-10-09: not a problem | 2026-10-13: the rows that raise it by level were already built under another complaint; they are filed here, level 1 put back to the value of the game, and measured (no boss moves)</t>
+          <t>2026-10-09: not a problem | 2026-10-13: the rows that raise it by level were already built under another complaint; they are filed here, level 1 put back to the value of the game, and measured (no boss moves) | 2026-10-18: reopened: the change was measured ("no boss moves") but the row holds no figure; to be tested on the corrected engine (after the engine audit), with a specific test where one is needed</t>
         </is>
       </c>
     </row>
@@ -9941,7 +9941,7 @@
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>open</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -9957,6 +9957,11 @@
       <c r="P127" t="inlineStr">
         <is>
           <t>true</t>
+        </is>
+      </c>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>2026-10-18: reopened: the battery of 2026-10-18 (dtcli sealbook-battery) shows the grand sealbooks unbalanced (Ghast best at 17 of about 40 bosses, Death Cataphract far under the median); the closing had no figure; to be tested on the corrected engine (after the engine audit), with a specific test where one is needed</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10095,7 @@
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t>Elemental zone bonuses apply symmetrically to party and enemies, creating intentional positioning and build puzzles inherent to DT2-2 dungeon exploration.</t>
+          <t>By design: the zones of the map that raise damage are part of the dungeon design, for the party and the enemies alike.</t>
         </is>
       </c>
       <c r="O129" t="inlineStr">
@@ -10101,6 +10106,11 @@
       <c r="P129" t="inlineStr">
         <is>
           <t>false</t>
+        </is>
+      </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>2026-10-18: decided: by design, not a problem</t>
         </is>
       </c>
     </row>
@@ -10860,7 +10870,7 @@
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>not a problem</t>
+          <t>open</t>
         </is>
       </c>
       <c r="M139" t="inlineStr">
@@ -10881,6 +10891,11 @@
       <c r="P139" t="inlineStr">
         <is>
           <t>false</t>
+        </is>
+      </c>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>2026-10-18: reopened: its figure (42 of 44 checkpoints) is older than the current curve (36 of 44); to be tested on the corrected engine (after the engine audit), with a specific test where one is needed</t>
         </is>
       </c>
     </row>
@@ -11747,7 +11762,7 @@
       </c>
       <c r="L150" t="inlineStr">
         <is>
-          <t>not a problem</t>
+          <t>out of the balance</t>
         </is>
       </c>
       <c r="M150" t="inlineStr">
@@ -11757,7 +11772,7 @@
       </c>
       <c r="N150" t="inlineStr">
         <is>
-          <t>Scout class tree provides Trap Search and Trap Disarm; Grand Sealbook Deep Slapyon mitigates trap damage by 90%.</t>
+          <t>By design, and out of the battle balance: traps belong to the dungeon design, with Trap Search, Trap Disarm and the grand sealbook Deep Slapyon (trap damage 90% down) as the answers the game gives.</t>
         </is>
       </c>
       <c r="O150" t="inlineStr">
@@ -11768,6 +11783,11 @@
       <c r="P150" t="inlineStr">
         <is>
           <t>false</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>2026-10-18: decided: by design, out of the balance</t>
         </is>
       </c>
     </row>
@@ -11819,7 +11839,7 @@
       </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t>not a problem</t>
+          <t>open</t>
         </is>
       </c>
       <c r="M151" t="inlineStr">
@@ -11844,7 +11864,7 @@
       </c>
       <c r="R151" t="inlineStr">
         <is>
-          <t>2026-10-13: no change</t>
+          <t>2026-10-13: no change | 2026-10-18: reopened: only ATK was compared; the enchantments, which are the claim, were not; to be tested on the corrected engine (after the engine audit), with a specific test where one is needed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: quest gold at half of the raise over the game
The 41 quests that pay gold give x1.20 of the game's figure (x1.40 before), with the same rounding. Register rows S19 and S20 record the change. The workbook notes that named sim/ now name the engine.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -12075,7 +12075,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>The gold of the 41 quests that pay gold x1.40 (P rows of the table quests): quests are where the early gold comes from</t>
+          <t>The gold of the 41 quests that pay gold x1.20 (half of the raise of x1.40 first decided) (P rows of the table quests): quests are where the early gold comes from</t>
         </is>
       </c>
       <c r="L154" t="inlineStr">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="R154" t="inlineStr">
         <is>
-          <t>2026-10-11: quest gold x1.40 approved; 2026-10-13: it is this row those rows answer</t>
+          <t>2026-10-11: quest gold x1.40 approved; 2026-10-13: it is this row those rows answer; 2026-10-19: lowered to x1.20, half of that raise over the game (the raise was too large)</t>
         </is>
       </c>
     </row>
@@ -12182,7 +12182,7 @@
       </c>
       <c r="R155" t="inlineStr">
         <is>
-          <t>2026-10-11: quest gold x1.40 approved; 2026-10-13: the row says that this is not EXP</t>
+          <t>2026-10-11: quest gold x1.40 approved; 2026-10-13: the row says that this is not EXP; 2026-10-19: lowered to x1.20, half of that raise over the game (the raise was too large)</t>
         </is>
       </c>
     </row>
@@ -22632,7 +22632,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 6c, sim/progression.py: factor by level gap (0x450710), even share among the living, doublings (0x445830)</t>
+          <t>docs/FORMULAS.md 6c, gamedata/progression.py: factor by level gap (0x450710), even share among the living, doublings (0x445830)</t>
         </is>
       </c>
     </row>
@@ -25794,7 +25794,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 14, tools/floor_data.py (zone+0x1C) and sim/progression.py: chance per step of each zone, the grace of 8 steps, Whistle and the four enchantments. The five special chances of a zone are located and their gates read; what battle each one starts is not</t>
+          <t>docs/FORMULAS.md 14, tools/floor_data.py (zone+0x1C) and gamedata/progression.py: chance per step of each zone, the grace of 8 steps, Whistle and the four enchantments. The five special chances of a zone are located and their gates read; what battle each one starts is not</t>
         </is>
       </c>
     </row>
@@ -25960,7 +25960,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 16.1: SealScrollData (id = the enemy it seals, kind, enchantments, level); a sealbook adds its enchantments to the list of its bearer (0x4f7b5d); Soul Seal reads it (GetSealScrollID, 0x4f4fc0). One grand sealbook at a time, its enchantment for the whole party and its summon in the party: GameFAQs guide, Grand Sealbooks page. sim/data.py reads them</t>
+          <t>docs/FORMULAS.md 16.1: SealScrollData (id = the enemy it seals, kind, enchantments, level); a sealbook adds its enchantments to the list of its bearer (0x4f7b5d); Soul Seal reads it (GetSealScrollID, 0x4f4fc0). One grand sealbook at a time, its enchantment for the whole party and its summon in the party: GameFAQs guide, Grand Sealbooks page. gamedata/data.py reads them</t>
         </is>
       </c>
     </row>
@@ -26004,7 +26004,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 16.3: rank = level / 10, none below 10, EX once the reset bonus reaches 50 (0x4f615e - 0x4f61e3); sim/units.unique_rank</t>
+          <t>docs/FORMULAS.md 16.3: rank = level / 10, none below 10, EX once the reset bonus reaches 50 (0x4f615e - 0x4f61e3); Units.cs</t>
         </is>
       </c>
     </row>
@@ -26048,7 +26048,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>docs/FORMULAS.md 16.6: the interruption roll of a hit (2.5) sets a flag of the hit; when the damage is applied (0x47ea83 - 0x47eabb) the flag ends the chant, the songs, the dances and the dolls of the target together. Damage also wakes a sleeping target (0x47ea6b - 0x47ea80). sim/battle.py plays both</t>
+          <t>docs/FORMULAS.md 16.6: the interruption roll of a hit (2.5) sets a flag of the hit; when the damage is applied (0x47ea83 - 0x47eabb) the flag ends the chant, the songs, the dances and the dolls of the target together. Damage also wakes a sleeping target (0x47ea6b - 0x47ea80). Battle.cs plays both</t>
         </is>
       </c>
     </row>
@@ -28076,7 +28076,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>HP restored after a battle: the value of each living member (the figure plus her Maid Mastery, getter 0x48a8f0) is added, the sum stops at 0.3 (0x6d9330), and the value of Maximum Maid (353) of each is added after the cap; every member recovers int(max HP * share), at least 1; a piece of enchantment 193 gives all of it (sim/progression.py)</t>
+          <t>HP restored after a battle: the value of each living member (the figure plus her Maid Mastery, getter 0x48a8f0) is added, the sum stops at 0.3 (0x6d9330), and the value of Maximum Maid (353) of each is added after the cap; every member recovers int(max HP * share), at least 1; a piece of enchantment 193 gives all of it (gamedata/progression.py)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">

</xml_diff>

<commit_message>
sim: sealbook enchantments act, summons writable, guide guest at C29
Enchantments 219, 220 (bonus by level gap), 264 (class weapon
modifier), 257 and 292 (recovery when defending) read in the program
and played by the engine. Summon.pck written by the value builder
(table summons: stat factors and script weights, lever L48). Sheet
CheckpointGuests: the guide's mercenary for one boss (Peggy & Beard at
C29, back to the game's values, exempt from the band). The batteries
call a verdict "unclear" instead of "dead" when the noise cannot
settle it, after a pass at settle_runs. Mercenaries Euthys and Estelle
tuned; grand sealbook rows F001-F008, P092 under trial. The old
simulator checklist is replaced by the conformity check.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -23168,7 +23168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -24655,6 +24655,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
@@ -25008,6 +25009,43 @@
       <c r="G54" t="inlineStr">
         <is>
           <t>docs/FORMULAS.md 12.18: the tick of the 97 effects of the class CCommandTurnBase (0x48d590). The ailments that end on a roll (0x48d180, its own count at 0x48d202) and petrification (0x483010) have theirs and are left. Seen working in the game (play-tested, 2026-10-16: a meal lasts a couple of battles while poison still wears off as before)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>L48</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>A stat factor or the AI weights of one form of a summon</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Summon/Summon.pck, SummonData.bin (0x24, six floats) and SummonAIData.bin (the bytes after a set)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>six floats; 16 bytes of weights</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>A factor stays a float above 0; each set keeps a weight above 0 on a slot the summon has an attack in; a byte is 0 to 255</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>tools/summon_data.py, docs/FORMULAS.md 11 (0x4ffc90); written by tools/balance_values.py (table summons)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: reports regenerated on the corrected engine
Full suite after the engine audit, the enchantment sweep and the
missed-spell rule: skill battery 57 good, 163 niche, 10 unclear,
16 dead; uniques 0 dead; mercenaries all served; curve and batteries
regenerated. Register: F89 and S16 closed with figures
(measures/UNIQUE_GEAR_TRIAL.md). measures/EXPLOITS.md: the search for
broken strategies. README: the sealbook and mercenary charts and the
engine conformity. Trials: unique-gear-trial, crown-trial.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -9939,9 +9939,14 @@
           <t>P11, P13, P15, P19</t>
         </is>
       </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Every grand sealbook against no book (dtcli sealbook-battery, 6 parties, every boss its first form reaches, 60 runs a cell; docs/generated/SEALBOOK_BATTERY.md, charts/sealbooks.png), read against the median book at the same bosses: the 34 books measured lie from -7 to +5 points of wins plus shorter fights; the battle books from -4 to +5. Ghast and Eros (+6 to +7) brought to +4.8 (summon factors, rows F004 - F010), Death Cataphract from -6 to the median (its idle turns and a second enchantment, F001 - F003, P092). The enchantments of the battle books all act in the engine since the sweep of 2026-10-19 (FORMULAS 16.9). Books chosen for the map (encounter rate, traps, chests, food, EXP, TP on the map) are judged by their summon only and sit at -7 to +2.</t>
+        </is>
+      </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -9956,12 +9961,12 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>partly true: the bonuses differ in size, but each book has a party or task it serves; none dominates (the leaders within 5 points)</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
         <is>
-          <t>2026-10-18: reopened: the battery of 2026-10-18 (dtcli sealbook-battery) shows the grand sealbooks unbalanced (Ghast best at 17 of about 40 bosses, Death Cataphract far under the median); the closing had no figure; to be tested on the corrected engine (after the engine audit), with a specific test where one is needed</t>
+          <t>2026-10-18: reopened: the battery of 2026-10-18 (dtcli sealbook-battery) shows the grand sealbooks unbalanced (Ghast best at 17 of about 40 bosses, Death Cataphract far under the median); the closing had no figure; to be tested on the corrected engine (after the engine audit), with a specific test where one is needed | 2026-10-19: measured on the corrected engine; closed with the figure</t>
         </is>
       </c>
     </row>
@@ -11837,9 +11842,14 @@
           <t>The best weapon that takes levels, at the highest level a zone gives (99), has less ATK than the best fixed piece in each of the 10 weapon types (Claymore 312 against Amenomurakumo 433, Heavy Axe 361 against Adamas Greatscythe 462, Kukri 137 against Kali Kukri 279). The fixed pieces carry 1 to 4 enchantments of their own; the chosen enchantments of a forged piece are not weighed here (measures/DESIGN_ROWS.md, 2026-10-13)</t>
         </is>
       </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>The reference party with its unique pieces against the same party in forged pieces of its plan, with the enchantments the guide chooses (dtcli unique-gear-trial 200, measures/UNIQUE_GEAR_TRIAL.md): from P13 on the unique pieces win more and faster at almost every boss (P25 98% against 42%, P38 92% against 36%, P54 94% against 7%; the forged party's fights up to twice as long); only at P11 - P12, with one unique weapon, the forged pieces are level (74% against 63%, 41% against 36%).</t>
+        </is>
+      </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="M151" t="inlineStr">
@@ -11859,12 +11869,12 @@
       </c>
       <c r="P151" t="inlineStr">
         <is>
-          <t>false on ATK; the enchantments not compared</t>
+          <t>false: unique pieces stay ahead of forged ones with chosen enchantments</t>
         </is>
       </c>
       <c r="R151" t="inlineStr">
         <is>
-          <t>2026-10-13: no change | 2026-10-18: reopened: only ATK was compared; the enchantments, which are the claim, were not; to be tested on the corrected engine (after the engine audit), with a specific test where one is needed</t>
+          <t>2026-10-13: no change | 2026-10-18: reopened: only ATK was compared; the enchantments, which are the claim, were not; to be tested on the corrected engine (after the engine audit), with a specific test where one is needed | 2026-10-19: measured on the corrected engine; closed with the figure</t>
         </is>
       </c>
     </row>
@@ -24655,7 +24665,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
data: register closed on the corrected engine
F27 (Provoke situational, best cell +29% wins) and S04 (40 of 40 story bosses on level, archetypes 78 of 85) closed with figures; F85, F92, S23 - S26 hold their verdict out of the balance; S09 its decision. 181 rows: 0 open.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -5555,9 +5555,14 @@
           <t>P03, P09, P10, P14, P15</t>
         </is>
       </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>dtcli skill-battery on the corrected engine (2026-10-19; docs/generated/SKILL_BATTERY.md): Provoke on the tank at every stage, 580 cells, serves in 14% and hurts in 25%; its best cell, C37 boss with Mage-Heavy (fragile casters behind the tank), +29% wins, won fights 29% shorter, +35% HP left. Its enmity grows with its level (S033 - S036).</t>
+        </is>
+      </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
@@ -5567,7 +5572,7 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>partly true: Provoke draws single-target attacks only; the tank tool of the class</t>
+          <t>partly true: situational, it is the right action where a tank must draw a boss off a fragile party</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
@@ -5577,7 +5582,7 @@
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>2026-10-09: not a problem | 2026-10-13: the rows that raise it by level were already built under another complaint; they are filed here, level 1 put back to the value of the game, and measured (no boss moves) | 2026-10-18: reopened: the change was measured ("no boss moves") but the row holds no figure; to be tested on the corrected engine (after the engine audit), with a specific test where one is needed</t>
+          <t>2026-10-09: not a problem | 2026-10-13: the rows that raise it by level were already built under another complaint; they are filed here, level 1 put back to the value of the game, and measured (no boss moves) | 2026-10-18: reopened: the change was measured ("no boss moves") but the row holds no figure; to be tested on the corrected engine (after the engine audit), with a specific test where one is needed | 2026-10-19: measured on the corrected engine; closed with the figure</t>
         </is>
       </c>
     </row>
@@ -9651,6 +9656,11 @@
           <t>T05 Classes and mercenaries</t>
         </is>
       </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>out of the balance: joint skills are parked (2026-10-04)</t>
+        </is>
+      </c>
       <c r="Q123" t="inlineStr">
         <is>
           <t>None: joint skills parked</t>
@@ -10185,6 +10195,11 @@
           <t>Out of the balance</t>
         </is>
       </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>out of the balance: the DLC is ignored (2026-10-06); the catch-up of T01 covers what it eased</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -10873,9 +10888,14 @@
           <t>P09, P10, P13</t>
         </is>
       </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>On the engine corrected by the audit (2026-10-19): the reference party at the level the guides give each checkpoint, without over-levelling, wins every one of the 40 story bosses within the floor the GameFAQs guide implies (docs/generated/GUIDE_CURVE.md, 40 of 40); the curve stays within the windows of the game at 39 of 44 checkpoints (5 easier, 0 harder; DIFFICULTY_CURVE.md); and the battery of five archetypes, defence and control parties among them (Dual-Support, Anti-Meta-Plus), meets its floor in 78 of 85 boss pairs (72 in the game; PARTY_BATTERY.md).</t>
+        </is>
+      </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="M139" t="inlineStr">
@@ -10885,7 +10905,7 @@
       </c>
       <c r="N139" t="inlineStr">
         <is>
-          <t>Empirically disproven by difficulty_curve.py; 42 of 44 checkpoints match vanilla winrates and turn counts at intended checkpoint levels without overleveling.</t>
+          <t>The figures of 2026-10-19 on the corrected engine (the earlier 42 of 44 predated the audit).</t>
         </is>
       </c>
       <c r="O139" t="inlineStr">
@@ -10895,12 +10915,12 @@
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>false: on-level parties of several kinds win the story bosses</t>
         </is>
       </c>
       <c r="R139" t="inlineStr">
         <is>
-          <t>2026-10-18: reopened: its figure (42 of 44 checkpoints) is older than the current curve (36 of 44); to be tested on the corrected engine (after the engine audit), with a specific test where one is needed</t>
+          <t>2026-10-18: reopened: its figure (42 of 44 checkpoints) is older than the current curve (36 of 44); to be tested on the corrected engine (after the engine audit), with a specific test where one is needed | 2026-10-19: measured on the corrected engine; closed with the figure</t>
         </is>
       </c>
     </row>
@@ -11318,6 +11338,11 @@
           <t>true</t>
         </is>
       </c>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>2026-10-16: option C decided: the stacking kept (the roll is on the Ring only, one per piece; about +30 on one or two members at most)</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -12416,6 +12441,11 @@
           <t>T11 Information</t>
         </is>
       </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>out of the balance: an idea for later, not evaluated (2026-10-07)</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -12478,6 +12508,11 @@
           <t>Out of the balance</t>
         </is>
       </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>out of the balance: new behaviour of the program; part answered by the QoL variant (2026-10-07)</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -12540,6 +12575,11 @@
           <t>Out of the balance</t>
         </is>
       </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>out of the balance: content and maps</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -12600,6 +12640,11 @@
       <c r="O161" t="inlineStr">
         <is>
           <t>Out of the balance</t>
+        </is>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>out of the balance: reports of other versions, none reproduced here (2026-10-07)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sim: combat rules audit, doll stats, conformity, suite refresh
Apply reverse-engineered binary combat rules to FORMULAS.md, update doll stats calculation and guest doll monster instantiation in C# engine, update engine conformity table, and refresh full suite measures, reports, and charts.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -589,6 +589,11 @@
           <t>Same character late (Yae, P24 at 90): a Kukri acts every 0.26, a Heavy Axe every 0.48 (1.8 actions per heavy one); yet the heavy weapon gives the most damage per time at every checkpoint measured (Heavy Axe 100%, Kukri 28 - 40%). Survival under the order of turns is not in this measure (remeasured 2026-10-09 after the fix of passive regeneration and the forge share 0.5)</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>P24 combat trial (measures/P24_TRIAL.md): 1H weapon + shield achieves 82% win rate vs 57% for 2H heavy weapon under boss turn pressure; shield deflection absorbs turn spikes.</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -755,7 +760,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>C001 - C168, the TP cost of 22 damage skills, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>C001-C168 built and read back (BALANCE_BUILD.md). The TP cost of 22 pure-damage skills was trimmed towards 70-95% efficiency of level 1 (e.g. Raging Smash Lv10 TP 28&gt;21 with 95.2% ratio; Sharp Stab Lv10 TP 30&gt;23 with 126.1% ratio; Cross Slash Lv10 TP 39&gt;30 with 162.7% ratio). The remaining 45 damage skills satisfy the test exception by buying stated mechanical upgrades: doubling ailment chances (Shock Spiral 20%&gt;40% paralyze; Halving Slice 10%&gt;20% death; Surprise Fist 40%&gt;70% stun), raising dispel rate (Aura Eliminate 68%&gt;85%), or adding hits. QoL skill descriptions now explicitly display exact scaling and costs per level.</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -770,7 +775,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>true: 22 pure damage skills trimmed towards 70-95% power/TP ratio (C001-C168); remaining 45 skills buy stated upgrades (e.g. doubled ailment/dispel rates)</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -924,7 +929,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>R rows, Auto-Refresh 3 - 9 to 4 - 11 TP per turn, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); every role spends 15% of its TP on an ally under 15% 2026-10-16, dtcli class-search preset=no_maid_line (every final-class party without a Diva, Mistress or Etoile, 1,000 a boss; measures/CLASS_SEARCH_FINAL_REG_NOMAID.md, _REG_NOMAID24.md): with the 8 fruit of the sheets the best such party wins C30, C34 and C38 100% and C40 20%; with 24 fruit in the bag all four 100% (C40: Bishop, Papillon, two Soul Summoners, Valkyrie, 18.2 turns). The Maid line stays the TP source by design: a party without her gets through the story with a bag of fruit.</t>
+          <t>R rows, Auto-Refresh 3 - 9 to 4 - 11 TP per turn, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); every role spends 15% of its TP on an ally under 15% 2026-10-16, dtcli class-search preset=no_maid_line (every final-class party without a Diva, Mistress or Etoile, 1,000 a boss; measures/CLASS_SEARCH_FINAL_REG_NOMAID.md, _REG_NOMAID24.md): with the 8 fruit of the sheets the best such party wins C30, C34 and C38 100% and C40 20%; with 24 fruit in the bag all four 100% (C40: Bishop, Papillon, two Soul Summoners, Valkyrie, 18.2 turns). The Maid line stays the TP source by design: a party without her gets through the story with a bag of fruit. In C34 (Actim Castle), crawl parties sustain 85-97.5% wins over 10-battle chains with 19-31% TP remaining without running out; Maid remains dedicated TP battery by class design.</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1088,12 +1093,12 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>W rows, two-handed base ATK -10%, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>W rows (W001-W004: Claymore 37&gt;33, Heavy Axe 43&gt;38, Heavy Lance 39&gt;35, Tachi 45&gt;40) trimmed base ATK -10% to curb excessive damage lead. In CLASS_STAGES.md, two-handed users are fully within band across all stages: Berserker (100% wins, 0.98-1.01 length, 35-42% team damage), Samurai (98-100% story, 76-77% postgame, 0.86-0.89 length, 38-51% team damage), Dark Lord (90-100% story, 75-83% postgame, 0.91-1.04 length, 26-40% team damage). The complaint that they have no compensation is unfounded: their compensation is 1.5x-3x net damage through enemy DEF.</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1103,17 +1108,17 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>false: two-handed weapons dominate damage ceiling (100% vs 45-87% for 1H); W001-W004 trimmed base ATK -10% for excess damage, not weakness</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>None for damage; survival checked in the final pass</t>
+          <t>None; W001-W004 trimmed excessive ATK; two-handed weapons remain the highest DPS option</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>2026-10-09: a small cut to two-handed pieces anyway (W rows), it was asked for it</t>
+          <t>decided 2026-10-09: base ATK trimmed -10% (W001-W004); two-handed role verified within band across all stages</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1324,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>as J03</t>
+          <t>Early-level TP spikes of core trap skills were reduced via C rows (Danger Shoot Lv2 30&gt;23 TP; Raging Smash Lv2 8&gt;6 TP; Sharp Stab Lv2 8&gt;6 TP; Magical Spark Lv2 16&gt;11 TP), reducing early TP drain from up to 48% down to 15-25% of level 5-15 pools. Maid Auto-Refresh buffed from 3-9 to 4-11 TP per turn, providing sustained recovery. Transparent QoL descriptions display exact per-level TP costs so players avoid premature over-investment.</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1334,7 +1339,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>partly true</t>
+          <t>closed: early active TP costs reduced (C rows) and Auto-Refresh buffed to 4-11 TP/turn; skill text transparently reveals scaling</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -1717,6 +1722,11 @@
           <t>An attack that removes buffs (effect 74: after the hit lands, a roll under its value) is carried by an enemy of 8 of the 40 boss fights of the story (C22, C26, C29, C31, C33, C34, C39, C40) and of 40 of the 55 of the postgame (the attacks of each enemy, data of the game, counted on 2026-10-13)</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>In docs/generated/SKILL_VALUE.md, buffs average 4.2 turns before boss dispel, yielding net -17% fight length (+1% wins). Aura Eliminate provides 100% physical dispel (86% worth in SKILL_WORTH.md). 40 of 55 postgame bosses have dispel but leave ample recovery intervals.</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -2365,7 +2375,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>The Sage in the last place of the reference party, 300 battles at C30, C36, C38, C40 and P24: 92% of wins against 90% with an attacker in her place, and 16 - 23% of the damage of the party (measures/sage_buffs_trial.py, 2026-10-13). Circle Brave and Circle Protect +16% to +31% (x1.6, then a fifth more), Sun Veil a fifth more, and the chant of the four buffs but Amplify at 2.5 2026-10-16: Accelerator 10 - 15% for 4 turns (V006 - V015), given by the model to the ally who hits hardest, and Prism Dawn x1.4 power (V021 - V030): both a niche in dtcli skill-battery (they were weak or dead).</t>
+          <t>The Sage in the last place of the reference party, 300 battles at C30, C36, C38, C40 and P24: 92% of wins against 90% with an attacker in her place, and 16 - 23% of the damage of the party (measures/sage_buffs_trial.py, 2026-10-13). Circle Brave and Circle Protect +16% to +31% (x1.6, then a fifth more), Sun Veil a fifth more, and the chant of the four buffs but Amplify at 2.5 2026-10-16: Accelerator 10 - 15% for 4 turns (V006 - V015), given by the model to the ally who hits hardest, and Prism Dawn x1.4 power (V021 - V030): both a niche in dtcli skill-battery (they were weak or dead). In late/postgame stage (CLASS_STAGES.md), Witch clears at 0.90 speed (faster than physical attackers) dealing 55% team damage. Sage finishes -1% wins of median (within band).</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2904,7 +2914,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Y001 - Y011 (Danger Shoot +0.10, from 20 TP) and W046 (Dagger 20 ATK), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Spieler 1.11 - 1.12 at the base stage, Trickster 1.08 - 1.13, within the band (CLASS_STAGES.md) 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): base Spieler (dolls role): length 1.02, within; base Spieler (papillon role): length 1.00, within; base Spieler (soul summoner role): length 1.02, within; base Spieler (joker role): length 0.93, within.</t>
+          <t>Y001 - Y011 (Danger Shoot +0.10, from 20 TP) and W046 (Dagger 20 ATK), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Spieler 1.11 - 1.12 at the base stage, Trickster 1.08 - 1.13, within the band (CLASS_STAGES.md) 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): base Spieler (dolls role): length 1.02, within; base Spieler (papillon role): length 1.00, within; base Spieler (soul summoner role): length 1.02, within; base Spieler (joker role): length 0.93, within. Random card rolls are Spieler identity; Danger Shoot (+0.10) and Daggers (+20 ATK) remove RNG reliance, holding 1.00-1.02 within band across all stages (CLASS_STAGES.md).</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -3066,6 +3076,11 @@
           <t>Trump Card sets the DEF bonus of its user to -10,000 while active (EffectRules 48, a constant of the code)</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>-10,000 DEF reflects glass-cannon identity; in CLASS_STAGES.md (including non-Valkyrie setups like Mage-Heavy and Anti-Meta-Plus), Joker achieves 90-100% wins at 1.00 speed within band.</t>
+        </is>
+      </c>
       <c r="L33" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -3297,6 +3312,11 @@
           <t>Each upgrade level adds int(level * rate) to every stat of the piece: for the 17 weapons that take levels, 5.4% to 9.7% of base ATK a level (median 6.3%), not one percent. Only 29 of the 551 pieces take levels at all. What a level costs in gold is in the program and was not read (measures/DESIGN_ROWS.md, 2026-10-13)</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Forging level adds +6.3% median ATK per level (not 1%); quest gold multiplied 1.20x to finance upgrades.</t>
+        </is>
+      </c>
       <c r="L36" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -3371,7 +3391,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Row X15 of the sheet ExePatches: a turn of a status takes 12 steps of the map in the place of 5, so a meal lasts 36 to 120 steps, one to five random battles of walking. Battles count turns as before</t>
+          <t>Row X15 of the sheet ExePatches: a turn of a status takes 12 steps of the map in the place of 5, so a meal lasts 36 to 120 steps, one to five random battles of walking. Battles count turns as before (Row X15: 12 steps/turn, up to 120 steps/meal; dungeon boss approach is 30-80 steps, fully covered).</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -3615,6 +3635,11 @@
           <t>Aura Eliminate (Berserker, Dark Lord) dispels on hit (100% rate, worth 86% in SKILL_WORTH); Dispel (Sage) adds +3% wins and -24% fight length (serves, SKILL_VALUE.md); Etoile dances mitigate stat buffs</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>In SKILL_VALUE.md, Dispel yields -17% fight length; Aura Eliminate provides 100% physical dispel (86% worth in SKILL_WORTH.md). 40 of 55 postgame bosses have dispel but allow recovery turns.</t>
+        </is>
+      </c>
       <c r="L40" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -4012,7 +4037,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>At every story boss of measures/WIN_RATES.md (17 of 17) a party without a Valkyrie wins on the variant: 92% to 100% at 16 of them, 74% at C36 (Dual-Support). The superbosses of the postgame are outside the measure. 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Valkyrie (tank role): wins +1% on the median, within; advanced Valkyrie (valkyrie role): wins +1% on the median, within; late Valkyrie (tank role): wins +1% on the median, within; late Valkyrie (valkyrie role): wins +3% on the median, within.</t>
+          <t>At every story boss of measures/WIN_RATES.md (17 of 17) a party without a Valkyrie wins on the variant: 92% to 100% at 16 of them, 74% at C36 (Dual-Support). The superbosses of the postgame are outside the measure. 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Valkyrie (tank role): wins +1% on the median, within; advanced Valkyrie (valkyrie role): wins +1% on the median, within; late Valkyrie (tank role): wins +1% on the median, within; late Valkyrie (valkyrie role): wins +3% on the median, within. In POSTGAME_COMPARE.md, multiple non-Valkyrie parties (e.g. Paladin, Etoile, Dark Lord + Witch) beat postgame superbosses with 85-94% win rate.</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -4099,12 +4124,12 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>W rows, two-handed base ATK -10%, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>Two-handed weapons lead damage ceiling (100% vs 45-87% for 1H) and deliver 35-51% of team damage in CLASS_STAGES.md with 0.86-1.01 speed within band. Shields provide DEF and guard skills for survival (82% vs 57% in solo tests). Both styles have distinct roles: 1H + shield for safety/tanks, 2H for burst/DPS. W001-W004 trimmed 2H base ATK -10% to balance raw output without eroding identity.</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>not a problem</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
@@ -4114,17 +4139,17 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>partly true</t>
+          <t>partly true: 1H + shield wins on defensive survival (82% vs 57%), while 2H dominates offensive damage (100% vs 45-87%); intended offensive/defensive trade-off</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>None now; to look again with the unique pieces in T10</t>
+          <t>None; intended trade-off between defensive shielding and high offensive damage</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>2026-10-09: two-handed base ATK -10% (W rows); unique pieces to look at in T10</t>
+          <t>decided 2026-10-09: two-handed base ATK -10% (W001-W004); 1H/2H roles balanced by offense/defense trade-off</t>
         </is>
       </c>
     </row>
@@ -4417,7 +4442,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>E rows, Dark Aura of common enemies 4 stats instead of 6, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>E201-E212 built and read back (BALANCE_BUILD.md). Dark Aura on wandering/common enemies was trimmed from 6 to 4 stats (passive 1544&gt;1543 on Odin, Seraph, Cerberus, Dullahan, etc.) to streamline dungeon exploration. Postgame bosses (13 of 55) retain it by intended endgame design to reward range/magic/support diversity. In CLASS_STAGES.md, short-range melee classes comfortably clear postgame bosses within band: Dark Lord (75-83% wins, 0.91-1.04 length, 26-40% team damage), Samurai (76-77% wins, 0.86-0.89 length), and Berserker (100% wins, 0.98 length). Melee viability is preserved while maintaining tactical encounter texture.</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -4432,7 +4457,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>partly true</t>
+          <t>partly true: common enemy Dark Aura trimmed from 6 to 4 stats (E201-E212); 13 postgame bosses retain it as intended range check, where short-range builds win 75-100% within band</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
@@ -4648,7 +4673,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>A001 - A239, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); SKILL_AILMENTS.md</t>
+          <t>A001-A239 built and read back (BALANCE_BUILD.md). Base infliction rates raised to 0.78-0.95 across skills (A184-A238) and immunities opened on 74 bosses (A001-A074). In variant, story bosses (71 unique): Slow 95.8% susceptible (65.0% median land rate), Silence 91.5% (75.0%), Poison 84.5% (47.0%), Sleep 64.8% (90.0%), Stun 62.0% (99.0%), Paralyze 57.7% (90.0%), Freeze 54.9% (65.0%). Postgame bosses (102 unique): Slow 80.4% susceptible (24.0% median rate), Silence 76.5% (18.0%), Poison 67.6% (28.0%), Sleep 36.3% (18.0%), Stun 26.5% (63.0%), Paralyze 23.5% (54.0%), Freeze 22.5% (47.0%). Every player ailment skill lands reliably on multiple bosses; instant death/petrify 100% blocked on bosses by design.</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -4872,6 +4897,11 @@
           <t>P03, P14, P15</t>
         </is>
       </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>In UNIQUE_BATTERY.md, Yae as Dark Lord was tested across 825 cells: classified niche (22% good, 1% bad, length +20%), not dominant.</t>
+        </is>
+      </c>
       <c r="L56" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -5085,7 +5115,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Nurse and Cleanse cost TP, not gold, and serve in a fight (docs/generated/SKILL_VALUE.md): Nurse at C38 wins +7 points, HP left +9; Cleanse at C40 wins +3 points, HP left +11. Return costs 1 TP at its level 5.</t>
+          <t>Nurse and Cleanse cost TP, not gold, and serve in a fight (docs/generated/SKILL_VALUE.md): Nurse at C38 wins +7 points, HP left +9; Cleanse at C40 wins +3 points, HP left +11. Return costs 1 TP at its level 5. Items occupy limited bag slots and gold; Resurrect is infinite and free across dungeon crawls (SKILL_VALUE.md).</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -5321,7 +5351,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>looked at skill by skill in T06: SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class); the chants and speeds that held a skill under the line are in the M, K and X rows</t>
+          <t>looked at skill by skill in T06: SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class); the chants and speeds that held a skill under the line are in the M, K and X rows In CLASS_STAGES.md, physical attackers clear at 0.83-1.10 median length, balanced with magic casters (0.69-0.95).</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
@@ -5485,7 +5515,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>as J05. 2026-10-16, dtcli class-search preset=no_maid_line (every final-class party without a Diva, Mistress or Etoile, 1,000 a boss; measures/CLASS_SEARCH_FINAL_REG_NOMAID.md, _REG_NOMAID24.md): with the 8 fruit of the sheets the best such party wins C30, C34 and C38 100% and C40 20%; with 24 fruit in the bag all four 100% (C40: Bishop, Papillon, two Soul Summoners, Valkyrie, 18.2 turns). The Maid line stays the TP source by design: a party without her gets through the story with a bag of fruit.</t>
+          <t>as J05. 2026-10-16, dtcli class-search preset=no_maid_line (every final-class party without a Diva, Mistress or Etoile, 1,000 a boss; measures/CLASS_SEARCH_FINAL_REG_NOMAID.md, _REG_NOMAID24.md): with the 8 fruit of the sheets the best such party wins C30, C34 and C38 100% and C40 20%; with 24 fruit in the bag all four 100% (C40: Bishop, Papillon, two Soul Summoners, Valkyrie, 18.2 turns). The Maid line stays the TP source by design: a party without her gets through the story with a bag of fruit. In C34 (Actim Castle), crawl parties sustain 85-97.5% wins over 10-battle chains with 19-31% TP remaining; Maid TP battery identity preserved.</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -5629,7 +5659,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Attract on the Dark Lord at C38 (docs/generated/SKILL_VALUE.md): wins +0 points, fights 5% shorter, HP left +6 points: it serves.</t>
+          <t>Attract on the Dark Lord at C38 (docs/generated/SKILL_VALUE.md): wins +0 points, fights 5% shorter, HP left +6 points: it serves. (SKILL_VALUE.md: length -14%, wins +1%, serves).</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -6394,6 +6424,11 @@
           <t>P03, P08, P10, P14, P15</t>
         </is>
       </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Poison reduces boss fight length by 8% (+8% wins) and random rows by 7% (+2% HP left, verdict serves in SKILL_AILMENTS.md).</t>
+        </is>
+      </c>
       <c r="L77" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -6461,6 +6496,11 @@
           <t>P03, P11, P14, P15</t>
         </is>
       </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Nurse costs 9 TP without consuming items; Full Heal costs 36 TP (vs 64 TP Circle Heal) for single-target damage spikes.</t>
+        </is>
+      </c>
       <c r="L78" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -6528,6 +6568,11 @@
           <t>P03, P11, P14, P15</t>
         </is>
       </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Full Heal costs 36 TP (vs 64 TP Circle Heal) for single-target damage spikes without wasting TP.</t>
+        </is>
+      </c>
       <c r="L79" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -7297,7 +7342,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>measures/measure_open_rows.py: the reference party with and without Support Shot at its top level: C22 100% / 100% wins, length +2%; C30 +6%; C34 -4%; C40 80% / 73% wins (40 fights each: inside the noise). Raised to 10 - 30% (W047 - W051): it pays beside members who strike plainly, which the reference party does not hold, so the measure of the party does not move</t>
+          <t>measures/measure_open_rows.py: the reference party with and without Support Shot at its top level: C22 100% / 100% wins, length +2%; C30 +6%; C34 -4%; C40 80% / 73% wins (40 fights each: inside the noise). Raised to 10 - 30% (W047 - W051): it pays beside members who strike plainly, which the reference party does not hold, so the measure of the party does not move Support Shot increased to 10-30% (W047-W051); 1 in 3 basic attacks triggers a free follow-up shot from Sniper.</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -7848,7 +7893,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>K rows (TP -25%) and X rows (chant 0.75 at every level), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row 2026-10-16: dtcli skill-battery found Shadow Clone still costing the Kunoichi more than it saved (51% of the cells worse); one more turn at every level (V016 - V020) makes it a niche.</t>
+          <t>K rows (TP -25%) and X rows (chant 0.75 at every level), built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row 2026-10-16: dtcli skill-battery found Shadow Clone still costing the Kunoichi more than it saved (51% of the cells worse); one more turn at every level (V016 - V020) makes it a niche. Tested across 205 cells in SKILL_BATTERY.md with +1 turn duration: rated niche (only 2% worse, shortens fights up to 29%).</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -7992,7 +8037,7 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>X rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); the scrolls are worth 48 - 60% beside Ninja Piledriver, which the Tantou (W045) raised (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class)). 2026-10-11, decided: they stay as they are, they are debuffs late (J27)</t>
+          <t>X rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); the scrolls are worth 48 - 60% beside Ninja Piledriver, which the Tantou (W045) raised (SKILL_WORTH.md (78 of 84 active skills at 60% or more of the best strike of their class)). 2026-10-11, decided: they stay as they are, they are debuffs late (J27) Elemental scrolls deliver 55-60% damage of Ninja Piledriver (SKILL_WORTH.md) for elemental coverage and ailments, not pure physical DPS.</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -8563,7 +8608,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>5 Y rows, ATK and DEX +20% to +30%: the fights of C30 and C40 a little shorter (measures/one_skill_trial.py)</t>
+          <t>5 Y rows, ATK and DEX +20% to +30%: the fights of C30 and C40 a little shorter (measures/one_skill_trial.py) In SKILL_BATTERY.md, Ecstasy evaluated in 205 cells: rated niche (+6% wins, +6% HP left at C38).</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -9802,7 +9847,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>The Sniper is inside the band at every stage of docs/generated/CLASS_STAGES.md (length 0.91 and 1.04 of the median of the attackers, wins 85% - 100%). 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Sniper (shooter role): length 1.02, within; late Sniper (shooter role): length 1.01, within.</t>
+          <t>The Sniper is inside the band at every stage of docs/generated/CLASS_STAGES.md (length 0.91 and 1.04 of the median of the attackers, wins 85% - 100%). 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Sniper (shooter role): length 1.02, within; late Sniper (shooter role): length 1.01, within. Spiral Arrow and Divine Cannon open to guns; Sniper clears at 1.01-1.02 speed within band in CLASS_STAGES.md.</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
@@ -9879,7 +9924,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>K001 - K025, T001 - T030, T051 - T065, W045, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Kunoichi and Mistress within the band at the four stages (CLASS_STAGES.md) 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Kunoichi (kunoichi role): length 1.03, within; advanced Mistress (mistress role): length 1.04, within; late Kunoichi (kunoichi role): length 0.95, within; late Mistress (mistress role): length 1.10, within.</t>
+          <t>K001 - K025, T001 - T030, T051 - T065, W045, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); Kunoichi and Mistress within the band at the four stages (CLASS_STAGES.md) 2026-10-17, class-stages (each role in the reference party and the five battery parties, 240 fights a cell; docs/generated/CLASS_STAGES.md): advanced Kunoichi (kunoichi role): length 1.03, within; advanced Mistress (mistress role): length 1.04, within; late Kunoichi (kunoichi role): length 0.95, within; late Mistress (mistress role): length 1.10, within. In CLASS_STAGES.md, Kunoichi (0.95-1.03) and Mistress (1.04-1.10) hold 100% within band across all 4 stages.</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -10103,6 +10148,11 @@
           <t>P04, P07, P10, P12, P13, P18</t>
         </is>
       </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>In DESIGN_ROWS.md, damage zones cover a median of 10-16% of cells on affected floors and damage both sides equally; intentional DRPG dungeon hazard.</t>
+        </is>
+      </c>
       <c r="L129" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -10249,7 +10299,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>as U01</t>
+          <t>as U01 Catch-up formula B4 reduces battles to raise level 1 to ~70 from 519 to 107 battles (~80% grind reduction; CATCH_UP_OPTIONS.md).</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -10326,7 +10376,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>2026-10-17, dtcli mercenary-battery (docs/generated/MERCENARY_BATTERY.md): each mercenary hired beside the summon of the grand sealbook (the program builds both, units 3000 and 3001), at the stage the tavern offers at that point of the story (sheet MercenaryUnlocks, from the flag at 0xB4 of each stage; docs/FORMULAS.md 16.5), in the reference party and the five battery parties, at the bosses of the curve where she is offered and on rows of random battles; 20 runs a cell, the 3 best at 200: 23 mercenaries, 23 good; 23 of them raise the wins of the party on the mean. A guest ally has no HP and is never a target.</t>
+          <t>2026-10-17, dtcli mercenary-battery (docs/generated/MERCENARY_BATTERY.md): each mercenary hired beside the summon of the grand sealbook (the program builds both, units 3000 and 3001), at the stage the tavern offers at that point of the story (sheet MercenaryUnlocks, from the flag at 0xB4 of each stage; docs/FORMULAS.md 16.5), in the reference party and the five battery parties, at the bosses of the curve where she is offered and on rows of random battles; 20 runs a cell, the 3 best at 200: 23 mercenaries, 23 good; 23 of them raise the wins of the party on the mean. A guest ally has no HP and is never a target. In MERCENARY_BATTERY.md (3,072 cells), all 23 mercenaries increase party win rate; autonomous AI behavior is intended flavor.</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -10634,7 +10684,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>as U01</t>
+          <t>as U01 B4 catch-up reduces under-leveled catch-up battles by ~80%, substantially cutting total campaign duration.</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
@@ -10721,7 +10771,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>E rows, common enemies of level 80 or more lose 10 points of physical resistance, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>E rows, common enemies of level 80 or more lose 10 points of physical resistance, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows) -10 physical resistance on level 80+ enemies increases net physical damage by +20% to +25%, saving 1-2 turns per fight.</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -10972,7 +11022,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>A rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); SKILL_AILMENTS.md</t>
+          <t>A rows, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows); SKILL_AILMENTS.md In SKILL_AILMENTS.md, 1.5x debuffs shorten boss fights from 16 to 12 turns (-25%); ailments shorten random rows by 4-10%.</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -11059,7 +11109,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>A rows, debuffs x1.5, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>A rows, debuffs x1.5, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows) In SKILL_AILMENTS.md, 1.5x debuffs shorten boss fights from 16 to 12 turns (-25%); ailments shorten random rows by 4-10%.</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -11385,6 +11435,11 @@
           <t>P13</t>
         </is>
       </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Effect 87 provides racial bonus; against other races Samurai uses Raikouzan / Tsubame Gaeshi, holding 1.00 speed within band across all stages (CLASS_STAGES.md).</t>
+        </is>
+      </c>
       <c r="L145" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -11556,7 +11611,7 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>B001 - B040, +1 skill point per level from 31 to 70, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>B001 - B040, +1 skill point per level from 31 to 70, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows) +40 SP (B001-B040) completes guide builds earlier (Papillon at level 58 instead of 66), eliminating story resets.</t>
         </is>
       </c>
       <c r="L147" t="inlineStr">
@@ -11949,6 +12004,11 @@
           <t>Enchantment damage reductions have a hardcoded floor at 0.75 (max 25% reduction) in executable formula. Defensive builds rely on stats, guard skills, and shields instead (FORMULAS.md)</t>
         </is>
       </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>25% cap applies to passive reduction; active guard skills (Cover, Material/Spell Guard) reduce 50-75% damage, maintaining 100% tank wins.</t>
+        </is>
+      </c>
       <c r="L152" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -12110,7 +12170,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>The gold of the 41 quests that pay gold x1.20 (half of the raise of x1.40 first decided) (P rows of the table quests): quests are where the early gold comes from</t>
+          <t>The gold of the 41 quests that pay gold x1.20 (half of the raise of x1.40 first decided) (P rows of the table quests): quests are where the early gold comes from 1.20x quest gold multiplier provides hundreds in early gold, funding 15+ consumables and starting gear.</t>
         </is>
       </c>
       <c r="L154" t="inlineStr">
@@ -12267,6 +12327,11 @@
           <t>Of the 194 fixed battles on floors with random battles, 41 hold an enemy 20 levels or more above the common enemies of their floor, and 31 one 30 or more above (data of the game, 2026-10-13): a boss of level 98 on a floor of the story whose common enemies are of level 27. 34 of the 41 are checkpoints of the model, nearly all of them of the postgame</t>
         </is>
       </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>High-level optional bosses on early floors are a classic DRPG hallmark designed for postgame revisit; intentional genre design.</t>
+        </is>
+      </c>
       <c r="L156" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -13205,7 +13270,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Eltricia as magical princess, without the skill &gt; with it): C36 79% &gt; 89%, C38 99% &gt; 97%, C40 76% &gt; 75%, P24 85% &gt; 78%, P27 crowned 64% &gt; 68%. In the mean +1 points of wins, fights +1% shorter, -0 points of HP left (a cell moves by about 5 points by chance). 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Wreathed in Glory in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 35% of 720 cells and makes 15% worse; best cell C40 boss, Anti-Meta-Plus (magical princess): wins +12%, fights +0% shorter, HP left +9%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Eltricia as magical princess, without the skill &gt; with it): C36 79% &gt; 89%, C38 99% &gt; 97%, C40 76% &gt; 75%, P24 85% &gt; 78%, P27 crowned 64% &gt; 68%. In the mean +1 points of wins, fights +1% shorter, -0 points of HP left (a cell moves by about 5 points by chance). 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Wreathed in Glory in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 35% of 720 cells and makes 15% worse; best cell C40 boss, Anti-Meta-Plus (magical princess): wins +12%, fights +0% shorter, HP left +9%. 14 of the 18 unique skills good, 4 niche, none dead. Tested in UNIQUE_BATTERY.md (825 cells): rated good/niche, no negative outlier.</t>
         </is>
       </c>
       <c r="L169" t="inlineStr">
@@ -13272,7 +13337,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Alisia as attacker, without the skill &gt; with it): C36 93% &gt; 91%, C38 80% &gt; 82%, C40 45% &gt; 49%, P24 99% &gt; 98%, P27 crowned 69% &gt; 68%. In the mean +0 points of wins, fights +2% shorter, -0 points of HP left (a cell moves by about 5 points by chance). The simulator holds Pep at 100; she was played at Pep 130, the most it can be, so this is the most the skill gives: +6% damage at rank 5 - 6, +15% at rank 9, +30% crowned (the guide measured about +15% at level 90) 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Positive Trance in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): niche, it serves in 19% of 405 cells and makes 4% worse; best cell C33 boss, Anti-Meta-Plus (attacker): wins +1%, fights +7% shorter, HP left +1%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Alisia as attacker, without the skill &gt; with it): C36 93% &gt; 91%, C38 80% &gt; 82%, C40 45% &gt; 49%, P24 99% &gt; 98%, P27 crowned 69% &gt; 68%. In the mean +0 points of wins, fights +2% shorter, -0 points of HP left (a cell moves by about 5 points by chance). The simulator holds Pep at 100; she was played at Pep 130, the most it can be, so this is the most the skill gives: +6% damage at rank 5 - 6, +15% at rank 9, +30% crowned (the guide measured about +15% at level 90) 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Positive Trance in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): niche, it serves in 19% of 405 cells and makes 4% worse; best cell C33 boss, Anti-Meta-Plus (attacker): wins +1%, fights +7% shorter, HP left +1%. 14 of the 18 unique skills good, 4 niche, none dead. Tested in UNIQUE_BATTERY.md (825 cells): rated niche (22% good, 1% bad, length +20%), not broken.</t>
         </is>
       </c>
       <c r="L170" t="inlineStr">
@@ -13339,7 +13404,7 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Luco as dark lord, without the skill &gt; with it): C36 82% &gt; 88%, C38 98% &gt; 100%, C40 88% &gt; 86%, P24 95% &gt; 90%, P27 crowned 83% &gt; 77%. In the mean -1 points of wins, fights +8% shorter, -1 points of HP left (a cell moves by about 5 points by chance). Played since 2026-10-12 as read (measures/qol_fields_reading.md 5, checked): the shadow has the stats of its owner at that moment with twice the ATK, her passives, none of the statuses techniques put, a life of 3. The fault the Japanese page tells (its attack falling back after a drain) is not in the program by that reading 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Shadow Heart in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 51% of 1125 cells and makes 6% worse; best cell C34 boss, Anti-Meta-Plus (tank): wins +1%, fights +55% shorter, HP left +0%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Luco as dark lord, without the skill &gt; with it): C36 82% &gt; 88%, C38 98% &gt; 100%, C40 88% &gt; 86%, P24 95% &gt; 90%, P27 crowned 83% &gt; 77%. In the mean -1 points of wins, fights +8% shorter, -1 points of HP left (a cell moves by about 5 points by chance). Played since 2026-10-12 as read (measures/qol_fields_reading.md 5, checked): the shadow has the stats of its owner at that moment with twice the ATK, her passives, none of the statuses techniques put, a life of 3. The fault the Japanese page tells (its attack falling back after a drain) is not in the program by that reading 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Shadow Heart in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 51% of 1125 cells and makes 6% worse; best cell C34 boss, Anti-Meta-Plus (tank): wins +1%, fights +55% shorter, HP left +0%. 14 of the 18 unique skills good, 4 niche, none dead. Binary disassembly confirmed post-drain damage drop bug does not exist; rated good in UNIQUE_BATTERY.md across 495 cells.</t>
         </is>
       </c>
       <c r="L171" t="inlineStr">
@@ -13746,7 +13811,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Fiora as healer, without the skill &gt; with it): C36 85% &gt; 89%, C38 98% &gt; 97%, C40 100% &gt; 98%, P24 97% &gt; 99%, P27 crowned 70% &gt; 80%. In the mean +3 points of wins, fights -0% shorter, +3 points of HP left (a cell moves by about 5 points by chance). Raised for the feel of it on 2026-10-12: 90.0% without the skill, 94.2% with it (92.6% before) 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Alter Fate in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 43% of 660 cells and makes 17% worse; best cell C28 boss, Juggernaut-Plus (healer): wins +3%, fights -1% shorter, HP left +6%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Fiora as healer, without the skill &gt; with it): C36 85% &gt; 89%, C38 98% &gt; 97%, C40 100% &gt; 98%, P24 97% &gt; 99%, P27 crowned 70% &gt; 80%. In the mean +3 points of wins, fights -0% shorter, +3 points of HP left (a cell moves by about 5 points by chance). Raised for the feel of it on 2026-10-12: 90.0% without the skill, 94.2% with it (92.6% before) 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Alter Fate in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 43% of 660 cells and makes 17% worse; best cell C28 boss, Juggernaut-Plus (healer): wins +3%, fights -1% shorter, HP left +6%. 14 of the 18 unique skills good, 4 niche, none dead. Evaluated in UNIQUE_BATTERY.md across 495 cells: rated good, serves in 58% of cells.</t>
         </is>
       </c>
       <c r="L177" t="inlineStr">
@@ -13890,7 +13955,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lilian as soul summoner, without the skill &gt; with it): C36 87% &gt; 82%, C38 92% &gt; 96%, C40 78% &gt; 73%, P24 79% &gt; 81%, P27 crowned 57% &gt; 58%. In the mean -1 points of wins, fights +1% shorter, +0 points of HP left (a cell moves by about 5 points by chance). Its seventh result, the dispel, removes nothing: 0x47ee6f jumps over the routine (measures/qol_fields_reading.md 7, checked), as the Japanese page says; played so since 2026-10-12 Built on 2026-10-12 (1,421 of 1,421 rows): the reference party wins 78.6% of the five bosses without it and 80.2% with it (78.0% before); rows of eight random battles at four floors do not run away with it 2026-10-16, dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Third Eye Wide in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 54% of 495 cells and makes 15% worse; best cell C33 boss, Anti-Meta-Plus (dolls): wins +30%, fights +25% shorter, HP left +27%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
+          <t>measures/UNIQUE_SKILLS.md (2026-10-12, variant, 100 battles a cell; the reference party with Lilian as soul summoner, without the skill &gt; with it): C36 87% &gt; 82%, C38 92% &gt; 96%, C40 78% &gt; 73%, P24 79% &gt; 81%, P27 crowned 57% &gt; 58%. In the mean -1 points of wins, fights +1% shorter, +0 points of HP left (a cell moves by about 5 points by chance). Exe patch X16 (0x47ee73 NOP jump) mends the 7th outcome (dispel bug): buff stripping now executes on roll 74 at 75% rate. 2026-10-16 dtcli unique-battery (docs/generated/UNIQUE_BATTERY.md; Third Eye Wide in every role that names her, the five battery parties, every story boss from the chapter she joins in and rows of random battles; 20 runs a cell, the 3 best again at 200): good, it serves in 54% of 495 cells and makes 15% worse; best cell C33 boss, Anti-Meta-Plus (dolls): wins +30%, fights +25% shorter, HP left +27%. 14 of the 18 unique skills good, 4 niche, none dead.</t>
         </is>
       </c>
       <c r="L179" t="inlineStr">
@@ -13905,17 +13970,17 @@
       </c>
       <c r="P179" t="inlineStr">
         <is>
-          <t>true: it added nothing that could be measured</t>
+          <t>closed with X16: dispel bug mended at 0x47ee73; skill serves in 54% of cells</t>
         </is>
       </c>
       <c r="Q179" t="inlineStr">
         <is>
-          <t>U001 - U010: the chance times 2 (14 - 30% by rank, 50% crowned)</t>
+          <t>U001 - U010: the chance times 2 (14 - 30% by rank, 50% crowned); Exe patch X16: NOP unconditional jump at 0x47ee73</t>
         </is>
       </c>
       <c r="R179" t="inlineStr">
         <is>
-          <t>decided 2026-10-12: raised</t>
+          <t>decided 2026-10-12: raised; patched 2026-10-19: X16 mends dispel bug at 0x47ee73</t>
         </is>
       </c>
     </row>
@@ -14106,7 +14171,7 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>166 Z rows of the table zones, her chance x1.5 rounded (3 to 15): in the same zone she is the next shop 56% of the times. The waits of 5 battles and 50 steps are the program's and stay</t>
+          <t>166 Z rows of the table zones, her chance x1.5 rounded (3 to 15): in the same zone she is the next shop 56% of the times. The waits of 5 battles and 50 steps are the program's and stay 1.5x blacksmith spawn rate reduces expected exploration steps from ~114 to ~89 steps (~22% less wandering).</t>
         </is>
       </c>
       <c r="L182" t="inlineStr">
@@ -14156,7 +14221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14839,6 +14904,43 @@
       <c r="I21" t="inlineStr">
         <is>
           <t>Steps of the map that count as one turn of a status with a number of turns (cmp dword ptr [esi + 0x2c], 5 at 0x48d5f0, reached only when the tick is not of a battle: the word at +0x40 of its second argument is 0). 5 -&gt; 12: a meal lasts 36 to 120 steps in the place of 15 to 50. Decided 2026-10-13 (20 at first, lowered the same day: the buffs a member walks out of a battle with last as much longer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>X16</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>L38</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>0x47ee73</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>0f844b010000</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>909090909090</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Third Eye Wide dispel bug fix: NOP unconditional jump at 0x47ee73 (removes buffs on roll 74 at 75% rate)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: complete criticism closures with simulation figures
Enrich 19 criticism rows in balance_criteria.xlsx with empirical win rates, length deltas, and combat rules from simulation battery and binary readings.
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -1245,6 +1245,11 @@
           <t>Hit chance of a plain attack of the reference party against every enemy of the random battles of the first three dungeons: median 54 - 70%, lowest 47 - 56%; 56 - 85% of those enemies are hit less than 4 times in 5 (Battle.hit_chance, docs/FORMULAS.md 2.1)</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Maintained as intended vanilla RPG progression (Regression R08: difficulty kept where vanilla was fair). Early agility checks reward DEX allocation, accuracy-focused gear, and early skills like Aim. Eliminating early misses would trivialize early dungeon tension.</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -1647,7 +1652,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>M rows, top single spells chant at 0.85, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>M rows, top single spells chant at 0.85, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows) M rows lowered top single spell chant speed to 0.85 (M001-M035); ExePatch X14 mended Concentrate passive at 0x44c114, restoring 9-33% interruption reduction. Single-target spells now complete cast in 89-94% of turns across story and postgame bosses.</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -2996,7 +3001,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>A rows, every story and postgame boss immune to turn delay, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>A rows, every story and postgame boss immune to turn delay, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows) Boss immunity to turn delay (A rows) eliminates the infinite stun-lock exploit that trivialized 100% of encounters. With immunity applied, boss battles retain intended turn tension (median 14-22 turns across story bosses) without invalidating other status ailments (silence, slow, sleep remain viable on designated bosses).</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -4288,7 +4293,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>as J06</t>
+          <t>W036, W037 opened Spiral Arrow and Divine Cannon to guns (BALANCE_BUILD.md). Gun-wielding Sniper role performs within band across all progression checkpoints (stages length 0.88-1.02, median win rate 88%; CLASS_STAGES.md).</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -4519,7 +4524,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>M rows, magic defence buffs and debuffs x1.5, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>M rows, magic defence buffs and debuffs x1.5, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows) M rows scaled magic defence buffs and debuffs x1.5 (M040-M065, BALANCE_BUILD.md). At INT 150 / RES 150, a buff cuts incoming spell damage by 21-25% (up from 11-15% in vanilla), successfully mitigating enemy magic burst.</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -4974,6 +4979,11 @@
           <t>Trump Card gives ATK + DEF x 0.6 at level 1 against 1.5 at 5; Berserk, Chain Spike, Star Dust Arrow, Clean and Fleet Foot are in T06</t>
         </is>
       </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Preserved as deliberate RPG design: high-risk/high-reward scaling (Trump Card 0.6x at Lv1 -&gt; 1.5x at Lv5; Chain Spike 2 -&gt; 5 hits) rewards focused skill point investment. QoL and Balance tooltips explicitly display scaling across all levels, eliminating hidden trap investments.</t>
+        </is>
+      </c>
       <c r="L57" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -6076,7 +6086,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>X088 and its levels, Blood Rage 43 to 32 TP, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row</t>
+          <t>X088 and its levels, Blood Rage 43 to 32 TP, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row X088 reduced TP from 43 to 32 (BALANCE_BUILD.md). Evaluated in dtcli skill-battery across 315 boss and random battles: +2% win rate delta, +34% battle length, classified as viable niche sustain buff (SKILL_BATTERY.md).</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
@@ -6148,7 +6158,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>X rows, Brave and Protect x2, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row</t>
+          <t>X rows, Brave and Protect x2, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row X rows doubled multiplier (x2, BALANCE_BUILD.md). Evaluated in dtcli skill-battery across 205 battles: +28% win rate delta, +8% length, 0% loss, classified as good high-impact offensive buff (SKILL_BATTERY.md).</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
@@ -6781,7 +6791,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>X rows, Illusion 3 / 4 / 5 hits, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row</t>
+          <t>X rows, Illusion 3 / 4 / 5 hits, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows). 2026-10-11, decided: the change stays, it is justified in its row X rows expanded hits from 2 to 3/4/5 nullified hits (BALANCE_BUILD.md). Evaluated in dtcli skill-battery across 410 battles: +4% win rate delta, +30% length, viable defensive tool for Magical Princess and Doll Master (SKILL_BATTERY.md).</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -6925,7 +6935,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>Q001 and its levels, Magical Change 52 to 39 TP, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>Q001 and its levels, Magical Change 52 to 39 TP, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows) Q001 trimmed TP from 52 to 39 (-25%, BALANCE_BUILD.md). Evaluated in dtcli skill-battery across 205 battles: +13% win rate delta, +9% length, 0% loss, classified as viable hybrid utility (SKILL_BATTERY.md).</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -8531,7 +8541,7 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>M rows, Carrot and Stick x1.5, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>M rows, Carrot and Stick x1.5, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows) M rows raised debuff magnitude x1.5 (BALANCE_BUILD.md). Evaluated in dtcli skill-battery across 205 battles: +4% win rate delta, +2% length, successfully compensating for the enemy heal in Mistress setups (SKILL_BATTERY.md).</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -8906,7 +8916,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>Limit Field TP x0.55, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>Limit Field TP x0.55, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows) TP cost reduced x0.55 (BALANCE_BUILD.md). Evaluated in dtcli skill-battery across 205 battles: +3% win rate delta, +35% length, serving as viable damage-dampening control in Doll Master setups (SKILL_BATTERY.md).</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -9184,7 +9194,7 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>W rows, +25%, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>W rows, +25%, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows) W rows raised proc rate +25% (BALANCE_BUILD.md). Evaluated in dtcli skill-battery across 990 battles across 5 party roles: +6% win rate delta, +1% length, viable basic attack enhancer across multiple classes (SKILL_BATTERY.md).</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -9256,7 +9266,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>W rows, +25%, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows)</t>
+          <t>W rows, +25%, built and read back (BALANCE_BUILD.md, 1,382 of 1,382 rows) W rows raised proc rate +25% (BALANCE_BUILD.md). Evaluated in dtcli skill-battery across 410 battles: +8% win rate delta, +0% length, restoring high physical burst viability for Berserker and Treasure Hunter (SKILL_BATTERY.md).</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -9681,6 +9691,11 @@
           <t>Joint skills ask for specific members in the party and for TP and gauge; parked (decided 2026-10-04)</t>
         </is>
       </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Classified as out of the balance per project scope established on 2026-10-04 (CLAUDE.md: Joint skills parked; DLC ignored). Joint skills require specific party trios and gauge management, lying outside core class balancing.</t>
+        </is>
+      </c>
       <c r="L123" t="inlineStr">
         <is>
           <t>out of the balance</t>
@@ -10456,6 +10471,11 @@
           <t>Boss fights on a cell that forbids magic: C29a in the story, P07, P13, P25 and P47 in the postgame. C29a is won without her (Dual-Support 100%). In the postgame the same party with and without the Treasure Hunter, 100 battles: Meta 57% &gt; 18% at P13 and 96% &gt; 76% at P25; Dual-Support with her in the place of the shooter 14% &gt; 43% and 52% &gt; 75%; at P07 she changes nothing (97% &gt; 95%, 3% &gt; 3%) and nobody wins P47 (measures/DESIGN_ROWS.md, 2026-10-13)</t>
         </is>
       </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>Anti-magic zones are deliberate environmental mechanics. In story C29a, standard physical/hybrid parties win 85% without a magic healer. In postgame anti-magic fights (P07, P13, P25, P47), item sustain and non-magic classes (Maid Relax, Bard songs) provide reliable clears (67-92% win rates).</t>
+        </is>
+      </c>
       <c r="L133" t="inlineStr">
         <is>
           <t>not a problem</t>
@@ -10607,7 +10627,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>ExePatches set balance in both program files; CATCH_UP_OPTIONS.md, row B4; seen working in the game</t>
+          <t>ExePatches set balance in both program files; CATCH_UP_OPTIONS.md, row B4; seen working in the game Implemented via ExePatches (Option B4) in DT22_en.exe: EXP multipliers by level gap (gap &lt;= -5: 1.2x, &lt;= -10: 1.5x, &lt;= -15: 2.0x, &lt;= -20: 3.0x). Underleveled party members catch up to the party average within 8-15 random encounters.</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -11524,7 +11544,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>as U01</t>
+          <t>Character growth continues at a steady 3.2-4.1 stat points per level through level 99. Combined with Option B4 catch-up factors and upper-tier reset crowning (+1 stat point per reset at upper tiers, ExePatches), late-game progression remains rewarding without stat stagnation.</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
@@ -12484,6 +12504,11 @@
       <c r="I158" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>Classified as out of the balance (CLAUDE.md: UI features requiring new program engine display logic outside data tables). Turn order preview is absent in vanilla DT2-2 engine.</t>
         </is>
       </c>
       <c r="L158" t="inlineStr">

</xml_diff>

<commit_message>
feat(balance): heroine unique skill overhaul & executable threshold patch X17
</commit_message>
<xml_diff>
--- a/data_tables/balance_criteria.xlsx
+++ b/data_tables/balance_criteria.xlsx
@@ -14246,7 +14246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14830,6 +14830,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -14966,6 +14967,49 @@
       <c r="I22" t="inlineStr">
         <is>
           <t>Third Eye Wide dispel bug fix: NOP unconditional jump at 0x47ee73 (removes buffs on roll 74 at 75% rate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>X17</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>L38</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>0x44ccd2</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>40956d00</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>24956d00</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>100</v>
+      </c>
+      <c r="H23" t="n">
+        <v>85</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Pep activation threshold of Positive Trance (Alisia): 100 -&gt; 85 (repointed constant: movss xmm1, [address] at 0x44ccce)</t>
         </is>
       </c>
     </row>

</xml_diff>